<commit_message>
1st designed added (INA 226)
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280FF984-D9F3-4C0D-B786-CFB6B8741FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="21490" yWindow="1460" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
+    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +25,95 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Package</t>
+  </si>
+  <si>
+    <t>MPN</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Distributor PN</t>
+  </si>
+  <si>
+    <t>Distributor</t>
+  </si>
+  <si>
+    <t>Datasheet</t>
+  </si>
+  <si>
+    <t>Distributor Link</t>
+  </si>
+  <si>
+    <t>Library Ref</t>
+  </si>
+  <si>
+    <t>Library Path</t>
+  </si>
+  <si>
+    <t>Footprint Ref</t>
+  </si>
+  <si>
+    <t>Footprint Path</t>
+  </si>
+  <si>
+    <t>050-0001</t>
+  </si>
+  <si>
+    <t>Monitores y reguladores de corriente y energía Hi-Side Msmt Bi-Dir Current/Pwr Mon A 59 A 595-INA226AIDGST</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>MSOP-10</t>
+  </si>
+  <si>
+    <t>INA226AIDGSR</t>
+  </si>
+  <si>
+    <t>595-INA226AIDGSR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/ina226.pdf?ts=1772078114731&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FINA226</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/INA226AIDGSR?qs=tQG3bEuiOZD4quG3egR36g%3D%3D&amp;srsltid=AfmBOopOjh8KVXQVeHwZlO8DxeOetC6-xgaoNkKslHEV4iGJ_SkIIo7K</t>
+  </si>
+  <si>
+    <t>INA226</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Ics.SchLib</t>
+  </si>
+  <si>
+    <t>eUSR_PcbLibrary/eUSR_PcbLibrary.PcbLib</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +121,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,14 +160,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +466,182 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.08984375" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" customWidth="1"/>
+    <col min="8" max="8" width="12.453125" customWidth="1"/>
+    <col min="9" max="9" width="11.1796875" customWidth="1"/>
+    <col min="10" max="10" width="14.7265625" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="13.1796875" customWidth="1"/>
+    <col min="13" max="13" width="12.54296875" customWidth="1"/>
+    <col min="14" max="14" width="17.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="93.81640625" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" customWidth="1"/>
+    <col min="6" max="6" width="17.81640625" customWidth="1"/>
+    <col min="7" max="7" width="16.7265625" customWidth="1"/>
+    <col min="9" max="9" width="24.7265625" customWidth="1"/>
+    <col min="10" max="10" width="23.6328125" customWidth="1"/>
+    <col min="12" max="12" width="22.1796875" customWidth="1"/>
+    <col min="13" max="13" width="14.90625" customWidth="1"/>
+    <col min="14" max="14" width="21.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{1CFCC581-B5E5-4159-8EE1-35A941FCD4DF}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{78125F11-BE4E-4312-8E61-0550889BB81F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
070-0002 and 070-0003 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06409C09-0DBE-4737-8E92-BFF68DBA9FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3E5BF4-6ADE-4390-B2F5-7FB720DD6368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21490" yWindow="1460" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3400" uniqueCount="1680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3428" uniqueCount="1691">
   <si>
     <t>ID</t>
   </si>
@@ -5072,7 +5072,40 @@
     <t>TEN 2</t>
   </si>
   <si>
-    <t>TEN 2-2433</t>
+    <t>070-0002</t>
+  </si>
+  <si>
+    <t>Convertidores DC/DC para montaje pasante 6.5-36Vin 5V 2A SIP switching regulator</t>
+  </si>
+  <si>
+    <t>24V-5V</t>
+  </si>
+  <si>
+    <t>TSR 2-2450</t>
+  </si>
+  <si>
+    <t>495-TSR2-2450</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TRACO-Power/TSR-2-2450?qs=NtE2QagKf6RzknAolzm%2FTQ%3D%3D</t>
+  </si>
+  <si>
+    <t>070-0003</t>
+  </si>
+  <si>
+    <t>Convertidores DC/DC para montaje pasante 15-36Vin 12V 2A SIP switching regulator</t>
+  </si>
+  <si>
+    <t>24V-12V</t>
+  </si>
+  <si>
+    <t>TSR 2-24120</t>
+  </si>
+  <si>
+    <t>495-TSR2-24120</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TRACO-Power/TSR-2-24120?qs=NtE2QagKf6T34HiGRDOLrw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -16411,7 +16444,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="17.54296875" customWidth="1"/>
@@ -16477,7 +16510,7 @@
       <c r="E2" t="s">
         <v>1676</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" t="s">
         <v>46</v>
       </c>
       <c r="G2" t="s">
@@ -16499,19 +16532,106 @@
         <v>47</v>
       </c>
       <c r="M2" t="s">
+        <v>1678</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
         <v>1679</v>
       </c>
-      <c r="N2" t="s">
+      <c r="B3" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1673</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1682</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1683</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1674</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1684</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1678</v>
+      </c>
+      <c r="L3" t="s">
+        <v>47</v>
+      </c>
+      <c r="M3" t="s">
+        <v>1678</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>1685</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1686</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1687</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1673</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1688</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1689</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1674</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1690</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1678</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
+        <v>1678</v>
+      </c>
+      <c r="N4" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="https://www.mouser.es/manufacturer/traco-power/" xr:uid="{ECDB474B-3F6C-47CA-A9E3-99AC9E81CCAB}"/>
-    <hyperlink ref="I2" r:id="rId2" xr:uid="{08280A44-0F58-4FDE-B5FD-3A95A0F423CB}"/>
-    <hyperlink ref="J2" r:id="rId3" xr:uid="{85F326FF-BAE0-4072-815D-1EE4E7995C53}"/>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{08280A44-0F58-4FDE-B5FD-3A95A0F423CB}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{85F326FF-BAE0-4072-815D-1EE4E7995C53}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Diodes and Fuses added to Database
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,20 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{134ACE75-A3F6-4402-9049-AB2B5C56D66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A714708A-4030-41BF-8D74-53C922F5E575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21490" yWindow="1460" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
     <sheet name="010 - Resistors - SMD" sheetId="4" r:id="rId2"/>
     <sheet name="015 - Resistors - Shunt" sheetId="7" r:id="rId3"/>
     <sheet name="020 - Inductor" sheetId="5" r:id="rId4"/>
-    <sheet name="030 - Diodes" sheetId="9" r:id="rId5"/>
-    <sheet name="040 - Fuses" sheetId="10" r:id="rId6"/>
-    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId7"/>
-    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId8"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId9"/>
+    <sheet name="030 - Diode - Rectifier" sheetId="9" r:id="rId5"/>
+    <sheet name="031 - Diode - Schottky" sheetId="11" r:id="rId6"/>
+    <sheet name="033 - Diode - LED" sheetId="12" r:id="rId7"/>
+    <sheet name="040 - Fuses" sheetId="10" r:id="rId8"/>
+    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId9"/>
+    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId10"/>
+    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3428" uniqueCount="1691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4281" uniqueCount="2168">
   <si>
     <t>ID</t>
   </si>
@@ -5106,6 +5108,1437 @@
   </si>
   <si>
     <t>FUSE 2P</t>
+  </si>
+  <si>
+    <t>Shenzhen JDT Fuse</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>50A SMD Fuse 750mA 63V 63V 1206 Fuses ROHS</t>
+  </si>
+  <si>
+    <t>750mA</t>
+  </si>
+  <si>
+    <t>0466.750NRHF</t>
+  </si>
+  <si>
+    <t>Littelfuse</t>
+  </si>
+  <si>
+    <t>C187594</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2304140030_Littelfuse-0466-750NRHF_C187594.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Fuses_Littelfuse-0466-750NRHF_C187594.html</t>
+  </si>
+  <si>
+    <t>FUSE</t>
+  </si>
+  <si>
+    <t>FUSE SMD 1206</t>
+  </si>
+  <si>
+    <t>3A 125V (with holder) SMD,9.7x5mm Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>SMD,9.7x5mm</t>
+  </si>
+  <si>
+    <t>0154003.DRT</t>
+  </si>
+  <si>
+    <t>C206913</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2409302135_Littelfuse-0154003-DRT_C206913.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Disposable-fuses_Littelfuse-0154003-DRT_C206913.html</t>
+  </si>
+  <si>
+    <t>LITTLE154</t>
+  </si>
+  <si>
+    <t>50A SMD Fuse 1A 63V 63V 1206 Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>C136343</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2305151205_Shenzhen-JDT-Fuse-JFC1206-1100FS_C136343.pdf</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/Shenzhen_JdtFuse-JFC12061100FS/C136343</t>
+  </si>
+  <si>
+    <t>16V 250mA 100A 500mA 1206 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>250mA</t>
+  </si>
+  <si>
+    <t>C2830238</t>
+  </si>
+  <si>
+    <t>Jinrui Electronic Materials Co.</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2105311902_Jinrui-Electronic-Materials-Co--JK-nSMD025-16V_C2830238.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Resettable-Fuses_Jinrui-Electronic-Materials-Co-JK-nSMD025-16V_C2830238.html</t>
+  </si>
+  <si>
+    <t>50A SMD Fuse 5A 125V 125V SMD,6.1x2.7mm Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>SMD,6.1x2.7mm</t>
+  </si>
+  <si>
+    <t>0454005.MR</t>
+  </si>
+  <si>
+    <t>C179007</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410122030_Littelfuse-0454005-MR_C179007.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/Disposable-fuses_Littelfuse-0454005-MR_C179007.html</t>
+  </si>
+  <si>
+    <t>FUSE SMD 6.1x2.7mm</t>
+  </si>
+  <si>
+    <t>50A SMD Fuse 3A 63V 1206 Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>12H1300C</t>
+  </si>
+  <si>
+    <t>Shenzhen lanson Elec</t>
+  </si>
+  <si>
+    <t>C182445</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410122025_Shenzhen-lanson-Elec-12H1300C_C182445.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/Disposable-fuses_Shenzhen-lanson-Elec-12H1300C_C182445.html</t>
+  </si>
+  <si>
+    <t>50A SMD Fuse 1A 63V 1206 Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>12H1100C</t>
+  </si>
+  <si>
+    <t>C182308</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410122025_Shenzhen-lanson-Elec-12H1100C_C182308.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/Disposable-fuses_Shenzhen-lanson-Elec-12H1100C_C182308.html</t>
+  </si>
+  <si>
+    <t>16V 2.5A 40A 5A 1812 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>2,5A</t>
+  </si>
+  <si>
+    <t>1812L250/16GR</t>
+  </si>
+  <si>
+    <t>LUTE</t>
+  </si>
+  <si>
+    <t>C19078727</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2310251505_LUTE-1812L250-16GR_C19078727.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Resettable-Fuses_LUTE-1812L250-16GR_C19078727.html?s_z=n_JK-nSMD200</t>
+  </si>
+  <si>
+    <t>FUSE SMD 1812</t>
+  </si>
+  <si>
+    <t>24V 1.5A 40A 3A 40mΩ 1812 PTC Resettable Fuses RoHS</t>
+  </si>
+  <si>
+    <t>1.5A</t>
+  </si>
+  <si>
+    <t>1812L150/24GR</t>
+  </si>
+  <si>
+    <t>C22392774</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C22392774.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C22392774.html?s_z=n_1812L150%252F24GR</t>
+  </si>
+  <si>
+    <t>Fuses with Leads - Through Hole 10A 250V SR-5F</t>
+  </si>
+  <si>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>THT,D8.5xL7.6mm</t>
+  </si>
+  <si>
+    <t>SR-5F-10A-AP</t>
+  </si>
+  <si>
+    <t>Eaton Electronics</t>
+  </si>
+  <si>
+    <t>504-SR-5F-10A-AP</t>
+  </si>
+  <si>
+    <t>https://www.eaton.com/content/dam/eaton/products/electronic-components/resources/data-sheet/eaton-sr-5f-subminiature-fast-acting-fuses-data-sheet.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Eaton-Electronics/SR-5F-10A-AP?qs=jGANiKWBgcj73AguR930Aw%3D%3D</t>
+  </si>
+  <si>
+    <t>FUSE SR-5F</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 16V 2A Surface Mount 1812</t>
+  </si>
+  <si>
+    <t>2A</t>
+  </si>
+  <si>
+    <t>1812L200/16GR</t>
+  </si>
+  <si>
+    <t>C18198340</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C18198340.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C18198340.html?s_z=n_1812L200%252F16GR</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 16V 2A Surface Mount 1206</t>
+  </si>
+  <si>
+    <t>1206L200/16NR</t>
+  </si>
+  <si>
+    <t>C22374899</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C22374899.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C22374899.html</t>
+  </si>
+  <si>
+    <t>4A 72V Fuse Surface Mount 1206</t>
+  </si>
+  <si>
+    <t>4A</t>
+  </si>
+  <si>
+    <t>BSMD1206C-1400T</t>
+  </si>
+  <si>
+    <t>BHFUSE</t>
+  </si>
+  <si>
+    <t>C41367227</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C41367227.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C41367227.html</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 32V 0603 4A V/FA HALIDE FREE</t>
+  </si>
+  <si>
+    <t>0467004.NRHF</t>
+  </si>
+  <si>
+    <t>576-0467004.NRHF</t>
+  </si>
+  <si>
+    <t>https://www.littelfuse.com/assetdocs/littelfuse_fuse_467_datasheet.pdf?assetguid=4a59f034-1cca-460e-a5ba-e1e66247c76d</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Littelfuse/0467004.NRHF?qs=PalBzRKzfnueyHMjEWtHJQ%3D%3D</t>
+  </si>
+  <si>
+    <t>FUSE SMD 0603</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 32V 0603 2A V/FA HALIDE FREE</t>
+  </si>
+  <si>
+    <t>0467002.NRHF</t>
+  </si>
+  <si>
+    <t>576-0467002.NRHF</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Littelfuse/0467002.NRHF?qs=n5MbhIql%252BRnna7dCryodUA%3D%3D</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 33V 100mA Surface Mount 0603</t>
+  </si>
+  <si>
+    <t>100mA</t>
+  </si>
+  <si>
+    <t>0603L010/33XR</t>
+  </si>
+  <si>
+    <t>C7472521</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C7472516.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C7472521.html?s_z=n_0603L010%252F33XR</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 30V 2A Surface Mount 1812</t>
+  </si>
+  <si>
+    <t>1812L200/30GR</t>
+  </si>
+  <si>
+    <t>C18198342</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C19078727.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C18198342.html?s_z=n_1812L200%252F30GR</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 30V 5A Surface Mount 2920</t>
+  </si>
+  <si>
+    <t>2920</t>
+  </si>
+  <si>
+    <t>2920L500/30GR</t>
+  </si>
+  <si>
+    <t>C19078763</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C19078763.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C19078763.html</t>
+  </si>
+  <si>
+    <t>FUSE SMD 2920</t>
+  </si>
+  <si>
+    <t>Polymeric PTC Resettable Fuse 24V 3A Surface Mount 1812</t>
+  </si>
+  <si>
+    <t>1812L300/24GR</t>
+  </si>
+  <si>
+    <t>C20627123</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C20627123.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C20627123.html</t>
+  </si>
+  <si>
+    <t>040-0002</t>
+  </si>
+  <si>
+    <t>040-0003</t>
+  </si>
+  <si>
+    <t>040-0004</t>
+  </si>
+  <si>
+    <t>040-0005</t>
+  </si>
+  <si>
+    <t>040-0006</t>
+  </si>
+  <si>
+    <t>040-0007</t>
+  </si>
+  <si>
+    <t>040-0008</t>
+  </si>
+  <si>
+    <t>040-0009</t>
+  </si>
+  <si>
+    <t>040-0010</t>
+  </si>
+  <si>
+    <t>040-0011</t>
+  </si>
+  <si>
+    <t>040-0012</t>
+  </si>
+  <si>
+    <t>040-0013</t>
+  </si>
+  <si>
+    <t>040-0014</t>
+  </si>
+  <si>
+    <t>040-0015</t>
+  </si>
+  <si>
+    <t>040-0016</t>
+  </si>
+  <si>
+    <t>040-0017</t>
+  </si>
+  <si>
+    <t>040-0018</t>
+  </si>
+  <si>
+    <t>040-0019</t>
+  </si>
+  <si>
+    <t>040-0020</t>
+  </si>
+  <si>
+    <t>030-0001</t>
+  </si>
+  <si>
+    <t>920mV@2A 25ns 2A 50V SMA Fast Recovery / High Efficiency Diodes ROHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">920mV@2A </t>
+  </si>
+  <si>
+    <t>SMA</t>
+  </si>
+  <si>
+    <t>ES2AA-13-F</t>
+  </si>
+  <si>
+    <t>Diodes Incorporated</t>
+  </si>
+  <si>
+    <t>C151575</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2304140030_Diodes-Incorporated-ES2AA-13-F_C151575.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Fast-Recovery-High-Efficiency-Diodes_Diodes-Incorporated-ES2AA-13-F_C151575.html?s_z=n_ES2AA-13-F</t>
+  </si>
+  <si>
+    <t>DIODE</t>
+  </si>
+  <si>
+    <t>DIODE SMA</t>
+  </si>
+  <si>
+    <t>030-0002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1V@100mA 200mA 30V SOD-323 Schottky Diodes ROHS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1V@100mA 200mA </t>
+  </si>
+  <si>
+    <t>SOD-323</t>
+  </si>
+  <si>
+    <t>BAT54WS</t>
+  </si>
+  <si>
+    <t>hongjiacheng</t>
+  </si>
+  <si>
+    <t>C7502694</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2308281443_hongjiacheng-BAT54WS_C7502694.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Schottky-Diodes_hongjiacheng-BAT54WS_C7502694.html?s_z=n_BAT54</t>
+  </si>
+  <si>
+    <t>DIODE SOD323</t>
+  </si>
+  <si>
+    <t>030-0003</t>
+  </si>
+  <si>
+    <t>1V@10mA 4ns 200mA 100V  SOT-23 Switching Diodes ROHS</t>
+  </si>
+  <si>
+    <t>1V@10mA 200mA</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>MMBD4148CC</t>
+  </si>
+  <si>
+    <t>onsemi</t>
+  </si>
+  <si>
+    <t>C236939</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121737_onsemi-MMBD4148CC_C236939.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Switching-Diodes_onsemi-MMBD4148CC_C236939.html?s_z=n_MMBD4148CC</t>
+  </si>
+  <si>
+    <t>DIODE CC</t>
+  </si>
+  <si>
+    <t>DIODE SOT-23</t>
+  </si>
+  <si>
+    <t>030-0004</t>
+  </si>
+  <si>
+    <t>1A 1kV 1.1V@1A SOD-123FL Diodes - General Purpose ROHS</t>
+  </si>
+  <si>
+    <t>SOD-123</t>
+  </si>
+  <si>
+    <t>SM4007PL A7</t>
+  </si>
+  <si>
+    <t>Slkor(SLKORMICRO Elec.)</t>
+  </si>
+  <si>
+    <t>C426570</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_1912111437_Slkor-SLKORMICRO-Elec--SM4007PL-A7_C426570.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Diodes-General-Purpose_Slkor-SLKORMICRO-Elec-SM4007PL-A7_C426570.html?s_z=n_C426570</t>
+  </si>
+  <si>
+    <t>030-0005</t>
+  </si>
+  <si>
+    <t>80A 40V Independent 520mV@3A 3A SOD-123FL Single Diodes ROHS</t>
+  </si>
+  <si>
+    <t>40V 3A</t>
+  </si>
+  <si>
+    <t>SOD-123FL</t>
+  </si>
+  <si>
+    <t>DSK34</t>
+  </si>
+  <si>
+    <t>TWGMC</t>
+  </si>
+  <si>
+    <t>C727076</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C727076.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C727076.html</t>
+  </si>
+  <si>
+    <t>SOD-123FL2</t>
+  </si>
+  <si>
+    <t>030-0006</t>
+  </si>
+  <si>
+    <t>Rectifiers 6.0 Amp 600 Volt 400 Amp IFSM</t>
+  </si>
+  <si>
+    <t>600V 22A</t>
+  </si>
+  <si>
+    <t>P600</t>
+  </si>
+  <si>
+    <t>P600J-E3/73</t>
+  </si>
+  <si>
+    <t>Vishay General Semiconductor</t>
+  </si>
+  <si>
+    <t>625-P600J-E3/73</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/88692/p600a.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-General-Semiconductor/P600J-E3-73?qs=E3OxquYwg8HdCumpNQmXxA%3D%3D</t>
+  </si>
+  <si>
+    <t>P600J</t>
+  </si>
+  <si>
+    <t>030-0007</t>
+  </si>
+  <si>
+    <t>Rectifiers Ultrafast, DO-41, 50V, 1A, 175C</t>
+  </si>
+  <si>
+    <t>50V 1A</t>
+  </si>
+  <si>
+    <t>DO-41</t>
+  </si>
+  <si>
+    <t>UF4001</t>
+  </si>
+  <si>
+    <t>Diotec Semiconductor</t>
+  </si>
+  <si>
+    <t>637-UF4001</t>
+  </si>
+  <si>
+    <t>https://diotec.com/request/datasheet/uf4001.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Diotec-Semiconductor/UF4001?qs=OlC7AqGiEDm1RpsmSECQSQ%3D%3D</t>
+  </si>
+  <si>
+    <t>030-0008</t>
+  </si>
+  <si>
+    <t>Rectifiers Ultrafast, DO-214AC, 1200V, 1A</t>
+  </si>
+  <si>
+    <t>1200V 1A</t>
+  </si>
+  <si>
+    <t>DO-214AC</t>
+  </si>
+  <si>
+    <t>STTH112A-FS</t>
+  </si>
+  <si>
+    <t>FUXINSEMI</t>
+  </si>
+  <si>
+    <t>C5563725</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C5563725.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C5563725.html?s_z=n_STTH112</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Diode.SchLib</t>
+  </si>
+  <si>
+    <t>031-0001</t>
+  </si>
+  <si>
+    <t>40V 550mV@2A 2A 0603 Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>40V 550mV@2A 2A</t>
+  </si>
+  <si>
+    <t>NSR20F40NXT5G</t>
+  </si>
+  <si>
+    <t>C153761</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_1809111720_onsemi-NSR20F40NXT5G_C153761.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Schottky-Diodes_onsemi-NSR20F40NXT5G_C153761.html</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY</t>
+  </si>
+  <si>
+    <t>DIODE SMD 0603</t>
+  </si>
+  <si>
+    <t>031-0002</t>
+  </si>
+  <si>
+    <t>40V 900mV@100mA 300mA SOD-523 Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>40V 900mV@100mA 300mA</t>
+  </si>
+  <si>
+    <t>SOD-523</t>
+  </si>
+  <si>
+    <t>BAT54KFILM</t>
+  </si>
+  <si>
+    <t>C283259</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2304140030_STMicroelectronics-BAT54KFILM_C283259.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Schottky-Diodes_STMicroelectronics-BAT54KFILM_C283259.html</t>
+  </si>
+  <si>
+    <t>031-0003</t>
+  </si>
+  <si>
+    <t>40V Independent Type 550mV@5A 5A SMA(DO-214AC) Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>40V 550mV@5A 5A</t>
+  </si>
+  <si>
+    <t>SS54</t>
+  </si>
+  <si>
+    <t>MDD(Microdiode Semiconductor)</t>
+  </si>
+  <si>
+    <t>C22452</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2411211945_MDD-Microdiode-Semiconductor-SS54_C22452.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Schottky-Diodes_MDD-Microdiode-Semiconductor-SS54_C22452.html?s_z=n_C22452</t>
+  </si>
+  <si>
+    <t>031-0004</t>
+  </si>
+  <si>
+    <t>30V 1 pair in series 1V@100mA 200mA SOT-23 Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>30V 1V@100mA 200mA</t>
+  </si>
+  <si>
+    <t>BAT54S</t>
+  </si>
+  <si>
+    <t>C727126</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410122023_TWGMC-BAT54S_C727126.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Schottky-Barrier-Diodes-SBD_TWGMC-BAT54S_C727126.html</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 3P</t>
+  </si>
+  <si>
+    <t>031-0005</t>
+  </si>
+  <si>
+    <t>60V 10A 700mV@10A SMB Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>60V 700mV@10A 10A</t>
+  </si>
+  <si>
+    <t>DO-214AA</t>
+  </si>
+  <si>
+    <t>SS1060B</t>
+  </si>
+  <si>
+    <t>C18208635</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2309281727_Slkor-SLKORMICRO-Elec--SS1060B_C18208635.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/Schottky-Diodes_Slkor-SLKORMICRO-Elec-SS1060B_C18208635.html?s_z=s_Diodes%257CSchottky%2520Diodes</t>
+  </si>
+  <si>
+    <t>031-0006</t>
+  </si>
+  <si>
+    <t>Zener Diodes 5.1 Volt 0.5W 5%</t>
+  </si>
+  <si>
+    <t>5.1V 100nA</t>
+  </si>
+  <si>
+    <t>DO-35-2</t>
+  </si>
+  <si>
+    <t>BZX55C5V1-TR</t>
+  </si>
+  <si>
+    <t>Vishay Semiconductors</t>
+  </si>
+  <si>
+    <t>78-BZX55C5V1</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/85604/bzx55.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Semiconductors/BZX55C5V1-TR?qs=WLTup5mM6hhy%252Bqloxl7%2FIQ%3D%3D&amp;utm_id=20109199436&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=emeacorp&amp;gad_source=1&amp;gad_campaignid=20109199436&amp;gbraid=0AAAAADn_wf2RhF_lSG_YlgnN1Yzlq3oak&amp;gclid=Cj0KCQiAhtvMBhDBARIsAL26pjE6pviBOpVaBUJ07A83YFMQUf7QkOHJpiHMP9nHJbQo8SvNA6LellYaAlJaEALw_wcB</t>
+  </si>
+  <si>
+    <t>031-0007</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 40V SMA(DO-214AC)</t>
+  </si>
+  <si>
+    <t>SMA(DO-214AC)</t>
+  </si>
+  <si>
+    <t>SS34</t>
+  </si>
+  <si>
+    <t>GOODWORK</t>
+  </si>
+  <si>
+    <t>C908680</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C908680.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C908680.html?s_z=n_SS34</t>
+  </si>
+  <si>
+    <t>031-0008</t>
+  </si>
+  <si>
+    <t>Diode 40V 1A Surface Mount SMA(DO-214AC)</t>
+  </si>
+  <si>
+    <t>41V 1A</t>
+  </si>
+  <si>
+    <t>SS14</t>
+  </si>
+  <si>
+    <t>JSMSEMI</t>
+  </si>
+  <si>
+    <t>C2837270</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C2837270.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C2837270.html?s_z=n_C2837270</t>
+  </si>
+  <si>
+    <t>031-0009</t>
+  </si>
+  <si>
+    <t>Diode 40V 200mA Surface Mount 0603</t>
+  </si>
+  <si>
+    <t>580mV@2A</t>
+  </si>
+  <si>
+    <t>CD0603-B0240R</t>
+  </si>
+  <si>
+    <t>BOURNS</t>
+  </si>
+  <si>
+    <t>C3312582</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C3312582.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C3312582.html</t>
+  </si>
+  <si>
+    <t>DIODE_SMD_0603</t>
+  </si>
+  <si>
+    <t>031-0010</t>
+  </si>
+  <si>
+    <t>Diodos y rectificadores Schottky 10A, 200V, SMPC TRENCH SKY RECT.</t>
+  </si>
+  <si>
+    <t>200V 10A</t>
+  </si>
+  <si>
+    <t>SMPC (TO-277A-3)</t>
+  </si>
+  <si>
+    <t>V10P22HM3_A/H</t>
+  </si>
+  <si>
+    <t>78-V10P22HM3_A/H</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/87002/v10p22.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/V10P22HM3_A-H?qs=sGAEpiMZZMtbRapU8LlZD8qu4xuMq4%252BSxFIcXPYKbhU%252BdoNGIetOdA%3D%3D</t>
+  </si>
+  <si>
+    <t>TO-277A-3</t>
+  </si>
+  <si>
+    <t>031-0011</t>
+  </si>
+  <si>
+    <t>Diode 60V 3A Surface Mount SOD-123FL</t>
+  </si>
+  <si>
+    <t>60V 3A</t>
+  </si>
+  <si>
+    <t>S-LMBR360FT1G</t>
+  </si>
+  <si>
+    <t>LRC</t>
+  </si>
+  <si>
+    <t>C5383051</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C5383051.pdf?spm=wm.sxq.inf.ggs___wm.ssy.bg.5.xh&amp;lcsc_vid=RABbXwFTQFhZUlVVRVZYUlJXEwdcBAFSTgJbUVxeT1IxVlNRQ1FeUFRQT1hdVTsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slQlJWVFRTRk8GEwkK</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C5383051.html?s_z=n_Schottky%252C%2520MBR360&amp;spm=wm.ssy.bg.5.xh&amp;lcsc_vid=RABbXwFTQFhZUlVVRVZYUlJXEwdcBAFSTgJbUVxeT1IxVlNRQ1FeUFRQT1hdVTsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slQlJWVFRTRk8GEwkK</t>
+  </si>
+  <si>
+    <t>032-0001</t>
+  </si>
+  <si>
+    <t>6A@8/20us 12V 5.1V 5V FBP-02C ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>FBP-02C</t>
+  </si>
+  <si>
+    <t>ESD5471X-2/TR</t>
+  </si>
+  <si>
+    <t>WILLSEMI(Will Semicon)</t>
+  </si>
+  <si>
+    <t>C239631</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2004031411_WILLSEMI-Will-Semicon-ESD5471X-2-TR_C239631.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/span-style-background-color-ff0-ESD-span-and-Surge-Protection-TVS-span-style-background-color-ff0-ESD-span_WILLSEMI-Will-Semicon-ESD5471X-2-TR_C239631.html</t>
+  </si>
+  <si>
+    <t>TVS</t>
+  </si>
+  <si>
+    <t>032-0002</t>
+  </si>
+  <si>
+    <t>5A 100W 15V 6V Bidirectional 5V DFN1006 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>DFN1006</t>
+  </si>
+  <si>
+    <t>AZ5825-01F</t>
+  </si>
+  <si>
+    <t>KUU</t>
+  </si>
+  <si>
+    <t>C5119557</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2207261800_KUU-AZ5825-01F_C5119557.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_KUU-AZ5825-01F_C5119557.html</t>
+  </si>
+  <si>
+    <t>032-0003</t>
+  </si>
+  <si>
+    <t>7A 11V 72W 8.4V Bidirectional 5V 0402 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>ESD5451N-TP</t>
+  </si>
+  <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
+    <t>C2830311</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2411121100_TECH-PUBLIC-ESD5451N-TP_C2830311.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_TECH-PUBLIC-ESD5451N-TP_C2830311.html</t>
+  </si>
+  <si>
+    <t>TVS SMD 0402</t>
+  </si>
+  <si>
+    <t>032-0004</t>
+  </si>
+  <si>
+    <t>1A 9.8V 5.4V Unidirectional 5V SOD-923 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>SOD-923</t>
+  </si>
+  <si>
+    <t>ESD9L5.0ST5G</t>
+  </si>
+  <si>
+    <t>C82326</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410010231_onsemi-ESD9L5-0ST5G_C82326.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_onsemi-ESD9L5-0ST5G_C82326.html</t>
+  </si>
+  <si>
+    <t>032-0005</t>
+  </si>
+  <si>
+    <t>100W 30V 6.5V 5.5V SLP1616-6 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>SLP1616-6</t>
+  </si>
+  <si>
+    <t>RCLAMP0854P.TCT</t>
+  </si>
+  <si>
+    <t>SEMTECH</t>
+  </si>
+  <si>
+    <t>C842842</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2411011545_SEMTECH-RCLAMP0854P-TCT_C842842.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_SEMTECH-RCLAMP0854P-TCT_C842842.html</t>
+  </si>
+  <si>
+    <t>RCLAMP0854P-TCT</t>
+  </si>
+  <si>
+    <t>SLP1616P6-6L</t>
+  </si>
+  <si>
+    <t>032-0006</t>
+  </si>
+  <si>
+    <t>54.4A 1.5kW 27.6V 18.9V 17V DO-214AB ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>DO-214AB</t>
+  </si>
+  <si>
+    <t>SMCJ17A</t>
+  </si>
+  <si>
+    <t>C2938306</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410122003_Littelfuse-SMCJ17A_C2938306.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_Littelfuse-SMCJ17A_C2938306.html?s_z=n_SMCJ17A</t>
+  </si>
+  <si>
+    <t>TVS S</t>
+  </si>
+  <si>
+    <t>032-0007</t>
+  </si>
+  <si>
+    <t>Independent Type 5W 19V SMB Zener Diodes ROHS</t>
+  </si>
+  <si>
+    <t>SMBJ5356B-MS</t>
+  </si>
+  <si>
+    <t>MSKSEMI</t>
+  </si>
+  <si>
+    <t>C18547763</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121938_Littelfuse-015402-5DR_C206922.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/Zener-Diodes_MSKSEMI-SMBJ5356B-MS_C18547763.html?s_z=n_C18547763</t>
+  </si>
+  <si>
+    <t>DO-214AA B</t>
+  </si>
+  <si>
+    <t>032-0008</t>
+  </si>
+  <si>
+    <t>30.2A 19.9V 13.3V 12V SMB ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>SMBJ12A</t>
+  </si>
+  <si>
+    <t>YFW</t>
+  </si>
+  <si>
+    <t>C2898391</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121738_YFW-SMBJ12A_C2898391.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/TVS_YFW-SMBJ12A_C2898391.html</t>
+  </si>
+  <si>
+    <t>032-0009</t>
+  </si>
+  <si>
+    <t>400W SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>CDSOT23-SM712</t>
+  </si>
+  <si>
+    <t>C404012</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121813_BOURNS-CDSOT23-SM712_C404012.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_BOURNS-CDSOT23-SM712_C404012.html?s_z=n_CDSOT23-SM712</t>
+  </si>
+  <si>
+    <t>Dual TVS</t>
+  </si>
+  <si>
+    <t>032-0010</t>
+  </si>
+  <si>
+    <t>369W 12.3V 4V 3.3V SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>GSOT03C-E3-08</t>
+  </si>
+  <si>
+    <t>C435893</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121813_Vishay-Intertech-GSOT03C-E3-08_C435893.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_Vishay-Intertech-GSOT03C-E3-08_C435893.html?s_z=n_GSOT03C-E3-08</t>
+  </si>
+  <si>
+    <t>ESD 2-line</t>
+  </si>
+  <si>
+    <t>032-0011</t>
+  </si>
+  <si>
+    <t>6A 320W 38V 26.5V Bidirectional 24V SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>ESD2CAN24-ES</t>
+  </si>
+  <si>
+    <t>ElecSuper</t>
+  </si>
+  <si>
+    <t>C19170841</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2412061751_ElecSuper-ESD2CAN24-ES_C19170841.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_ElecSuper-ESD2CAN24-ES_C19170841.html?s_z=n_ESD2CAN24</t>
+  </si>
+  <si>
+    <t>032-0012</t>
+  </si>
+  <si>
+    <t>DFN2510-10L ESD and Surge Protection 4 channels(TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>DFN2510-10L</t>
+  </si>
+  <si>
+    <t>ESD73034D-10/TR</t>
+  </si>
+  <si>
+    <t>C2941834</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2410121434_WILLSEMI-Will-Semicon-ESD73034D-10-TR_C2941834.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-Protection-Devices_WILLSEMI-Will-Semicon-ESD73034D-10-TR_C2941834.html</t>
+  </si>
+  <si>
+    <t>ESD73034D</t>
+  </si>
+  <si>
+    <t>032-0013</t>
+  </si>
+  <si>
+    <t>ESD Protection Diodes / TVS Diodes WE-TVS Diode Array 3.3V 0.18pF 2Channel</t>
+  </si>
+  <si>
+    <t>DFN-1210-6</t>
+  </si>
+  <si>
+    <t>Wurth Elektronik</t>
+  </si>
+  <si>
+    <t>710-824012823</t>
+  </si>
+  <si>
+    <t>MOUSER</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/824012823.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/824012823?qs=rrS6PyfT74dPtw7q26tZFg%3D%3D</t>
+  </si>
+  <si>
+    <t>DFN1210-6L</t>
+  </si>
+  <si>
+    <t>032-0014</t>
+  </si>
+  <si>
+    <t>25A 20V 4V Unidirectional 3.3V SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>PESD3V3S2UT-ES</t>
+  </si>
+  <si>
+    <t>C5199192</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/datasheet/lcsc_datasheet_2504101957_ElecSuper-PESD3V3L2BT-ES_C5180242.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_ElecSuper-PESD3V3S2UT-ES_C5199192.html</t>
+  </si>
+  <si>
+    <t>032-0015</t>
+  </si>
+  <si>
+    <t>4A@8/20us 100W@8/20us 15V 4.2V 3.3V SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>TPESD3V3X2UTR</t>
+  </si>
+  <si>
+    <t>C48586723</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/datasheet/lcsc_datasheet_2504281715_TECH-PUBLIC-TPESD3V3X2UTR_C48586723.pdf</t>
+  </si>
+  <si>
+    <t>DIODE 3P R</t>
+  </si>
+  <si>
+    <t>032-0016</t>
+  </si>
+  <si>
+    <t>6A 15V 150W 9V 5V SOT-23-6 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>SOT-23-6</t>
+  </si>
+  <si>
+    <t>USBLC6-2SC6</t>
+  </si>
+  <si>
+    <t>C5250994</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/datasheet/lcsc_datasheet_2410121815_TWGMC-USBLC6-2SC6_C5250994.pdf</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_TWGMC-USBLC6-2SC6_C5250994.html?s_z=n_C5250994</t>
+  </si>
+  <si>
+    <t>DUAL_TVS_DIODE</t>
+  </si>
+  <si>
+    <t>032-0017</t>
+  </si>
+  <si>
+    <t>SOT-23 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>RLST23A032C</t>
+  </si>
+  <si>
+    <t>RUILON(Shenzhen Ruilongyuan Elec)</t>
+  </si>
+  <si>
+    <t>C46970949</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/lcsc_datasheet_2504101957_RUILON-Shenzhen-Ruilongyuan-Elec-RLST23A032C_C46970949.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/ESD-and-Surge-Protection-TVS-ESD_RUILON-Shenzhen-Ruilongyuan-Elec-RLST23A032C_C46970949.html?s_z=n_RLST23A032C</t>
+  </si>
+  <si>
+    <t>032-0018</t>
+  </si>
+  <si>
+    <t>40A@8/20us 27.7V 1.12kW@8/20us 25.9V Unidirectional 22V WSON-6-EP(2x2) ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
+    <t>WSON-6-EP(2x2)</t>
+  </si>
+  <si>
+    <t>TVS2200DRVR</t>
+  </si>
+  <si>
+    <t>C523793</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C523793.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C523793.html?s_z=n_TVS2200DRVR</t>
+  </si>
+  <si>
+    <t>032-0019</t>
+  </si>
+  <si>
+    <t>High-speed serial interface common mode filter with ESD protection</t>
+  </si>
+  <si>
+    <t>microQFN-6L</t>
+  </si>
+  <si>
+    <t>ECMF2-40A100N6</t>
+  </si>
+  <si>
+    <t>C5267592</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C5267592.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C5267592.html?s_z=n_ECMF2-40A100N6</t>
+  </si>
+  <si>
+    <t>MICROQFN-6L</t>
+  </si>
+  <si>
+    <t>032-0020</t>
+  </si>
+  <si>
+    <t>Zener Diode 7.5V 250mW Surface Mount SOT-23</t>
+  </si>
+  <si>
+    <t>BZX84C7V5LT1G</t>
+  </si>
+  <si>
+    <t>C236201</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C236201.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C236201.html</t>
+  </si>
+  <si>
+    <t>ZENER_SOT23</t>
+  </si>
+  <si>
+    <t>032-0021</t>
+  </si>
+  <si>
+    <t>10.3VC Clamp 38.8A Ipp TVS DIODE DO-214AC(SMA)</t>
+  </si>
+  <si>
+    <t>DO-214AC(SMA)</t>
+  </si>
+  <si>
+    <t>SMAJ6.0A</t>
+  </si>
+  <si>
+    <t>C223993</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C223993.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C223993.html</t>
+  </si>
+  <si>
+    <t>032-0022</t>
+  </si>
+  <si>
+    <t>TVS DIODE 14VWM 23.2VC DO-214AA</t>
+  </si>
+  <si>
+    <t>SMBJ13A</t>
+  </si>
+  <si>
+    <t>C151252</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/datasheet/C151252.pdf</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C151252.html</t>
   </si>
 </sst>
 </file>
@@ -5115,7 +6548,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5201,8 +6634,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5213,6 +6669,12 @@
       <patternFill patternType="solid">
         <fgColor theme="2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0CECE"/>
+        <bgColor rgb="FFD0CECE"/>
       </patternFill>
     </fill>
   </fills>
@@ -5246,7 +6708,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5281,6 +6743,56 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -9685,6 +11197,254 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="4" max="4" width="17.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1669</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1670</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1671</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1674</v>
+      </c>
+      <c r="F2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1675</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>1672</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>1673</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1676</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1676</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>1677</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1671</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1680</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1681</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1672</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1682</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1676</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M3" t="s">
+        <v>1676</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>1683</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1685</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1671</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1686</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1687</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1672</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1688</v>
+      </c>
+      <c r="K4" t="s">
+        <v>1676</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M4" t="s">
+        <v>1676</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{08280A44-0F58-4FDE-B5FD-3A95A0F423CB}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{85F326FF-BAE0-4072-815D-1EE4E7995C53}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
   <dimension ref="A1:N136"/>
@@ -15981,7 +17741,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652841DA-3619-42EE-A536-61B58BE1B457}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -16028,21 +17788,1975 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="32" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>1833</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>1834</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>1835</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>1836</v>
+      </c>
+      <c r="F2" s="32" t="s">
+        <v>1837</v>
+      </c>
+      <c r="G2" s="32" t="s">
+        <v>1838</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="32" t="s">
+        <v>1839</v>
+      </c>
+      <c r="J2" s="32" t="s">
+        <v>1840</v>
+      </c>
+      <c r="K2" s="32" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L2" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M2" s="32" t="s">
+        <v>1842</v>
+      </c>
+      <c r="N2" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="32" t="s">
+        <v>1843</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>1844</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>1845</v>
+      </c>
+      <c r="D3" s="32" t="s">
+        <v>1846</v>
+      </c>
+      <c r="E3" s="32" t="s">
+        <v>1847</v>
+      </c>
+      <c r="F3" s="32" t="s">
+        <v>1848</v>
+      </c>
+      <c r="G3" s="32" t="s">
+        <v>1849</v>
+      </c>
+      <c r="H3" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="32" t="s">
+        <v>1850</v>
+      </c>
+      <c r="J3" s="32" t="s">
+        <v>1851</v>
+      </c>
+      <c r="K3" s="32" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L3" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M3" s="32" t="s">
+        <v>1852</v>
+      </c>
+      <c r="N3" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="32" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>1854</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>1855</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>1857</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>1859</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="32" t="s">
+        <v>1860</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>1861</v>
+      </c>
+      <c r="K4" s="32" t="s">
+        <v>1862</v>
+      </c>
+      <c r="L4" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>1863</v>
+      </c>
+      <c r="N4" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="32" t="s">
+        <v>1864</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>1865</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>1866</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>1867</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>1868</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>1869</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>1870</v>
+      </c>
+      <c r="J5" s="33" t="s">
+        <v>1871</v>
+      </c>
+      <c r="K5" s="32" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L5" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M5" s="32" t="s">
+        <v>1866</v>
+      </c>
+      <c r="N5" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="32" t="s">
+        <v>1872</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>1873</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>1874</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>1875</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>1876</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>1878</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>1879</v>
+      </c>
+      <c r="J6" s="31" t="s">
+        <v>1880</v>
+      </c>
+      <c r="K6" s="32" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L6" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M6" s="31" t="s">
+        <v>1881</v>
+      </c>
+      <c r="N6" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="32" t="s">
+        <v>1882</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>1883</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>1884</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>1885</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>1886</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>1887</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>1888</v>
+      </c>
+      <c r="H7" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="31" t="s">
+        <v>1889</v>
+      </c>
+      <c r="J7" s="31" t="s">
+        <v>1890</v>
+      </c>
+      <c r="K7" s="35" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L7" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M7" s="35" t="s">
+        <v>1891</v>
+      </c>
+      <c r="N7" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="35" t="s">
+        <v>1892</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>1893</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>1894</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>1895</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>1896</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>1897</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>1898</v>
+      </c>
+      <c r="H8" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="37" t="s">
+        <v>1899</v>
+      </c>
+      <c r="J8" s="37" t="s">
+        <v>1900</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L8" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M8" s="35" t="s">
+        <v>1895</v>
+      </c>
+      <c r="N8" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="35" t="s">
+        <v>1901</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>1902</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>1903</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>1904</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>1905</v>
+      </c>
+      <c r="F9" s="31" t="s">
+        <v>1906</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>1907</v>
+      </c>
+      <c r="H9" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="31" t="s">
+        <v>1908</v>
+      </c>
+      <c r="J9" s="31" t="s">
+        <v>1909</v>
+      </c>
+      <c r="K9" s="35" t="s">
+        <v>1841</v>
+      </c>
+      <c r="L9" s="32" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M9" s="31" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N9" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I5" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="J5" r:id="rId2" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
+    <hyperlink ref="I8" r:id="rId3" xr:uid="{ABAB45EA-9261-4561-98A3-C830A74C7893}"/>
+    <hyperlink ref="J8" r:id="rId4" xr:uid="{E0090D85-56DB-4EF7-BD41-6F63EB17645B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2008B-4BF4-4C9A-883A-FEE5873AEAF4}">
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="16" customHeight="1">
+      <c r="A1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="39" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="39" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="39" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="39" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="16" customHeight="1">
+      <c r="A2" s="40" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>1912</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>1913</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>1914</v>
+      </c>
+      <c r="F2" s="40" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G2" s="40" t="s">
+        <v>1915</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>1916</v>
+      </c>
+      <c r="J2" s="40" t="s">
+        <v>1917</v>
+      </c>
+      <c r="K2" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L2" s="40" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M2" s="41" t="s">
+        <v>1919</v>
+      </c>
+      <c r="N2" s="40" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16" customHeight="1">
+      <c r="A3" s="40" t="s">
+        <v>1920</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>1921</v>
+      </c>
+      <c r="C3" s="40" t="s">
+        <v>1922</v>
+      </c>
+      <c r="D3" s="40" t="s">
+        <v>1923</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>1924</v>
+      </c>
+      <c r="F3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="40" t="s">
+        <v>1925</v>
+      </c>
+      <c r="H3" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="43" t="s">
+        <v>1926</v>
+      </c>
+      <c r="J3" s="40" t="s">
+        <v>1927</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L3" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M3" s="40" t="s">
+        <v>1923</v>
+      </c>
+      <c r="N3" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="16" customHeight="1">
+      <c r="A4" s="40" t="s">
+        <v>1928</v>
+      </c>
+      <c r="B4" s="40" t="s">
+        <v>1929</v>
+      </c>
+      <c r="C4" s="40" t="s">
+        <v>1930</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>1904</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>1931</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>1932</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>1933</v>
+      </c>
+      <c r="H4" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="40" t="s">
+        <v>1934</v>
+      </c>
+      <c r="J4" s="40" t="s">
+        <v>1935</v>
+      </c>
+      <c r="K4" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L4" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M4" s="40" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N4" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="16" customHeight="1">
+      <c r="A5" s="40" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>1937</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>1938</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>1939</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G5" s="40" t="s">
+        <v>1940</v>
+      </c>
+      <c r="H5" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="45" t="s">
+        <v>1941</v>
+      </c>
+      <c r="J5" s="45" t="s">
+        <v>1942</v>
+      </c>
+      <c r="K5" s="40" t="s">
+        <v>1943</v>
+      </c>
+      <c r="L5" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M5" s="41" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N5" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="16" customHeight="1">
+      <c r="A6" s="40" t="s">
+        <v>1944</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>1945</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>1946</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>1947</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F6" s="44" t="s">
+        <v>1868</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>1949</v>
+      </c>
+      <c r="H6" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="44" t="s">
+        <v>1950</v>
+      </c>
+      <c r="J6" s="44" t="s">
+        <v>1951</v>
+      </c>
+      <c r="K6" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L6" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M6" s="40" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N6" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="16" customHeight="1">
+      <c r="A7" s="40" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B7" s="38" t="s">
+        <v>1953</v>
+      </c>
+      <c r="C7" s="40" t="s">
+        <v>1954</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>1955</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>1956</v>
+      </c>
+      <c r="F7" s="40" t="s">
+        <v>1957</v>
+      </c>
+      <c r="G7" s="40" t="s">
+        <v>1958</v>
+      </c>
+      <c r="H7" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="48" t="s">
+        <v>1959</v>
+      </c>
+      <c r="J7" s="48" t="s">
+        <v>1960</v>
+      </c>
+      <c r="K7" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L7" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M7" s="40" t="s">
+        <v>1955</v>
+      </c>
+      <c r="N7" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="16" customHeight="1">
+      <c r="A8" s="40" t="s">
+        <v>1961</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>1962</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>1874</v>
+      </c>
+      <c r="D8" s="40" t="s">
+        <v>1963</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>1964</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>1965</v>
+      </c>
+      <c r="G8" s="40" t="s">
+        <v>1966</v>
+      </c>
+      <c r="H8" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="48" t="s">
+        <v>1967</v>
+      </c>
+      <c r="J8" s="38" t="s">
+        <v>1968</v>
+      </c>
+      <c r="K8" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L8" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M8" s="40" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N8" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="16" customHeight="1">
+      <c r="A9" s="40" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B9" s="38" t="s">
+        <v>1970</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>1971</v>
+      </c>
+      <c r="D9" s="40" t="s">
+        <v>1963</v>
+      </c>
+      <c r="E9" s="40" t="s">
+        <v>1972</v>
+      </c>
+      <c r="F9" s="40" t="s">
+        <v>1973</v>
+      </c>
+      <c r="G9" s="40" t="s">
+        <v>1974</v>
+      </c>
+      <c r="H9" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="48" t="s">
+        <v>1975</v>
+      </c>
+      <c r="J9" s="48" t="s">
+        <v>1976</v>
+      </c>
+      <c r="K9" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L9" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M9" s="40" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N9" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="16" customHeight="1">
+      <c r="A10" s="46" t="s">
+        <v>1977</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>1978</v>
+      </c>
+      <c r="C10" s="48" t="s">
+        <v>1979</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="47" t="s">
+        <v>1980</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>1981</v>
+      </c>
+      <c r="G10" s="46" t="s">
+        <v>1982</v>
+      </c>
+      <c r="H10" s="46" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="48" t="s">
+        <v>1983</v>
+      </c>
+      <c r="J10" s="38" t="s">
+        <v>1984</v>
+      </c>
+      <c r="K10" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L10" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M10" s="46" t="s">
+        <v>1985</v>
+      </c>
+      <c r="N10" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="16" customHeight="1">
+      <c r="A11" s="46" t="s">
+        <v>1986</v>
+      </c>
+      <c r="B11" s="38" t="s">
+        <v>1987</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>1988</v>
+      </c>
+      <c r="D11" s="47" t="s">
+        <v>1989</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>1990</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>1957</v>
+      </c>
+      <c r="G11" s="47" t="s">
+        <v>1991</v>
+      </c>
+      <c r="H11" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="48" t="s">
+        <v>1992</v>
+      </c>
+      <c r="J11" s="38" t="s">
+        <v>1993</v>
+      </c>
+      <c r="K11" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L11" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M11" s="46" t="s">
+        <v>1994</v>
+      </c>
+      <c r="N11" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16" customHeight="1">
+      <c r="A12" s="46" t="s">
+        <v>1995</v>
+      </c>
+      <c r="B12" s="38" t="s">
+        <v>1996</v>
+      </c>
+      <c r="C12" s="49" t="s">
+        <v>1997</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>1875</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>1998</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>1999</v>
+      </c>
+      <c r="G12" s="47" t="s">
+        <v>2000</v>
+      </c>
+      <c r="H12" s="46" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="48" t="s">
+        <v>2001</v>
+      </c>
+      <c r="J12" s="38" t="s">
+        <v>2002</v>
+      </c>
+      <c r="K12" s="40" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L12" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M12" s="40" t="s">
+        <v>1881</v>
+      </c>
+      <c r="N12" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I3" r:id="rId1" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
+    <hyperlink ref="I5" r:id="rId2" xr:uid="{00000000-0004-0000-0900-000001000000}"/>
+    <hyperlink ref="J5" r:id="rId3" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
+    <hyperlink ref="I7" r:id="rId4" xr:uid="{8F1A973E-B5AB-44F6-96AD-40713F29721B}"/>
+    <hyperlink ref="J7" r:id="rId5" display="https://www.mouser.es/ProductDetail/Vishay-Semiconductors/BZX55C5V1-TR?qs=WLTup5mM6hhy%252Bqloxl7%2FIQ%3D%3D&amp;utm_id=20109199436&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=emeacorp&amp;gad_source=1&amp;gad_campaignid=20109199436&amp;gbraid=0AAAAADn_wf2RhF_lSG_YlgnN1Yzlq3oak&amp;gclid=Cj0KCQiAhtvMBhDBARIsAL26pjE6pviBOpVaBUJ07A83YFMQUf7QkOHJpiHMP9nHJbQo8SvNA6LellYaAlJaEALw_wcB" xr:uid="{F2496565-AD95-4399-945A-CAC2965FBB51}"/>
+    <hyperlink ref="I8" r:id="rId6" xr:uid="{0E407122-DEDC-4464-8361-A36EA45E6AB5}"/>
+    <hyperlink ref="J9" r:id="rId7" xr:uid="{3E5FFD60-2B94-43D5-BD33-FCAB73A614C5}"/>
+    <hyperlink ref="I9" r:id="rId8" xr:uid="{FAF085BE-308D-4591-BB1A-0398244BD98C}"/>
+    <hyperlink ref="I10" r:id="rId9" xr:uid="{43EA2952-ABB5-4F52-94F7-A96F82DE8560}"/>
+    <hyperlink ref="I11" r:id="rId10" xr:uid="{E8167B89-7FBA-4877-BC25-3D4C05ED8AA6}"/>
+    <hyperlink ref="I12" r:id="rId11" xr:uid="{C4B46D5B-BD3F-4DBC-A61E-40C494B3D177}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="14.5" customHeight="1">
+      <c r="A1" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="51" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="51" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="51" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="51" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="51" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="52" t="s">
+        <v>2003</v>
+      </c>
+      <c r="B2" s="52" t="s">
+        <v>2004</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="55" t="s">
+        <v>2005</v>
+      </c>
+      <c r="E2" s="52" t="s">
+        <v>2006</v>
+      </c>
+      <c r="F2" s="52" t="s">
+        <v>2007</v>
+      </c>
+      <c r="G2" s="52" t="s">
+        <v>2008</v>
+      </c>
+      <c r="H2" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="52" t="s">
+        <v>2009</v>
+      </c>
+      <c r="J2" s="52" t="s">
+        <v>2010</v>
+      </c>
+      <c r="K2" s="52" t="s">
+        <v>2011</v>
+      </c>
+      <c r="L2" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="52" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B3" s="52" t="s">
+        <v>2013</v>
+      </c>
+      <c r="C3" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="52" t="s">
+        <v>2014</v>
+      </c>
+      <c r="E3" s="52" t="s">
+        <v>2015</v>
+      </c>
+      <c r="F3" s="52" t="s">
+        <v>2016</v>
+      </c>
+      <c r="G3" s="52" t="s">
+        <v>2017</v>
+      </c>
+      <c r="H3" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="53" t="s">
+        <v>2018</v>
+      </c>
+      <c r="J3" s="53" t="s">
+        <v>2019</v>
+      </c>
+      <c r="K3" s="52" t="s">
+        <v>2011</v>
+      </c>
+      <c r="L3" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M3" s="52" t="s">
+        <v>2014</v>
+      </c>
+      <c r="N3" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="52" t="s">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>2021</v>
+      </c>
+      <c r="C4" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="52" t="s">
+        <v>2022</v>
+      </c>
+      <c r="F4" s="52" t="s">
+        <v>2023</v>
+      </c>
+      <c r="G4" s="52" t="s">
+        <v>2024</v>
+      </c>
+      <c r="H4" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="57" t="s">
+        <v>2025</v>
+      </c>
+      <c r="J4" s="57" t="s">
+        <v>2026</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>2011</v>
+      </c>
+      <c r="L4" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M4" s="52" t="s">
+        <v>2027</v>
+      </c>
+      <c r="N4" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="52" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>2029</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="52" t="s">
+        <v>2030</v>
+      </c>
+      <c r="E5" s="59" t="s">
+        <v>2031</v>
+      </c>
+      <c r="F5" s="52" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G5" s="52" t="s">
+        <v>2032</v>
+      </c>
+      <c r="H5" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="57" t="s">
+        <v>2033</v>
+      </c>
+      <c r="J5" s="57" t="s">
+        <v>2034</v>
+      </c>
+      <c r="K5" s="52" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L5" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M5" s="52" t="s">
+        <v>2030</v>
+      </c>
+      <c r="N5" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="52" t="s">
+        <v>2035</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>2036</v>
+      </c>
+      <c r="C6" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>2037</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>2038</v>
+      </c>
+      <c r="F6" s="52" t="s">
+        <v>2039</v>
+      </c>
+      <c r="G6" s="52" t="s">
+        <v>2040</v>
+      </c>
+      <c r="H6" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="57" t="s">
+        <v>2041</v>
+      </c>
+      <c r="J6" s="57" t="s">
+        <v>2042</v>
+      </c>
+      <c r="K6" s="52" t="s">
+        <v>2043</v>
+      </c>
+      <c r="L6" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M6" s="52" t="s">
+        <v>2044</v>
+      </c>
+      <c r="N6" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="52" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>2046</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>2047</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>2048</v>
+      </c>
+      <c r="F7" s="52" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G7" s="52" t="s">
+        <v>2049</v>
+      </c>
+      <c r="H7" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="52" t="s">
+        <v>2050</v>
+      </c>
+      <c r="J7" s="52" t="s">
+        <v>2051</v>
+      </c>
+      <c r="K7" s="52" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L7" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M7" s="52" t="s">
+        <v>2047</v>
+      </c>
+      <c r="N7" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="52" t="s">
+        <v>2053</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>2054</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>1947</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>2055</v>
+      </c>
+      <c r="F8" s="52" t="s">
+        <v>2056</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>2057</v>
+      </c>
+      <c r="H8" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="52" t="s">
+        <v>2058</v>
+      </c>
+      <c r="J8" s="57" t="s">
+        <v>2059</v>
+      </c>
+      <c r="K8" s="52" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L8" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M8" s="52" t="s">
+        <v>2060</v>
+      </c>
+      <c r="N8" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="52" t="s">
+        <v>2061</v>
+      </c>
+      <c r="B9" s="52" t="s">
+        <v>2062</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>1947</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>2063</v>
+      </c>
+      <c r="F9" s="52" t="s">
+        <v>2064</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>2065</v>
+      </c>
+      <c r="H9" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="57" t="s">
+        <v>2066</v>
+      </c>
+      <c r="J9" s="57" t="s">
+        <v>2067</v>
+      </c>
+      <c r="K9" s="52" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L9" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M9" s="52" t="s">
+        <v>1947</v>
+      </c>
+      <c r="N9" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="52" t="s">
+        <v>2068</v>
+      </c>
+      <c r="B10" s="52" t="s">
+        <v>2069</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>2070</v>
+      </c>
+      <c r="E10" s="52" t="s">
+        <v>2070</v>
+      </c>
+      <c r="F10" s="52" t="s">
+        <v>1981</v>
+      </c>
+      <c r="G10" s="52" t="s">
+        <v>2071</v>
+      </c>
+      <c r="H10" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="52" t="s">
+        <v>2072</v>
+      </c>
+      <c r="J10" s="52" t="s">
+        <v>2073</v>
+      </c>
+      <c r="K10" s="52" t="s">
+        <v>2074</v>
+      </c>
+      <c r="L10" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M10" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N10" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="52" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B11" s="52" t="s">
+        <v>2076</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E11" s="52" t="s">
+        <v>2077</v>
+      </c>
+      <c r="F11" s="52" t="s">
+        <v>945</v>
+      </c>
+      <c r="G11" s="52" t="s">
+        <v>2078</v>
+      </c>
+      <c r="H11" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="52" t="s">
+        <v>2079</v>
+      </c>
+      <c r="J11" s="52" t="s">
+        <v>2080</v>
+      </c>
+      <c r="K11" s="52" t="s">
+        <v>2081</v>
+      </c>
+      <c r="L11" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M11" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N11" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="52" t="s">
+        <v>2082</v>
+      </c>
+      <c r="B12" s="52" t="s">
+        <v>2083</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>2084</v>
+      </c>
+      <c r="F12" s="52" t="s">
+        <v>2085</v>
+      </c>
+      <c r="G12" s="52" t="s">
+        <v>2086</v>
+      </c>
+      <c r="H12" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="52" t="s">
+        <v>2087</v>
+      </c>
+      <c r="J12" s="52" t="s">
+        <v>2088</v>
+      </c>
+      <c r="K12" s="52" t="s">
+        <v>2074</v>
+      </c>
+      <c r="L12" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M12" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N12" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="13.5" customHeight="1">
+      <c r="A13" s="52" t="s">
+        <v>2089</v>
+      </c>
+      <c r="B13" s="52" t="s">
+        <v>2090</v>
+      </c>
+      <c r="C13" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="52" t="s">
+        <v>2091</v>
+      </c>
+      <c r="E13" s="52" t="s">
+        <v>2092</v>
+      </c>
+      <c r="F13" s="52" t="s">
+        <v>2007</v>
+      </c>
+      <c r="G13" s="52" t="s">
+        <v>2093</v>
+      </c>
+      <c r="H13" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="54" t="s">
+        <v>2094</v>
+      </c>
+      <c r="J13" s="54" t="s">
+        <v>2095</v>
+      </c>
+      <c r="K13" s="52" t="s">
+        <v>2096</v>
+      </c>
+      <c r="L13" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M13" s="52" t="s">
+        <v>2091</v>
+      </c>
+      <c r="N13" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15" customHeight="1">
+      <c r="A14" s="52" t="s">
+        <v>2097</v>
+      </c>
+      <c r="B14" s="56" t="s">
+        <v>2098</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>2099</v>
+      </c>
+      <c r="E14" s="52">
+        <v>824012823</v>
+      </c>
+      <c r="F14" s="52" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G14" s="52" t="s">
+        <v>2101</v>
+      </c>
+      <c r="H14" s="52" t="s">
+        <v>2102</v>
+      </c>
+      <c r="I14" s="57" t="s">
+        <v>2103</v>
+      </c>
+      <c r="J14" s="57" t="s">
+        <v>2104</v>
+      </c>
+      <c r="K14" s="52">
+        <v>824012823</v>
+      </c>
+      <c r="L14" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M14" s="52" t="s">
+        <v>2105</v>
+      </c>
+      <c r="N14" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="52" t="s">
+        <v>2106</v>
+      </c>
+      <c r="B15" s="52" t="s">
+        <v>2107</v>
+      </c>
+      <c r="C15" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E15" s="52" t="s">
+        <v>2108</v>
+      </c>
+      <c r="F15" s="52" t="s">
+        <v>2085</v>
+      </c>
+      <c r="G15" s="52" t="s">
+        <v>2109</v>
+      </c>
+      <c r="H15" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="54" t="s">
+        <v>2110</v>
+      </c>
+      <c r="J15" s="54" t="s">
+        <v>2111</v>
+      </c>
+      <c r="K15" s="52" t="s">
+        <v>1943</v>
+      </c>
+      <c r="L15" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M15" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N15" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="52" t="s">
+        <v>2112</v>
+      </c>
+      <c r="B16" s="52" t="s">
+        <v>2113</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E16" s="52" t="s">
+        <v>2114</v>
+      </c>
+      <c r="F16" s="52" t="s">
+        <v>2023</v>
+      </c>
+      <c r="G16" s="52" t="s">
+        <v>2115</v>
+      </c>
+      <c r="H16" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" s="54" t="s">
+        <v>2116</v>
+      </c>
+      <c r="J16" s="54" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K16" s="52" t="s">
+        <v>2117</v>
+      </c>
+      <c r="L16" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M16" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N16" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="52" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B17" s="52" t="s">
+        <v>2119</v>
+      </c>
+      <c r="C17" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>2120</v>
+      </c>
+      <c r="E17" s="52" t="s">
+        <v>2121</v>
+      </c>
+      <c r="F17" s="52" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G17" s="52" t="s">
+        <v>2122</v>
+      </c>
+      <c r="H17" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="54" t="s">
+        <v>2123</v>
+      </c>
+      <c r="J17" s="54" t="s">
+        <v>2124</v>
+      </c>
+      <c r="K17" s="52" t="s">
+        <v>2125</v>
+      </c>
+      <c r="L17" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M17" s="52" t="s">
+        <v>2120</v>
+      </c>
+      <c r="N17" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="52" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B18" s="52" t="s">
+        <v>2127</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E18" s="52" t="s">
+        <v>2128</v>
+      </c>
+      <c r="F18" s="58" t="s">
+        <v>2129</v>
+      </c>
+      <c r="G18" s="58" t="s">
+        <v>2130</v>
+      </c>
+      <c r="H18" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="58" t="s">
+        <v>2131</v>
+      </c>
+      <c r="J18" s="58" t="s">
+        <v>2132</v>
+      </c>
+      <c r="K18" s="52" t="s">
+        <v>1943</v>
+      </c>
+      <c r="L18" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M18" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N18" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="52" t="s">
+        <v>2133</v>
+      </c>
+      <c r="B19" s="50" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C19" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="50" t="s">
+        <v>2135</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>2136</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>2137</v>
+      </c>
+      <c r="H19" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="50" t="s">
+        <v>2138</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>2139</v>
+      </c>
+      <c r="K19" s="52" t="s">
+        <v>2136</v>
+      </c>
+      <c r="L19" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M19" s="52" t="s">
+        <v>2136</v>
+      </c>
+      <c r="N19" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" s="52" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B20" s="50" t="s">
+        <v>2141</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="50" t="s">
+        <v>2142</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>2143</v>
+      </c>
+      <c r="F20" s="50" t="s">
+        <v>1658</v>
+      </c>
+      <c r="G20" s="50" t="s">
+        <v>2144</v>
+      </c>
+      <c r="H20" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" s="50" t="s">
+        <v>2145</v>
+      </c>
+      <c r="J20" s="50" t="s">
+        <v>2146</v>
+      </c>
+      <c r="K20" s="50" t="s">
+        <v>2143</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M20" s="50" t="s">
+        <v>2147</v>
+      </c>
+      <c r="N20" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" s="59" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B21" s="50" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C21" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="50" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>2150</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G21" s="50" t="s">
+        <v>2151</v>
+      </c>
+      <c r="H21" s="59" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" s="61" t="s">
+        <v>2152</v>
+      </c>
+      <c r="J21" s="50" t="s">
+        <v>2153</v>
+      </c>
+      <c r="K21" s="60" t="s">
+        <v>2154</v>
+      </c>
+      <c r="L21" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M21" s="52" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N21" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="59" t="s">
+        <v>2155</v>
+      </c>
+      <c r="B22" s="50" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="52" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F22" s="50" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G22" s="50" t="s">
+        <v>2159</v>
+      </c>
+      <c r="H22" s="59" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" s="50" t="s">
+        <v>2160</v>
+      </c>
+      <c r="J22" s="50" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K22" s="50" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L22" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M22" s="52" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N22" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="59" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B23" s="50" t="s">
+        <v>2163</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="52" t="s">
+        <v>1947</v>
+      </c>
+      <c r="E23" s="50" t="s">
+        <v>2164</v>
+      </c>
+      <c r="F23" s="50" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G23" s="50" t="s">
+        <v>2165</v>
+      </c>
+      <c r="H23" s="59" t="s">
+        <v>69</v>
+      </c>
+      <c r="I23" s="50" t="s">
+        <v>2166</v>
+      </c>
+      <c r="J23" s="61" t="s">
+        <v>2167</v>
+      </c>
+      <c r="K23" s="52" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M23" s="52" t="s">
+        <v>2060</v>
+      </c>
+      <c r="N23" s="52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I3" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
+    <hyperlink ref="J3" r:id="rId2" xr:uid="{00000000-0004-0000-0A00-000001000000}"/>
+    <hyperlink ref="I4" r:id="rId3" xr:uid="{00000000-0004-0000-0A00-000002000000}"/>
+    <hyperlink ref="J4" r:id="rId4" xr:uid="{00000000-0004-0000-0A00-000003000000}"/>
+    <hyperlink ref="I5" r:id="rId5" xr:uid="{00000000-0004-0000-0A00-000004000000}"/>
+    <hyperlink ref="J5" r:id="rId6" xr:uid="{00000000-0004-0000-0A00-000005000000}"/>
+    <hyperlink ref="I6" r:id="rId7" xr:uid="{00000000-0004-0000-0A00-000006000000}"/>
+    <hyperlink ref="J6" r:id="rId8" xr:uid="{00000000-0004-0000-0A00-000007000000}"/>
+    <hyperlink ref="J8" r:id="rId9" xr:uid="{00000000-0004-0000-0A00-000008000000}"/>
+    <hyperlink ref="I9" r:id="rId10" xr:uid="{00000000-0004-0000-0A00-000009000000}"/>
+    <hyperlink ref="J9" r:id="rId11" xr:uid="{00000000-0004-0000-0A00-00000A000000}"/>
+    <hyperlink ref="I13" r:id="rId12" xr:uid="{00000000-0004-0000-0A00-00000B000000}"/>
+    <hyperlink ref="J13" r:id="rId13" xr:uid="{00000000-0004-0000-0A00-00000C000000}"/>
+    <hyperlink ref="I14" r:id="rId14" xr:uid="{00000000-0004-0000-0A00-00000D000000}"/>
+    <hyperlink ref="J14" r:id="rId15" xr:uid="{00000000-0004-0000-0A00-00000E000000}"/>
+    <hyperlink ref="I15" r:id="rId16" xr:uid="{00000000-0004-0000-0A00-00000F000000}"/>
+    <hyperlink ref="J15" r:id="rId17" xr:uid="{00000000-0004-0000-0A00-000010000000}"/>
+    <hyperlink ref="I16" r:id="rId18" xr:uid="{00000000-0004-0000-0A00-000011000000}"/>
+    <hyperlink ref="J16" r:id="rId19" xr:uid="{00000000-0004-0000-0A00-000012000000}"/>
+    <hyperlink ref="I17" r:id="rId20" xr:uid="{00000000-0004-0000-0A00-000013000000}"/>
+    <hyperlink ref="J17" r:id="rId21" xr:uid="{00000000-0004-0000-0A00-000014000000}"/>
+    <hyperlink ref="I21" r:id="rId22" xr:uid="{E5D95628-DADF-425D-8DC6-0740E7A281C6}"/>
+    <hyperlink ref="J23" r:id="rId23" xr:uid="{21B09737-BF9A-463D-87B2-ED444DC9196C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="13" max="13" width="13.36328125" customWidth="1"/>
     <col min="14" max="14" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -16086,7 +19800,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -16130,15 +19844,879 @@
         <v>25</v>
       </c>
     </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>1694</v>
+      </c>
+      <c r="D3" s="26">
+        <v>1206</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>1695</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>1697</v>
+      </c>
+      <c r="H3" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>1698</v>
+      </c>
+      <c r="J3" s="23" t="s">
+        <v>1699</v>
+      </c>
+      <c r="K3" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" s="23"/>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>1702</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>1705</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>1706</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>1707</v>
+      </c>
+      <c r="J4" s="23" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K4" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" s="23" t="s">
+        <v>1709</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="23"/>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>1815</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>1710</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D5" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>1712</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>1691</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>1712</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>1713</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>1714</v>
+      </c>
+      <c r="K5" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L5" t="s">
+        <v>55</v>
+      </c>
+      <c r="M5" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+      <c r="O5" s="22"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>1816</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>1716</v>
+      </c>
+      <c r="D6" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>1717</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>1718</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>1717</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="24" t="s">
+        <v>1719</v>
+      </c>
+      <c r="J6" s="24" t="s">
+        <v>1720</v>
+      </c>
+      <c r="K6" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+      <c r="O6" s="22"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>1721</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>1722</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>1723</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>1724</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="25" t="s">
+        <v>1725</v>
+      </c>
+      <c r="J7" s="25" t="s">
+        <v>1726</v>
+      </c>
+      <c r="K7" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L7" t="s">
+        <v>55</v>
+      </c>
+      <c r="M7" s="25" t="s">
+        <v>1727</v>
+      </c>
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O7" s="22"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" t="s">
+        <v>1818</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>1728</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D8" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>1729</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>1730</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>1731</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="25" t="s">
+        <v>1732</v>
+      </c>
+      <c r="J8" s="25" t="s">
+        <v>1733</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L8" t="s">
+        <v>55</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O8" s="22"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>1819</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>1734</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D9" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>1735</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>1730</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>1736</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="25" t="s">
+        <v>1737</v>
+      </c>
+      <c r="J9" s="25" t="s">
+        <v>1738</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L9" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" s="22"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>1740</v>
+      </c>
+      <c r="D10" s="23">
+        <v>1812</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>1741</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>1743</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="24" t="s">
+        <v>1744</v>
+      </c>
+      <c r="J10" s="24" t="s">
+        <v>1745</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L10" t="s">
+        <v>55</v>
+      </c>
+      <c r="M10" s="23" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O10" s="22"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" t="s">
+        <v>1821</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>1748</v>
+      </c>
+      <c r="D11" s="23">
+        <v>1812</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>1750</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="22" t="s">
+        <v>1751</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>1752</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L11" t="s">
+        <v>55</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N11" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" s="22"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
+        <v>1822</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>1757</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>1758</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="29" t="s">
+        <v>1759</v>
+      </c>
+      <c r="J12" s="29" t="s">
+        <v>1760</v>
+      </c>
+      <c r="K12" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L12" t="s">
+        <v>55</v>
+      </c>
+      <c r="M12" s="28" t="s">
+        <v>1761</v>
+      </c>
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" s="22"/>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D13" s="22">
+        <v>1812</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>1764</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G13" s="28" t="s">
+        <v>1765</v>
+      </c>
+      <c r="H13" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="29" t="s">
+        <v>1766</v>
+      </c>
+      <c r="J13" s="29" t="s">
+        <v>1767</v>
+      </c>
+      <c r="K13" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L13" t="s">
+        <v>55</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N13" t="s">
+        <v>25</v>
+      </c>
+      <c r="O13" s="22"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D14" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>1770</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="22" t="s">
+        <v>1771</v>
+      </c>
+      <c r="J14" s="29" t="s">
+        <v>1772</v>
+      </c>
+      <c r="K14" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L14" t="s">
+        <v>55</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N14" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="22"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" t="s">
+        <v>1825</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1206</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>1775</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>1776</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>1777</v>
+      </c>
+      <c r="H15" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="22" t="s">
+        <v>1778</v>
+      </c>
+      <c r="J15" s="22" t="s">
+        <v>1779</v>
+      </c>
+      <c r="K15" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L15" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>1780</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>1781</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>1782</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="22" t="s">
+        <v>1783</v>
+      </c>
+      <c r="J16" s="22" t="s">
+        <v>1784</v>
+      </c>
+      <c r="K16" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M16" s="27" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="s">
+        <v>1827</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>1788</v>
+      </c>
+      <c r="H17" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="22" t="s">
+        <v>1789</v>
+      </c>
+      <c r="J17" s="22" t="s">
+        <v>1783</v>
+      </c>
+      <c r="K17" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M17" s="27" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>1790</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>1791</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>1792</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>1793</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="22" t="s">
+        <v>1794</v>
+      </c>
+      <c r="J18" s="22" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K18" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L18" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="27" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" t="s">
+        <v>1829</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>1796</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D19" s="22">
+        <v>1812</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>1797</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>1798</v>
+      </c>
+      <c r="H19" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="29" t="s">
+        <v>1799</v>
+      </c>
+      <c r="J19" s="22" t="s">
+        <v>1800</v>
+      </c>
+      <c r="K19" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L19" t="s">
+        <v>55</v>
+      </c>
+      <c r="M19" s="23" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>1801</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>1802</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>1803</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>1804</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" s="29" t="s">
+        <v>1805</v>
+      </c>
+      <c r="J20" s="29" t="s">
+        <v>1806</v>
+      </c>
+      <c r="K20" s="28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L20" t="s">
+        <v>55</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>1807</v>
+      </c>
+      <c r="N20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>1808</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D21" s="23">
+        <v>1812</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>1809</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>1810</v>
+      </c>
+      <c r="H21" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" s="22" t="s">
+        <v>1811</v>
+      </c>
+      <c r="J21" s="29" t="s">
+        <v>1812</v>
+      </c>
+      <c r="K21" s="23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L21" t="s">
+        <v>55</v>
+      </c>
+      <c r="M21" s="23" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{3DE7E9B7-7F71-48BD-A43F-56652EF48515}"/>
+    <hyperlink ref="I5" r:id="rId2" xr:uid="{00000000-0004-0000-0C00-000001000000}"/>
+    <hyperlink ref="J5" r:id="rId3" xr:uid="{00000000-0004-0000-0C00-000002000000}"/>
+    <hyperlink ref="I6" r:id="rId4" xr:uid="{00000000-0004-0000-0C00-000003000000}"/>
+    <hyperlink ref="J6" r:id="rId5" xr:uid="{00000000-0004-0000-0C00-000004000000}"/>
+    <hyperlink ref="I10" r:id="rId6" xr:uid="{00000000-0004-0000-0C00-000005000000}"/>
+    <hyperlink ref="J10" r:id="rId7" xr:uid="{00000000-0004-0000-0C00-000006000000}"/>
+    <hyperlink ref="I12" r:id="rId8" xr:uid="{DC4D0F7D-FABA-4F27-A8C4-C8F1159FEA34}"/>
+    <hyperlink ref="J12" r:id="rId9" xr:uid="{7C1A203F-2505-4DF3-8487-119DA9DE1A1B}"/>
+    <hyperlink ref="J13" r:id="rId10" xr:uid="{6F374EEE-953D-426D-AF07-D3E5C1F03D55}"/>
+    <hyperlink ref="I13" r:id="rId11" xr:uid="{959671DE-63B1-4C42-9AE2-A4D45EAFA482}"/>
+    <hyperlink ref="J14" r:id="rId12" xr:uid="{D0E41C99-5015-461D-998D-DD06CC299D2B}"/>
+    <hyperlink ref="I19" r:id="rId13" xr:uid="{EAFB85FD-4F43-4B6C-AEDE-D6E5C0E93BD1}"/>
+    <hyperlink ref="I20" r:id="rId14" xr:uid="{6C9DFF48-0956-4B25-8972-EC0656F1483E}"/>
+    <hyperlink ref="J20" r:id="rId15" xr:uid="{6EF40273-C6D8-4BC3-9EF6-1B4C76903848}"/>
+    <hyperlink ref="J21" r:id="rId16" xr:uid="{FFB17F08-401F-47B0-899B-612CD8B9FB6B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -16386,252 +20964,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
-  <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="4" max="4" width="17.54296875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1669</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1670</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1671</v>
-      </c>
-      <c r="E2" t="s">
-        <v>1674</v>
-      </c>
-      <c r="F2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G2" t="s">
-        <v>1675</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>1672</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>1673</v>
-      </c>
-      <c r="K2" t="s">
-        <v>1676</v>
-      </c>
-      <c r="L2" t="s">
-        <v>1689</v>
-      </c>
-      <c r="M2" t="s">
-        <v>1676</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
-        <v>1677</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1678</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1679</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1671</v>
-      </c>
-      <c r="E3" t="s">
-        <v>1680</v>
-      </c>
-      <c r="F3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" t="s">
-        <v>1681</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>1672</v>
-      </c>
-      <c r="J3" t="s">
-        <v>1682</v>
-      </c>
-      <c r="K3" t="s">
-        <v>1676</v>
-      </c>
-      <c r="L3" t="s">
-        <v>1689</v>
-      </c>
-      <c r="M3" t="s">
-        <v>1676</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" t="s">
-        <v>1683</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1684</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1685</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1671</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1686</v>
-      </c>
-      <c r="F4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G4" t="s">
-        <v>1687</v>
-      </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" t="s">
-        <v>1672</v>
-      </c>
-      <c r="J4" t="s">
-        <v>1688</v>
-      </c>
-      <c r="K4" t="s">
-        <v>1676</v>
-      </c>
-      <c r="L4" t="s">
-        <v>1689</v>
-      </c>
-      <c r="M4" t="s">
-        <v>1676</v>
-      </c>
-      <c r="N4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{08280A44-0F58-4FDE-B5FD-3A95A0F423CB}"/>
-    <hyperlink ref="J2" r:id="rId2" xr:uid="{85F326FF-BAE0-4072-815D-1EE4E7995C53}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
110-0055 and 110-0056 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A235B2DA-ECEA-46D4-91B3-71E35DD00E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC46636A-9846-467B-9B7C-C4FB9965F905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5356" uniqueCount="2585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5380" uniqueCount="2597">
   <si>
     <t>ID</t>
   </si>
@@ -7792,6 +7792,42 @@
   </si>
   <si>
     <t>Pleeda_PcbLibrary/Pleeda_PcbLibrary.PcbLib</t>
+  </si>
+  <si>
+    <t>110-0055</t>
+  </si>
+  <si>
+    <t>110-0056</t>
+  </si>
+  <si>
+    <t>Pluggable Terminal Blocks 12 Pos 3.5mm pitch Plug 24-16AWG Spring</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Phoenix-Contact/1844317?qs=p6trItWzfMW9CXyhJ87RMQ%3D%3D</t>
+  </si>
+  <si>
+    <t>12P</t>
+  </si>
+  <si>
+    <t>THT 3,5mm</t>
+  </si>
+  <si>
+    <t>Pluggable Terminal Blocks 12 Pos 3.5mm pitch Through Hole Header</t>
+  </si>
+  <si>
+    <t>651-1844317</t>
+  </si>
+  <si>
+    <t>651-1952364</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/507/9/phoenix_contact_1844317_en.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Phoenix-Contact/1952364?qs=6i0QExrCb7PyJNJO9S2%2Ffw%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/507/9/phoenix_contact_1952364_en.pdf</t>
   </si>
 </sst>
 </file>
@@ -7961,7 +7997,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8006,6 +8042,7 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -12910,7 +12947,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -15330,6 +15367,94 @@
         <v>1804920</v>
       </c>
       <c r="N55" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
+      <c r="A56" s="16" t="s">
+        <v>2585</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2591</v>
+      </c>
+      <c r="C56" s="28" t="s">
+        <v>2589</v>
+      </c>
+      <c r="D56" s="16" t="s">
+        <v>2590</v>
+      </c>
+      <c r="E56">
+        <v>1844317</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>2281</v>
+      </c>
+      <c r="G56" s="28" t="s">
+        <v>2592</v>
+      </c>
+      <c r="H56" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I56" s="27" t="s">
+        <v>2594</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>2588</v>
+      </c>
+      <c r="K56" s="7" t="s">
+        <v>2441</v>
+      </c>
+      <c r="L56" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M56">
+        <v>1844317</v>
+      </c>
+      <c r="N56" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
+      <c r="A57" s="16" t="s">
+        <v>2586</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2587</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2589</v>
+      </c>
+      <c r="D57" s="16" t="s">
+        <v>2590</v>
+      </c>
+      <c r="E57">
+        <v>1952364</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>2281</v>
+      </c>
+      <c r="G57" t="s">
+        <v>2593</v>
+      </c>
+      <c r="H57" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57" s="27" t="s">
+        <v>2596</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>2595</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>2540</v>
+      </c>
+      <c r="L57" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M57">
+        <v>1952364</v>
+      </c>
+      <c r="N57" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -15385,6 +15510,10 @@
     <hyperlink ref="J52" r:id="rId47" xr:uid="{E897E496-BD4D-4176-A529-0242E26116CB}"/>
     <hyperlink ref="I52" r:id="rId48" xr:uid="{A225907D-3E4C-4582-95BF-8DEDA99E88ED}"/>
     <hyperlink ref="I55" r:id="rId49" xr:uid="{A1002F44-75AF-44AC-BBCA-828DA38BB4E6}"/>
+    <hyperlink ref="J56" r:id="rId50" xr:uid="{8195B8EC-E2EB-40EB-9C49-2D817013AE1F}"/>
+    <hyperlink ref="I56" r:id="rId51" xr:uid="{CE941FB5-1D41-41B6-9CFD-C1256871C52E}"/>
+    <hyperlink ref="J57" r:id="rId52" xr:uid="{72ED46D3-1227-48FD-9800-7E78EA501F81}"/>
+    <hyperlink ref="I57" r:id="rId53" xr:uid="{30F29B76-2559-4C1E-A762-9F9E7C2882A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22651,6 +22780,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E65951-BFD2-4888-A0A6-19D5130CB4A6}">
   <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="41.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="25" t="s">

</xml_diff>

<commit_message>
110-0057, 110-0058, 110-0059, 110-0060 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D62A594-312B-4529-ABA1-0D99DBEEA679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD01ACC6-B416-44F9-9ABC-893A0914DBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25812" yWindow="2904" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5716" uniqueCount="2878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5760" uniqueCount="2896">
   <si>
     <t>ID</t>
   </si>
@@ -8672,6 +8672,60 @@
   </si>
   <si>
     <t>eUSR_SchLibrary/eUSR_SchLibrary - LEDs.SchLib</t>
+  </si>
+  <si>
+    <t>110-0057</t>
+  </si>
+  <si>
+    <t>110-0058</t>
+  </si>
+  <si>
+    <t>110-0059</t>
+  </si>
+  <si>
+    <t>110-0060</t>
+  </si>
+  <si>
+    <t>WR-MPC5 Male Header Dual Row</t>
+  </si>
+  <si>
+    <t>THT 5,7mm</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/657012240101.pdf</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/en/components/products/WTB_WR_MPC5_DUAL_ROW</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/657012250201.pdf</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/en/components/products/WTB_WR_MPC5_RECEPTACLE_PLUG_DUAL_ROW#/articles/WTB_WR_MCP5_DUAL_ROW_RECEPTACLE_HOUSING</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/657004140101.pdf</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/en/components/products/WTB_WR_MPC5_SINGLE_ROW</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/657004150201.pdf</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/en/components/products/WTB_WR_MPC5_RECEPTACLE_PLUG_SINGLE_ROW#/articles/WTB_WR_MPC5_SINGLE_ROW_RECEPTACLE_HOUSING</t>
+  </si>
+  <si>
+    <t>WR-MPC5 Receptacle Dual Row</t>
+  </si>
+  <si>
+    <t>WR-MPC5 Male Header Single Row</t>
+  </si>
+  <si>
+    <t>Receptacle Single Row</t>
+  </si>
+  <si>
+    <t>CONN 14P</t>
   </si>
 </sst>
 </file>
@@ -8841,7 +8895,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8890,6 +8944,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -14877,8 +14934,13 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="5" max="5" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="25" t="s">
@@ -17385,6 +17447,182 @@
         <v>1952364</v>
       </c>
       <c r="N57" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
+      <c r="A58" s="16" t="s">
+        <v>2878</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2882</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2587</v>
+      </c>
+      <c r="D58" s="16" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E58" s="30">
+        <v>657012240101</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G58" s="30">
+        <v>657012240101</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="I58" t="s">
+        <v>2884</v>
+      </c>
+      <c r="J58" t="s">
+        <v>2885</v>
+      </c>
+      <c r="K58" s="32" t="s">
+        <v>2895</v>
+      </c>
+      <c r="L58" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M58" s="30">
+        <v>657012240101</v>
+      </c>
+      <c r="N58" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
+      <c r="A59" s="16" t="s">
+        <v>2879</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2892</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2587</v>
+      </c>
+      <c r="D59" s="16" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E59" s="30">
+        <v>657012250201</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G59" s="30">
+        <v>657012250201</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="I59" t="s">
+        <v>2886</v>
+      </c>
+      <c r="J59" t="s">
+        <v>2887</v>
+      </c>
+      <c r="K59" s="3" t="s">
+        <v>2540</v>
+      </c>
+      <c r="L59" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M59" s="30">
+        <v>657012250201</v>
+      </c>
+      <c r="N59" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
+      <c r="A60" s="16" t="s">
+        <v>2880</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2893</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>2452</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E60" s="30">
+        <v>657004140101</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G60" s="30">
+        <v>657004140101</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="I60" t="s">
+        <v>2888</v>
+      </c>
+      <c r="J60" t="s">
+        <v>2889</v>
+      </c>
+      <c r="K60" s="32" t="s">
+        <v>2416</v>
+      </c>
+      <c r="L60" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M60" s="30">
+        <v>657004140101</v>
+      </c>
+      <c r="N60" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
+      <c r="A61" s="16" t="s">
+        <v>2881</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2894</v>
+      </c>
+      <c r="C61" s="16" t="s">
+        <v>2452</v>
+      </c>
+      <c r="D61" s="16" t="s">
+        <v>2883</v>
+      </c>
+      <c r="E61" s="30">
+        <v>657004150201</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G61" s="30">
+        <v>657004150201</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="I61" t="s">
+        <v>2890</v>
+      </c>
+      <c r="J61" t="s">
+        <v>2891</v>
+      </c>
+      <c r="K61" s="31" t="s">
+        <v>2540</v>
+      </c>
+      <c r="L61" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M61" s="30">
+        <v>657004150201</v>
+      </c>
+      <c r="N61" s="7" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Inductor CMM and Capacitors THT Electrol added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,25 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD01ACC6-B416-44F9-9ABC-893A0914DBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74AA2D8-E955-4948-8612-3823F2A6CDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
-    <sheet name="010 - Resistors - SMD" sheetId="4" r:id="rId2"/>
-    <sheet name="015 - Resistors - Shunt" sheetId="7" r:id="rId3"/>
-    <sheet name="020 - Inductor" sheetId="5" r:id="rId4"/>
-    <sheet name="030 - Diode - Rectifier" sheetId="9" r:id="rId5"/>
-    <sheet name="031 - Diode - Schottky" sheetId="11" r:id="rId6"/>
-    <sheet name="032 - Diode - TVS" sheetId="14" r:id="rId7"/>
-    <sheet name="033 - Diode - LED" sheetId="12" r:id="rId8"/>
-    <sheet name="040 - Fuses" sheetId="10" r:id="rId9"/>
-    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId10"/>
-    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId11"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId12"/>
-    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId13"/>
-    <sheet name="110 - Connectors" sheetId="13" r:id="rId14"/>
+    <sheet name="003 - Capacitors - THT Electrol" sheetId="17" r:id="rId2"/>
+    <sheet name="010 - Resistors - SMD" sheetId="4" r:id="rId3"/>
+    <sheet name="015 - Resistors - Shunt" sheetId="7" r:id="rId4"/>
+    <sheet name="020 - Inductor" sheetId="5" r:id="rId5"/>
+    <sheet name="023 - Inductor - CMM" sheetId="16" r:id="rId6"/>
+    <sheet name="030 - Diode - Rectifier" sheetId="9" r:id="rId7"/>
+    <sheet name="031 - Diode - Schottky" sheetId="11" r:id="rId8"/>
+    <sheet name="032 - Diode - TVS" sheetId="14" r:id="rId9"/>
+    <sheet name="033 - Diode - LED" sheetId="12" r:id="rId10"/>
+    <sheet name="040 - Fuses" sheetId="10" r:id="rId11"/>
+    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId12"/>
+    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId13"/>
+    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId14"/>
+    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId15"/>
+    <sheet name="110 - Connectors" sheetId="13" r:id="rId16"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5760" uniqueCount="2896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5814" uniqueCount="2916">
   <si>
     <t>ID</t>
   </si>
@@ -8726,6 +8728,66 @@
   </si>
   <si>
     <t>CONN 14P</t>
+  </si>
+  <si>
+    <t>023-0001</t>
+  </si>
+  <si>
+    <t>Common Mode Chokes / Filters WE-CMB Type XXL .5mH 35A 2.3mOhm</t>
+  </si>
+  <si>
+    <t>0.5mH 35A 2.3mOhm</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/7448263505?qs=2kOmHSv6VfR2wo62vNWXfg%3D%3D</t>
+  </si>
+  <si>
+    <t>47x43x23.5mm</t>
+  </si>
+  <si>
+    <t>710-7448263505</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/7448263505.pdf</t>
+  </si>
+  <si>
+    <t>IND CMM</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Inductor.SchLib</t>
+  </si>
+  <si>
+    <t>IND_CMM_THT_10x18.5mm</t>
+  </si>
+  <si>
+    <t>003-0001</t>
+  </si>
+  <si>
+    <t>Aluminium Electrolytic Capacitors - Radial Leaded WCAP-ATG5 470uF 50V 20% Radial</t>
+  </si>
+  <si>
+    <t>470uF 50V 20%</t>
+  </si>
+  <si>
+    <t>THT;D10xL20mm</t>
+  </si>
+  <si>
+    <t>Wurth Elektonik</t>
+  </si>
+  <si>
+    <t>710-860020675022</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/860020675022.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/860020675022?qs=0KOYDY2FL28clmrWTWQzzg%3D%3D</t>
+  </si>
+  <si>
+    <t>CAP polarized</t>
+  </si>
+  <si>
+    <t>CAP_10Dx20L</t>
   </si>
 </sst>
 </file>
@@ -8895,7 +8957,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8945,8 +9007,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -13352,6 +13413,2014 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="14.5" customHeight="1">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="7" t="s">
+        <v>2766</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>2767</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>2768</v>
+      </c>
+      <c r="D2" s="7">
+        <v>3535</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>2769</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>2770</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>2771</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>2772</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>2773</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>2775</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="7" t="s">
+        <v>2776</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>2777</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>2768</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>2778</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>2779</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>2780</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>2781</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>2782</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>2783</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="7" t="s">
+        <v>2784</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>2785</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>2786</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>2787</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>2788</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>2789</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>2790</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>2790</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>2783</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="7" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>2792</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>2793</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>2794</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>2795</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>2796</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>2797</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>2798</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>2783</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="7" t="s">
+        <v>2799</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>2800</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>2801</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>2802</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>2788</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>2803</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>2804</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>2805</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>2783</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="7" t="s">
+        <v>2806</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>2807</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>2808</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>2809</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>2810</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>2811</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>2812</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>2813</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>2814</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>2815</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>2816</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="7" t="s">
+        <v>2817</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>2818</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>2808</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>2819</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>2820</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>2821</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>2822</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>2823</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>2824</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>2825</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>2826</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="14.5" customHeight="1">
+      <c r="A9" s="7" t="s">
+        <v>2827</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>2828</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>2786</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>2829</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>2830</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>2831</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>2832</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>2833</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>2834</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>2835</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="7" t="s">
+        <v>2836</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>2837</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>2786</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>2838</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>2839</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>2840</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>2841</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>2842</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>2843</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="7" t="s">
+        <v>2844</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>2845</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>2846</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>2847</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>2848</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>2849</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>2850</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>2851</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>2843</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="7" t="s">
+        <v>2852</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>2808</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>2854</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>2855</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>2856</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>2857</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>2823</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>2858</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>2859</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>2815</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>2855</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="13.5" customHeight="1">
+      <c r="A13" s="7" t="s">
+        <v>2860</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>2861</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>2862</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>2863</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>2864</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>2865</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>2866</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>2867</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>2868</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>2869</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>2864</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15" customHeight="1">
+      <c r="A14" s="7" t="s">
+        <v>2870</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2871</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>2793</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>2872</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>2779</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>2873</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>2874</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>2875</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>2876</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="7" t="s">
+        <v>2106</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>2107</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>2108</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>2085</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>2109</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>2110</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>2111</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>1943</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="7" t="s">
+        <v>2112</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>2113</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>2114</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>2023</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>2115</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>2116</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>2116</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>2117</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="7" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>2119</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>2120</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>2121</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>2122</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>2123</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>2124</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>2125</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>2120</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="7" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>2127</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>2128</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>2129</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>2130</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>2131</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>2132</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>1943</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="7" t="s">
+        <v>2133</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>2135</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>2136</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>2137</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>2138</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>2139</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>2136</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>2136</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" s="7" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>2141</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>2142</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>2143</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>1658</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>2144</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>2145</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>2146</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>2143</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>2147</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" s="16" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>1856</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>2150</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>2151</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>2152</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>2153</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>2154</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="16" t="s">
+        <v>2155</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>2159</v>
+      </c>
+      <c r="H22" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>2160</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>2161</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>1904</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="16" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>2163</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>1947</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>2164</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>2165</v>
+      </c>
+      <c r="H23" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>2166</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>2167</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>2052</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>2060</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I15" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-00000F000000}"/>
+    <hyperlink ref="J15" r:id="rId2" xr:uid="{00000000-0004-0000-0A00-000010000000}"/>
+    <hyperlink ref="I16" r:id="rId3" xr:uid="{00000000-0004-0000-0A00-000011000000}"/>
+    <hyperlink ref="J16" r:id="rId4" xr:uid="{00000000-0004-0000-0A00-000012000000}"/>
+    <hyperlink ref="I17" r:id="rId5" xr:uid="{00000000-0004-0000-0A00-000013000000}"/>
+    <hyperlink ref="J17" r:id="rId6" xr:uid="{00000000-0004-0000-0A00-000014000000}"/>
+    <hyperlink ref="I21" r:id="rId7" xr:uid="{E5D95628-DADF-425D-8DC6-0740E7A281C6}"/>
+    <hyperlink ref="J23" r:id="rId8" xr:uid="{21B09737-BF9A-463D-87B2-ED444DC9196C}"/>
+    <hyperlink ref="J3" r:id="rId9" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
+    <hyperlink ref="I5" r:id="rId10" xr:uid="{00000000-0004-0000-0B00-000001000000}"/>
+    <hyperlink ref="J5" r:id="rId11" xr:uid="{00000000-0004-0000-0B00-000002000000}"/>
+    <hyperlink ref="I6" r:id="rId12" xr:uid="{00000000-0004-0000-0B00-000003000000}"/>
+    <hyperlink ref="J6" r:id="rId13" xr:uid="{00000000-0004-0000-0B00-000004000000}"/>
+    <hyperlink ref="F7" r:id="rId14" xr:uid="{00000000-0004-0000-0B00-000005000000}"/>
+    <hyperlink ref="I14" r:id="rId15" xr:uid="{BFE50862-7088-44B1-9DAF-F4C51270ACE8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="13" max="13" width="13.36328125" customWidth="1"/>
+    <col min="14" max="14" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1690</v>
+      </c>
+      <c r="L2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>1694</v>
+      </c>
+      <c r="D3" s="22">
+        <v>1206</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>1695</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>1697</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>1698</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>1699</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3" s="7"/>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>1702</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>1705</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>1706</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>1707</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>1709</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="7"/>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>1815</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>1710</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D5" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>1712</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>1691</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>1712</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>1713</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>1714</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L5" t="s">
+        <v>55</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>1816</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>1716</v>
+      </c>
+      <c r="D6" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>1717</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>1718</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>1717</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>1719</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>1720</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1721</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>1722</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>1723</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>1724</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>1725</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>1726</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L7" t="s">
+        <v>55</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>1727</v>
+      </c>
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" t="s">
+        <v>1818</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>1728</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D8" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>1729</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>1730</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>1731</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>1732</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>1733</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L8" t="s">
+        <v>55</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>1819</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1734</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>1735</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>1730</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>1736</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>1737</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>1738</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L9" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>1740</v>
+      </c>
+      <c r="D10" s="7">
+        <v>1812</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>1741</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>1743</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>1744</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>1745</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L10" t="s">
+        <v>55</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" t="s">
+        <v>1821</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>1748</v>
+      </c>
+      <c r="D11" s="7">
+        <v>1812</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>1750</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>1751</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>1752</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L11" t="s">
+        <v>55</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N11" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
+        <v>1822</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>1757</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>1758</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>1759</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>1760</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L12" t="s">
+        <v>55</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>1761</v>
+      </c>
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" s="3"/>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1812</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>1765</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>1766</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>1767</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L13" t="s">
+        <v>55</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N13" t="s">
+        <v>25</v>
+      </c>
+      <c r="O13" s="3"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D14" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>1771</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>1772</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L14" t="s">
+        <v>55</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N14" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="3"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" t="s">
+        <v>1825</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D15" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>1775</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>1776</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>1777</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>1778</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>1779</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L15" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>1780</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>1781</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>1782</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>1783</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>1784</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="s">
+        <v>1827</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>1788</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>1789</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>1783</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>1790</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>1791</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>1792</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>1793</v>
+      </c>
+      <c r="H18" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>1794</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K18" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L18" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>1785</v>
+      </c>
+      <c r="N18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" t="s">
+        <v>1829</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>1796</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1812</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>1797</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>1798</v>
+      </c>
+      <c r="H19" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>1799</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>1800</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L19" t="s">
+        <v>55</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>1801</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>1802</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>1803</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>1804</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>1805</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>1806</v>
+      </c>
+      <c r="K20" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L20" t="s">
+        <v>55</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>1807</v>
+      </c>
+      <c r="N20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>1808</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>1703</v>
+      </c>
+      <c r="D21" s="7">
+        <v>1812</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>1809</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>1810</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>1811</v>
+      </c>
+      <c r="J21" s="18" t="s">
+        <v>1812</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L21" t="s">
+        <v>55</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>1746</v>
+      </c>
+      <c r="N21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{3DE7E9B7-7F71-48BD-A43F-56652EF48515}"/>
+    <hyperlink ref="I5" r:id="rId2" xr:uid="{00000000-0004-0000-0C00-000001000000}"/>
+    <hyperlink ref="J5" r:id="rId3" xr:uid="{00000000-0004-0000-0C00-000002000000}"/>
+    <hyperlink ref="I6" r:id="rId4" xr:uid="{00000000-0004-0000-0C00-000003000000}"/>
+    <hyperlink ref="J6" r:id="rId5" xr:uid="{00000000-0004-0000-0C00-000004000000}"/>
+    <hyperlink ref="I10" r:id="rId6" xr:uid="{00000000-0004-0000-0C00-000005000000}"/>
+    <hyperlink ref="J10" r:id="rId7" xr:uid="{00000000-0004-0000-0C00-000006000000}"/>
+    <hyperlink ref="I12" r:id="rId8" xr:uid="{DC4D0F7D-FABA-4F27-A8C4-C8F1159FEA34}"/>
+    <hyperlink ref="J12" r:id="rId9" xr:uid="{7C1A203F-2505-4DF3-8487-119DA9DE1A1B}"/>
+    <hyperlink ref="J13" r:id="rId10" xr:uid="{6F374EEE-953D-426D-AF07-D3E5C1F03D55}"/>
+    <hyperlink ref="I13" r:id="rId11" xr:uid="{959671DE-63B1-4C42-9AE2-A4D45EAFA482}"/>
+    <hyperlink ref="J14" r:id="rId12" xr:uid="{D0E41C99-5015-461D-998D-DD06CC299D2B}"/>
+    <hyperlink ref="I19" r:id="rId13" xr:uid="{EAFB85FD-4F43-4B6C-AEDE-D6E5C0E93BD1}"/>
+    <hyperlink ref="I20" r:id="rId14" xr:uid="{6C9DFF48-0956-4B25-8972-EC0656F1483E}"/>
+    <hyperlink ref="J20" r:id="rId15" xr:uid="{6EF40273-C6D8-4BC3-9EF6-1B4C76903848}"/>
+    <hyperlink ref="J21" r:id="rId16" xr:uid="{FFB17F08-401F-47B0-899B-612CD8B9FB6B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -13601,7 +15670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -13655,7 +15724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
   <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -13849,7 +15918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -14932,7 +17001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
   <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -17481,7 +19550,7 @@
       <c r="J58" t="s">
         <v>2885</v>
       </c>
-      <c r="K58" s="32" t="s">
+      <c r="K58" s="31" t="s">
         <v>2895</v>
       </c>
       <c r="L58" s="7" t="s">
@@ -17569,7 +19638,7 @@
       <c r="J60" t="s">
         <v>2889</v>
       </c>
-      <c r="K60" s="32" t="s">
+      <c r="K60" s="31" t="s">
         <v>2416</v>
       </c>
       <c r="L60" s="7" t="s">
@@ -17613,7 +19682,7 @@
       <c r="J61" t="s">
         <v>2891</v>
       </c>
-      <c r="K61" s="31" t="s">
+      <c r="K61" s="3" t="s">
         <v>2540</v>
       </c>
       <c r="L61" s="7" t="s">
@@ -17688,6 +19757,113 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>2906</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2907</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2908</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2909</v>
+      </c>
+      <c r="E2">
+        <v>860020675022</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2910</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2911</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2912</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2913</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2914</v>
+      </c>
+      <c r="L2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" t="s">
+        <v>2915</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="M3" s="7"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{BB2EDAB8-75EB-46D2-BA14-384BF06E1A6E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
   <dimension ref="A1:N136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -23777,7 +25953,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -23927,7 +26103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C6B0FD-D8A3-44EC-9532-03DDA232F922}">
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -23981,7 +26157,108 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D956EFE-E955-4E62-8478-2294E6413DC1}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>2896</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2897</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2898</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2900</v>
+      </c>
+      <c r="E2">
+        <v>7448263505</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2901</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2902</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2899</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2903</v>
+      </c>
+      <c r="L2" t="s">
+        <v>2904</v>
+      </c>
+      <c r="M2" t="s">
+        <v>2905</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{1A9E4CB0-A8E7-4FC1-A9A7-FA5E28311F4C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652841DA-3619-42EE-A536-61B58BE1B457}">
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -24393,7 +26670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2008B-4BF4-4C9A-883A-FEE5873AEAF4}">
   <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -24944,7 +27221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E65951-BFD2-4888-A0A6-19D5130CB4A6}">
   <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -25964,2012 +28241,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
-  <dimension ref="A1:N23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:14" ht="14.5" customHeight="1">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="25" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="7" t="s">
-        <v>2766</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>2767</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>2768</v>
-      </c>
-      <c r="D2" s="7">
-        <v>3535</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>2769</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>2770</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>2771</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>2772</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>2773</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>2775</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" s="7" t="s">
-        <v>2776</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>2777</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>2768</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>2778</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>2779</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>2780</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>2781</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>2782</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>2783</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="7" t="s">
-        <v>2784</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>2785</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>2786</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>2787</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>2788</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>2789</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>2790</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>2790</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>2783</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5" s="7" t="s">
-        <v>2791</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>2792</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>2793</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>2794</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>2795</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>2796</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>2797</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>2798</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>2783</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="7" t="s">
-        <v>2799</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>2800</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>2801</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>2802</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>2788</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>2803</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>2804</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>2805</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>2783</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="7" t="s">
-        <v>2806</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>2807</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>2808</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>2809</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>2810</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>2811</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>2812</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>2813</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>2814</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>2815</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>2816</v>
-      </c>
-      <c r="N7" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="7" t="s">
-        <v>2817</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>2818</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>2808</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>2819</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>2820</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>2821</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>2822</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>2823</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>2824</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>2825</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>2826</v>
-      </c>
-      <c r="N8" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="14.5" customHeight="1">
-      <c r="A9" s="7" t="s">
-        <v>2827</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>2828</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>2786</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>2829</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>2830</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>2831</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>2832</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>2833</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>2834</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>2835</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="7" t="s">
-        <v>2836</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>2837</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>2786</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>2838</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>2839</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>2840</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>2841</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>2842</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L10" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>2843</v>
-      </c>
-      <c r="N10" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="7" t="s">
-        <v>2844</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>2845</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>2846</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>2847</v>
-      </c>
-      <c r="F11" s="17" t="s">
-        <v>2848</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>2849</v>
-      </c>
-      <c r="H11" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>2850</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>2851</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M11" s="16" t="s">
-        <v>2843</v>
-      </c>
-      <c r="N11" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="7" t="s">
-        <v>2852</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>2853</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>2808</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>2854</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>2855</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>2856</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>2857</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>2823</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>2858</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>2859</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>2815</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>2855</v>
-      </c>
-      <c r="N12" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>2860</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>2861</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>2862</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>2863</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>2864</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>2865</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>2866</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>2867</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>2868</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>2869</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>2864</v>
-      </c>
-      <c r="N13" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1">
-      <c r="A14" s="7" t="s">
-        <v>2870</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>2871</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>2793</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>2872</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>2779</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>2873</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>2874</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>2875</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>2774</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>2876</v>
-      </c>
-      <c r="N14" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="7" t="s">
-        <v>2106</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>2107</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>2108</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>2085</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>2109</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>2110</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>2111</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>1943</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="A16" s="7" t="s">
-        <v>2112</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>2113</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>2114</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>2023</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>2115</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>2116</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>2116</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>2117</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M16" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="N16" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14">
-      <c r="A17" s="7" t="s">
-        <v>2118</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>2119</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>2120</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>2121</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>1877</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>2122</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>2123</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>2124</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>2125</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M17" s="7" t="s">
-        <v>2120</v>
-      </c>
-      <c r="N17" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
-      <c r="A18" s="7" t="s">
-        <v>2126</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>2127</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>2128</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>2129</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>2130</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>2131</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>2132</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>1943</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
-      <c r="A19" s="7" t="s">
-        <v>2133</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>2134</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>2135</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>2136</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>2137</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>2138</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>2139</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>2136</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>2136</v>
-      </c>
-      <c r="N19" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14">
-      <c r="A20" s="7" t="s">
-        <v>2140</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>2141</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>2142</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>2143</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>1658</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>2144</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>2145</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>2146</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>2143</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>2147</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
-      <c r="A21" s="16" t="s">
-        <v>2148</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>2149</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>1856</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>2150</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>1858</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>2151</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I21" s="18" t="s">
-        <v>2152</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>2153</v>
-      </c>
-      <c r="K21" s="17" t="s">
-        <v>2154</v>
-      </c>
-      <c r="L21" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M21" s="7" t="s">
-        <v>1856</v>
-      </c>
-      <c r="N21" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14">
-      <c r="A22" s="16" t="s">
-        <v>2155</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>2156</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>2157</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>2158</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>2159</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>2160</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>2161</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>2052</v>
-      </c>
-      <c r="L22" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M22" s="7" t="s">
-        <v>1904</v>
-      </c>
-      <c r="N22" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14">
-      <c r="A23" s="16" t="s">
-        <v>2162</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>2163</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>1947</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>2164</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>2165</v>
-      </c>
-      <c r="H23" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>2166</v>
-      </c>
-      <c r="J23" s="18" t="s">
-        <v>2167</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>2052</v>
-      </c>
-      <c r="L23" s="7" t="s">
-        <v>2877</v>
-      </c>
-      <c r="M23" s="7" t="s">
-        <v>2060</v>
-      </c>
-      <c r="N23" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="I15" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-00000F000000}"/>
-    <hyperlink ref="J15" r:id="rId2" xr:uid="{00000000-0004-0000-0A00-000010000000}"/>
-    <hyperlink ref="I16" r:id="rId3" xr:uid="{00000000-0004-0000-0A00-000011000000}"/>
-    <hyperlink ref="J16" r:id="rId4" xr:uid="{00000000-0004-0000-0A00-000012000000}"/>
-    <hyperlink ref="I17" r:id="rId5" xr:uid="{00000000-0004-0000-0A00-000013000000}"/>
-    <hyperlink ref="J17" r:id="rId6" xr:uid="{00000000-0004-0000-0A00-000014000000}"/>
-    <hyperlink ref="I21" r:id="rId7" xr:uid="{E5D95628-DADF-425D-8DC6-0740E7A281C6}"/>
-    <hyperlink ref="J23" r:id="rId8" xr:uid="{21B09737-BF9A-463D-87B2-ED444DC9196C}"/>
-    <hyperlink ref="J3" r:id="rId9" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
-    <hyperlink ref="I5" r:id="rId10" xr:uid="{00000000-0004-0000-0B00-000001000000}"/>
-    <hyperlink ref="J5" r:id="rId11" xr:uid="{00000000-0004-0000-0B00-000002000000}"/>
-    <hyperlink ref="I6" r:id="rId12" xr:uid="{00000000-0004-0000-0B00-000003000000}"/>
-    <hyperlink ref="J6" r:id="rId13" xr:uid="{00000000-0004-0000-0B00-000004000000}"/>
-    <hyperlink ref="F7" r:id="rId14" xr:uid="{00000000-0004-0000-0B00-000005000000}"/>
-    <hyperlink ref="I14" r:id="rId15" xr:uid="{BFE50862-7088-44B1-9DAF-F4C51270ACE8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
-  <dimension ref="A1:O21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="13" max="13" width="13.36328125" customWidth="1"/>
-    <col min="14" max="14" width="16.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K2" t="s">
-        <v>1690</v>
-      </c>
-      <c r="L2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M2" t="s">
-        <v>50</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="A3" t="s">
-        <v>1813</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>1693</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>1694</v>
-      </c>
-      <c r="D3" s="22">
-        <v>1206</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>1695</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>1697</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>1698</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>1699</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L3" t="s">
-        <v>55</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-      <c r="O3" s="7"/>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="A4" t="s">
-        <v>1814</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>1702</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>1703</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>1704</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>1705</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>1706</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>1707</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>1708</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>1709</v>
-      </c>
-      <c r="N4" t="s">
-        <v>25</v>
-      </c>
-      <c r="O4" s="7"/>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="A5" t="s">
-        <v>1815</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>1710</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>1711</v>
-      </c>
-      <c r="D5" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>1712</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>1691</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>1712</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>1713</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>1714</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L5" t="s">
-        <v>55</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N5" t="s">
-        <v>25</v>
-      </c>
-      <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15">
-      <c r="A6" t="s">
-        <v>1816</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>1715</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>1716</v>
-      </c>
-      <c r="D6" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>1717</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>1718</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>1717</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>1719</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>1720</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L6" t="s">
-        <v>55</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N6" t="s">
-        <v>25</v>
-      </c>
-      <c r="O6" s="3"/>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" t="s">
-        <v>1817</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>1721</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>1692</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>1722</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>1723</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>1724</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>1725</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>1726</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L7" t="s">
-        <v>55</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>1727</v>
-      </c>
-      <c r="N7" t="s">
-        <v>25</v>
-      </c>
-      <c r="O7" s="3"/>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="A8" t="s">
-        <v>1818</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>1728</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>1703</v>
-      </c>
-      <c r="D8" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>1729</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>1730</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>1731</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>1732</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>1733</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L8" t="s">
-        <v>55</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N8" t="s">
-        <v>25</v>
-      </c>
-      <c r="O8" s="3"/>
-    </row>
-    <row r="9" spans="1:15">
-      <c r="A9" t="s">
-        <v>1819</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>1734</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>1711</v>
-      </c>
-      <c r="D9" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>1735</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>1730</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>1736</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>1737</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>1738</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L9" t="s">
-        <v>55</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N9" t="s">
-        <v>25</v>
-      </c>
-      <c r="O9" s="3"/>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>1820</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>1739</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>1740</v>
-      </c>
-      <c r="D10" s="7">
-        <v>1812</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>1741</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>1743</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>1744</v>
-      </c>
-      <c r="J10" s="15" t="s">
-        <v>1745</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L10" t="s">
-        <v>55</v>
-      </c>
-      <c r="M10" s="7" t="s">
-        <v>1746</v>
-      </c>
-      <c r="N10" t="s">
-        <v>25</v>
-      </c>
-      <c r="O10" s="3"/>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="A11" t="s">
-        <v>1821</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>1747</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>1748</v>
-      </c>
-      <c r="D11" s="7">
-        <v>1812</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>1749</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>1750</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>1751</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>1752</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L11" t="s">
-        <v>55</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>1746</v>
-      </c>
-      <c r="N11" t="s">
-        <v>25</v>
-      </c>
-      <c r="O11" s="3"/>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="A12" t="s">
-        <v>1822</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>1753</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>1754</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>1755</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>1756</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>1757</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>1758</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" s="18" t="s">
-        <v>1759</v>
-      </c>
-      <c r="J12" s="18" t="s">
-        <v>1760</v>
-      </c>
-      <c r="K12" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L12" t="s">
-        <v>55</v>
-      </c>
-      <c r="M12" s="17" t="s">
-        <v>1761</v>
-      </c>
-      <c r="N12" t="s">
-        <v>25</v>
-      </c>
-      <c r="O12" s="3"/>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" t="s">
-        <v>1823</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>1762</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>1763</v>
-      </c>
-      <c r="D13" s="3">
-        <v>1812</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>1764</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>1765</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="18" t="s">
-        <v>1766</v>
-      </c>
-      <c r="J13" s="18" t="s">
-        <v>1767</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L13" t="s">
-        <v>55</v>
-      </c>
-      <c r="M13" s="7" t="s">
-        <v>1746</v>
-      </c>
-      <c r="N13" t="s">
-        <v>25</v>
-      </c>
-      <c r="O13" s="3"/>
-    </row>
-    <row r="14" spans="1:15">
-      <c r="A14" t="s">
-        <v>1824</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>1768</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>1763</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>1769</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>1770</v>
-      </c>
-      <c r="H14" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>1771</v>
-      </c>
-      <c r="J14" s="18" t="s">
-        <v>1772</v>
-      </c>
-      <c r="K14" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L14" t="s">
-        <v>55</v>
-      </c>
-      <c r="M14" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N14" t="s">
-        <v>25</v>
-      </c>
-      <c r="O14" s="3"/>
-    </row>
-    <row r="15" spans="1:15">
-      <c r="A15" t="s">
-        <v>1825</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>1773</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>1774</v>
-      </c>
-      <c r="D15" s="7">
-        <v>1206</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>1775</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>1776</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>1777</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>1778</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>1779</v>
-      </c>
-      <c r="K15" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L15" t="s">
-        <v>55</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>1701</v>
-      </c>
-      <c r="N15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15">
-      <c r="A16" t="s">
-        <v>1826</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>1780</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>1774</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>1781</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G16" s="16" t="s">
-        <v>1782</v>
-      </c>
-      <c r="H16" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>1783</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>1784</v>
-      </c>
-      <c r="K16" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L16" t="s">
-        <v>55</v>
-      </c>
-      <c r="M16" s="16" t="s">
-        <v>1785</v>
-      </c>
-      <c r="N16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14">
-      <c r="A17" t="s">
-        <v>1827</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>1786</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>1763</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>1787</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>1696</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>1788</v>
-      </c>
-      <c r="H17" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>1789</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>1783</v>
-      </c>
-      <c r="K17" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L17" t="s">
-        <v>55</v>
-      </c>
-      <c r="M17" s="16" t="s">
-        <v>1785</v>
-      </c>
-      <c r="N17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
-      <c r="A18" t="s">
-        <v>1828</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>1790</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>1791</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>1792</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>1793</v>
-      </c>
-      <c r="H18" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>1794</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>1795</v>
-      </c>
-      <c r="K18" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L18" t="s">
-        <v>55</v>
-      </c>
-      <c r="M18" s="16" t="s">
-        <v>1785</v>
-      </c>
-      <c r="N18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
-      <c r="A19" t="s">
-        <v>1829</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>1796</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>1763</v>
-      </c>
-      <c r="D19" s="3">
-        <v>1812</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>1797</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>1798</v>
-      </c>
-      <c r="H19" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I19" s="18" t="s">
-        <v>1799</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>1800</v>
-      </c>
-      <c r="K19" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L19" t="s">
-        <v>55</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>1746</v>
-      </c>
-      <c r="N19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14">
-      <c r="A20" t="s">
-        <v>1830</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>1801</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>1692</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>1802</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>1803</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>1804</v>
-      </c>
-      <c r="H20" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="I20" s="18" t="s">
-        <v>1805</v>
-      </c>
-      <c r="J20" s="18" t="s">
-        <v>1806</v>
-      </c>
-      <c r="K20" s="17" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L20" t="s">
-        <v>55</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>1807</v>
-      </c>
-      <c r="N20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
-      <c r="A21" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>1808</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>1703</v>
-      </c>
-      <c r="D21" s="7">
-        <v>1812</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>1809</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>1742</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>1810</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>1811</v>
-      </c>
-      <c r="J21" s="18" t="s">
-        <v>1812</v>
-      </c>
-      <c r="K21" s="7" t="s">
-        <v>1700</v>
-      </c>
-      <c r="L21" t="s">
-        <v>55</v>
-      </c>
-      <c r="M21" s="7" t="s">
-        <v>1746</v>
-      </c>
-      <c r="N21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="16" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{3DE7E9B7-7F71-48BD-A43F-56652EF48515}"/>
-    <hyperlink ref="I5" r:id="rId2" xr:uid="{00000000-0004-0000-0C00-000001000000}"/>
-    <hyperlink ref="J5" r:id="rId3" xr:uid="{00000000-0004-0000-0C00-000002000000}"/>
-    <hyperlink ref="I6" r:id="rId4" xr:uid="{00000000-0004-0000-0C00-000003000000}"/>
-    <hyperlink ref="J6" r:id="rId5" xr:uid="{00000000-0004-0000-0C00-000004000000}"/>
-    <hyperlink ref="I10" r:id="rId6" xr:uid="{00000000-0004-0000-0C00-000005000000}"/>
-    <hyperlink ref="J10" r:id="rId7" xr:uid="{00000000-0004-0000-0C00-000006000000}"/>
-    <hyperlink ref="I12" r:id="rId8" xr:uid="{DC4D0F7D-FABA-4F27-A8C4-C8F1159FEA34}"/>
-    <hyperlink ref="J12" r:id="rId9" xr:uid="{7C1A203F-2505-4DF3-8487-119DA9DE1A1B}"/>
-    <hyperlink ref="J13" r:id="rId10" xr:uid="{6F374EEE-953D-426D-AF07-D3E5C1F03D55}"/>
-    <hyperlink ref="I13" r:id="rId11" xr:uid="{959671DE-63B1-4C42-9AE2-A4D45EAFA482}"/>
-    <hyperlink ref="J14" r:id="rId12" xr:uid="{D0E41C99-5015-461D-998D-DD06CC299D2B}"/>
-    <hyperlink ref="I19" r:id="rId13" xr:uid="{EAFB85FD-4F43-4B6C-AEDE-D6E5C0E93BD1}"/>
-    <hyperlink ref="I20" r:id="rId14" xr:uid="{6C9DFF48-0956-4B25-8972-EC0656F1483E}"/>
-    <hyperlink ref="J20" r:id="rId15" xr:uid="{6EF40273-C6D8-4BC3-9EF6-1B4C76903848}"/>
-    <hyperlink ref="J21" r:id="rId16" xr:uid="{FFB17F08-401F-47B0-899B-612CD8B9FB6B}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
110-0061 and 010-0136 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74AA2D8-E955-4948-8612-3823F2A6CDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F8A1BE-3970-4568-BD7A-4D709525CAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5814" uniqueCount="2916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5842" uniqueCount="2925">
   <si>
     <t>ID</t>
   </si>
@@ -8788,6 +8788,33 @@
   </si>
   <si>
     <t>CAP_10Dx20L</t>
+  </si>
+  <si>
+    <t>110-0061</t>
+  </si>
+  <si>
+    <t>HTSW-102-07-G-S</t>
+  </si>
+  <si>
+    <t>200-HTSW10207GS</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/85/1/htsw_th.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Samtec/HTSW-102-07-G-S?qs=FESYatJ8odI1BCBanfu%2FIg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0136</t>
+  </si>
+  <si>
+    <t>603-RC0603FR-7W10KL</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/508/1/PYU_RC_GROUP_51_ROHS_L.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/YAGEO/RC0603FR-7W10KL?qs=AQlKX63v8Ru%2F1n5uALWRmg%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -17003,7 +17030,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="5" max="5" width="16.36328125" bestFit="1" customWidth="1"/>
@@ -19692,6 +19719,50 @@
         <v>657004150201</v>
       </c>
       <c r="N61" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
+      <c r="A62" s="16" t="s">
+        <v>2916</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>2466</v>
+      </c>
+      <c r="C62" s="16" t="s">
+        <v>2170</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>2543</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>2917</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>2403</v>
+      </c>
+      <c r="G62" s="16" t="s">
+        <v>2918</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I62" s="7" t="s">
+        <v>2919</v>
+      </c>
+      <c r="J62" s="18" t="s">
+        <v>2920</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>2176</v>
+      </c>
+      <c r="L62" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>2322</v>
+      </c>
+      <c r="N62" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -19865,7 +19936,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N136"/>
+  <dimension ref="A1:N137"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -25856,7 +25927,52 @@
         <v>25</v>
       </c>
     </row>
+    <row r="137" spans="1:14">
+      <c r="A137" s="16" t="s">
+        <v>2921</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>906</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>907</v>
+      </c>
+      <c r="D137" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E137" s="7" t="s">
+        <v>908</v>
+      </c>
+      <c r="F137" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G137" s="16" t="s">
+        <v>2922</v>
+      </c>
+      <c r="H137" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I137" s="15" t="s">
+        <v>2923</v>
+      </c>
+      <c r="J137" s="2" t="s">
+        <v>2924</v>
+      </c>
+      <c r="K137" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L137" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M137" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N137" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="J5" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
     <hyperlink ref="I20" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
@@ -25947,9 +26063,10 @@
     <hyperlink ref="I126" r:id="rId87" xr:uid="{D5217351-58DE-4063-B05F-2AAD973A6964}"/>
     <hyperlink ref="I127" r:id="rId88" xr:uid="{445CA2DB-DCDC-4D49-B3FC-95650287197F}"/>
     <hyperlink ref="I136" r:id="rId89" xr:uid="{4FA7D577-C2BC-4C3D-92A8-50A98BB0C15F}"/>
+    <hyperlink ref="J137" r:id="rId90" xr:uid="{270FAB0D-B47D-4805-A699-C4BB16679313}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId90"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId91"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
050-0002, 050-0001, 001-0092, 001-0093, 010-0137, 015-0003, 010-0138, 033-0023, 010-0139, 010-0140, 010-0141 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F8A1BE-3970-4568-BD7A-4D709525CAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39849982-C04A-4265-AA5E-5CD885176695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5842" uniqueCount="2925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5968" uniqueCount="2992">
   <si>
     <t>ID</t>
   </si>
@@ -8815,6 +8815,207 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/YAGEO/RC0603FR-7W10KL?qs=AQlKX63v8Ru%2F1n5uALWRmg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0137</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 0.33W 10ohms 5% High Power AEC-Q200</t>
+  </si>
+  <si>
+    <t>71-CRCW060310R0JNEAH</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/20043/crcwhpe3.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/CRCW060310R0JNEAHP?qs=k2%2FDWSARqgEB1LI%252BjPBTjg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0138</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD CRCW 603 4K00 0.01 100 ppm/K</t>
+  </si>
+  <si>
+    <t>CRCW06034K00FKTA</t>
+  </si>
+  <si>
+    <t>71-CRCW06034K00FKTA</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/20008/dcrcw.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/CRCW06034K00FKTA?qs=WI1XYtAgnMkbyTUP7%2FnzOA%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0139</t>
+  </si>
+  <si>
+    <t>Resistores de película fina - SMD 1/10W 50 Ohm 75V .1%</t>
+  </si>
+  <si>
+    <t>50Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>RT0603BRE0750RL</t>
+  </si>
+  <si>
+    <t>603-RT0603BRE0750RL</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/72/1/PYU_RT_1_TO_0_01_ROHS_L.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/YAGEO/RT0603BRE0750RL?qs=sGAEpiMZZMtlubZbdhIBINSnPd898yDPudX1JlFp2aw%3D</t>
+  </si>
+  <si>
+    <t>010-0140</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 0603 330ohm 1% Anti-Surge AEC-Q200</t>
+  </si>
+  <si>
+    <t>330Ω 333mW ±1%</t>
+  </si>
+  <si>
+    <t>667-ERJ-PA3F3300V</t>
+  </si>
+  <si>
+    <t>https://industrial.panasonic.com/cdbs/www-data/pdf/RDO0000/RDO0000C334.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERJ-PA3F3300V?qs=BzJM0faLVqV%252BdjJR48HqGQ%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0141</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 1.8 kOhms 1/10 W 75 V 5% 0603 100 PPM / C - 55 C / + 155 C AEC-Q200</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/508/1/PYU_AC_51_ROHS_L.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/YAGEO/AC0603JR-071K8L?qs=ygRr%2Ftkhtesbqtk4RgJA%2FQ%3D%3D</t>
+  </si>
+  <si>
+    <t>603-AC0603JR-071K8L</t>
+  </si>
+  <si>
+    <t>AC0603JR-071K8L</t>
+  </si>
+  <si>
+    <t>LED de un solo color Green 525nm 1400mcd 2.85V 73deg 0603</t>
+  </si>
+  <si>
+    <t>VLMTG1400-GS08</t>
+  </si>
+  <si>
+    <t>78-VLMTG1400-GS08</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/84393/vlmtg1400.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Semiconductors/VLMTG1400-GS08?qs=gt1LBUVyoHlZ6yHd8iEIzQ%3D%3D</t>
+  </si>
+  <si>
+    <t>033-0014</t>
+  </si>
+  <si>
+    <t>033-0015</t>
+  </si>
+  <si>
+    <t>033-0016</t>
+  </si>
+  <si>
+    <t>033-0017</t>
+  </si>
+  <si>
+    <t>033-0018</t>
+  </si>
+  <si>
+    <t>033-0019</t>
+  </si>
+  <si>
+    <t>033-0020</t>
+  </si>
+  <si>
+    <t>033-0021</t>
+  </si>
+  <si>
+    <t>033-0022</t>
+  </si>
+  <si>
+    <t>033-0023</t>
+  </si>
+  <si>
+    <t>015-0003</t>
+  </si>
+  <si>
+    <t>Resistores de detección de corriente - SMD 3W 0.007ohm 1% 50ppm</t>
+  </si>
+  <si>
+    <t>7mΩ 3W ±1%</t>
+  </si>
+  <si>
+    <t>1225 (Reversed)</t>
+  </si>
+  <si>
+    <t>KRL6432E-M-R007-F-T1</t>
+  </si>
+  <si>
+    <t>Susumu</t>
+  </si>
+  <si>
+    <t>754-KRL6432EMR007FT1</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/826/1/n_catalog_partition19_en.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Susumu/KRL6432E-M-R007-F-T1?qs=FG09h9tFCuA5fgBuyupdEw%3D%3D</t>
+  </si>
+  <si>
+    <t>RES SMD 1225 Reversed</t>
+  </si>
+  <si>
+    <t>001-0092</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 16 V 0.1uF X7R 0603 10%</t>
+  </si>
+  <si>
+    <t>16V 0.1uF X7R</t>
+  </si>
+  <si>
+    <t>603-CC603KRX7R7BB104</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/508/1/UPY_GPHC_X7R_6_3V_TO_250V.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/YAGEO/CC0603KRX7R7BB104?qs=AgBp2OyFlx8KPmNTlFoWXA%3D%3D</t>
+  </si>
+  <si>
+    <t>001-0093</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 16V 1uF X7R 0603 10% HI CV</t>
+  </si>
+  <si>
+    <t>16V 1uF X7R</t>
+  </si>
+  <si>
+    <t>CC0603KRX7R7BB105</t>
+  </si>
+  <si>
+    <t>603-CC603KRX7R7BB105</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/YAGEO/CC0603KRX7R7BB105?qs=Z5EW3TBnpq2UUKiQ6CZTSQ%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -8984,7 +9185,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9035,6 +9236,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -9318,7 +9524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -13382,7 +13588,96 @@
         <v>25</v>
       </c>
     </row>
+    <row r="93" spans="1:14">
+      <c r="A93" s="4" t="s">
+        <v>2980</v>
+      </c>
+      <c r="B93" s="32" t="s">
+        <v>2981</v>
+      </c>
+      <c r="C93" s="35" t="s">
+        <v>2982</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E93" t="s">
+        <v>304</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G93" s="32" t="s">
+        <v>2983</v>
+      </c>
+      <c r="H93" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="I93" s="27" t="s">
+        <v>2984</v>
+      </c>
+      <c r="J93" s="27" t="s">
+        <v>2985</v>
+      </c>
+      <c r="K93" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L93" t="s">
+        <v>61</v>
+      </c>
+      <c r="M93" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N93" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14">
+      <c r="A94" s="4" t="s">
+        <v>2986</v>
+      </c>
+      <c r="B94" s="32" t="s">
+        <v>2987</v>
+      </c>
+      <c r="C94" s="35" t="s">
+        <v>2988</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E94" s="34" t="s">
+        <v>2989</v>
+      </c>
+      <c r="F94" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="G94" s="32" t="s">
+        <v>2990</v>
+      </c>
+      <c r="H94" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="I94" s="27" t="s">
+        <v>2984</v>
+      </c>
+      <c r="J94" s="36" t="s">
+        <v>2991</v>
+      </c>
+      <c r="K94" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L94" t="s">
+        <v>61</v>
+      </c>
+      <c r="M94" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N94" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I22" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="I23" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -13434,6 +13729,10 @@
     <hyperlink ref="I89" r:id="rId48" xr:uid="{54C8C95D-2C8A-4B14-B3F8-1B69A2587372}"/>
     <hyperlink ref="I82" r:id="rId49" xr:uid="{B234FDA3-9881-49C7-9757-E6B50F09E652}"/>
     <hyperlink ref="I92" r:id="rId50" xr:uid="{629DD39D-5539-4595-B551-7C70898E50E5}"/>
+    <hyperlink ref="I93" r:id="rId51" xr:uid="{C9324AD1-D443-4B4A-88F6-7342BEEBC444}"/>
+    <hyperlink ref="J93" r:id="rId52" xr:uid="{02ABAA1D-5CBA-4945-9449-F11890AA00C1}"/>
+    <hyperlink ref="I94" r:id="rId53" xr:uid="{CD066ABD-A9CF-4B23-B64F-6EFECB0682A9}"/>
+    <hyperlink ref="J94" r:id="rId54" xr:uid="{DE191AC8-7CDC-47D8-8778-80293EDB2FDD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13441,7 +13740,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14" ht="14.5" customHeight="1">
@@ -14062,7 +14361,7 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="7" t="s">
-        <v>2106</v>
+        <v>2960</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>2107</v>
@@ -14106,7 +14405,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="7" t="s">
-        <v>2112</v>
+        <v>2961</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>2113</v>
@@ -14150,7 +14449,7 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="7" t="s">
-        <v>2118</v>
+        <v>2962</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>2119</v>
@@ -14194,7 +14493,7 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="7" t="s">
-        <v>2126</v>
+        <v>2963</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>2127</v>
@@ -14238,7 +14537,7 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="7" t="s">
-        <v>2133</v>
+        <v>2964</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>2134</v>
@@ -14282,7 +14581,7 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="7" t="s">
-        <v>2140</v>
+        <v>2965</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>2141</v>
@@ -14325,8 +14624,8 @@
       </c>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="16" t="s">
-        <v>2148</v>
+      <c r="A21" s="7" t="s">
+        <v>2966</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>2149</v>
@@ -14369,8 +14668,8 @@
       </c>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="16" t="s">
-        <v>2155</v>
+      <c r="A22" s="7" t="s">
+        <v>2967</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>2156</v>
@@ -14413,8 +14712,8 @@
       </c>
     </row>
     <row r="23" spans="1:14">
-      <c r="A23" s="16" t="s">
-        <v>2162</v>
+      <c r="A23" s="7" t="s">
+        <v>2968</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>2163</v>
@@ -14456,7 +14755,52 @@
         <v>25</v>
       </c>
     </row>
+    <row r="24" spans="1:14">
+      <c r="A24" s="7" t="s">
+        <v>2969</v>
+      </c>
+      <c r="B24" s="32" t="s">
+        <v>2955</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>2793</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>2956</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>1957</v>
+      </c>
+      <c r="G24" s="32" t="s">
+        <v>2957</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" t="s">
+        <v>2958</v>
+      </c>
+      <c r="J24" s="36" t="s">
+        <v>2959</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>2774</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>2877</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>2876</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I15" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-00000F000000}"/>
     <hyperlink ref="J15" r:id="rId2" xr:uid="{00000000-0004-0000-0A00-000010000000}"/>
@@ -14473,6 +14817,7 @@
     <hyperlink ref="J6" r:id="rId13" xr:uid="{00000000-0004-0000-0B00-000004000000}"/>
     <hyperlink ref="F7" r:id="rId14" xr:uid="{00000000-0004-0000-0B00-000005000000}"/>
     <hyperlink ref="I14" r:id="rId15" xr:uid="{BFE50862-7088-44B1-9DAF-F4C51270ACE8}"/>
+    <hyperlink ref="J24" r:id="rId16" xr:uid="{BA37FCF7-BBC9-434F-AC42-00AE241CF11E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19936,7 +20281,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N137"/>
+  <dimension ref="A1:N142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -25968,6 +26313,226 @@
         <v>57</v>
       </c>
       <c r="N137" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14">
+      <c r="A138" s="16" t="s">
+        <v>2925</v>
+      </c>
+      <c r="B138" s="7" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C138" s="7" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D138" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E138" s="7" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F138" s="7" t="s">
+        <v>945</v>
+      </c>
+      <c r="G138" s="16" t="s">
+        <v>2927</v>
+      </c>
+      <c r="H138" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I138" s="7" t="s">
+        <v>2928</v>
+      </c>
+      <c r="J138" s="7" t="s">
+        <v>2929</v>
+      </c>
+      <c r="K138" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L138" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M138" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N138" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14">
+      <c r="A139" s="16" t="s">
+        <v>2930</v>
+      </c>
+      <c r="B139" s="33" t="s">
+        <v>2931</v>
+      </c>
+      <c r="C139" s="7" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D139" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E139" s="33" t="s">
+        <v>2932</v>
+      </c>
+      <c r="F139" s="7" t="s">
+        <v>945</v>
+      </c>
+      <c r="G139" s="34" t="s">
+        <v>2933</v>
+      </c>
+      <c r="H139" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I139" t="s">
+        <v>2934</v>
+      </c>
+      <c r="J139" t="s">
+        <v>2935</v>
+      </c>
+      <c r="K139" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L139" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M139" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N139" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14">
+      <c r="A140" s="16" t="s">
+        <v>2936</v>
+      </c>
+      <c r="B140" s="33" t="s">
+        <v>2937</v>
+      </c>
+      <c r="C140" s="7" t="s">
+        <v>2938</v>
+      </c>
+      <c r="D140" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E140" s="33" t="s">
+        <v>2939</v>
+      </c>
+      <c r="F140" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="G140" s="34" t="s">
+        <v>2940</v>
+      </c>
+      <c r="H140" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="I140" s="27" t="s">
+        <v>2941</v>
+      </c>
+      <c r="J140" s="27" t="s">
+        <v>2942</v>
+      </c>
+      <c r="K140" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L140" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M140" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N140" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14">
+      <c r="A141" s="16" t="s">
+        <v>2943</v>
+      </c>
+      <c r="B141" s="17" t="s">
+        <v>2944</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>2945</v>
+      </c>
+      <c r="D141" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E141" s="17" t="s">
+        <v>1566</v>
+      </c>
+      <c r="F141" s="17" t="s">
+        <v>1567</v>
+      </c>
+      <c r="G141" s="17" t="s">
+        <v>2946</v>
+      </c>
+      <c r="H141" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="I141" s="18" t="s">
+        <v>2947</v>
+      </c>
+      <c r="J141" s="3" t="s">
+        <v>2948</v>
+      </c>
+      <c r="K141" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L141" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M141" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N141" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14">
+      <c r="A142" s="16" t="s">
+        <v>2949</v>
+      </c>
+      <c r="B142" s="35" t="s">
+        <v>2950</v>
+      </c>
+      <c r="C142" s="17" t="s">
+        <v>1588</v>
+      </c>
+      <c r="D142" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E142" s="35" t="s">
+        <v>2954</v>
+      </c>
+      <c r="F142" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="G142" s="35" t="s">
+        <v>2953</v>
+      </c>
+      <c r="H142" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="I142" t="s">
+        <v>2951</v>
+      </c>
+      <c r="J142" t="s">
+        <v>2952</v>
+      </c>
+      <c r="K142" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L142" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M142" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N142" t="s">
         <v>25</v>
       </c>
     </row>
@@ -26064,15 +26629,17 @@
     <hyperlink ref="I127" r:id="rId88" xr:uid="{445CA2DB-DCDC-4D49-B3FC-95650287197F}"/>
     <hyperlink ref="I136" r:id="rId89" xr:uid="{4FA7D577-C2BC-4C3D-92A8-50A98BB0C15F}"/>
     <hyperlink ref="J137" r:id="rId90" xr:uid="{270FAB0D-B47D-4805-A699-C4BB16679313}"/>
+    <hyperlink ref="I140" r:id="rId91" xr:uid="{AF66F37C-DEF2-4C02-B09E-78216E8A0857}"/>
+    <hyperlink ref="J140" r:id="rId92" xr:uid="{5C7EACC9-1558-4F25-8631-38E695251F20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId91"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId93"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="20.26953125" customWidth="1"/>
@@ -26210,11 +26777,58 @@
         <v>25</v>
       </c>
     </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>2970</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2971</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2972</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2973</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2974</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2975</v>
+      </c>
+      <c r="G4" t="s">
+        <v>2976</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>2977</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>2978</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M4" t="s">
+        <v>2979</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{9FEE5192-80A9-4D8D-B0ED-453C4A95B2F9}"/>
     <hyperlink ref="J2" r:id="rId2" xr:uid="{40967CA2-E6AE-4524-9EF5-66E92DD6A7B6}"/>
     <hyperlink ref="I3" r:id="rId3" xr:uid="{EDE33321-C187-4A8F-8366-9AEDB9FF4C7B}"/>
+    <hyperlink ref="I4" r:id="rId4" xr:uid="{DA619253-40A2-482C-A99F-F72A13182916}"/>
+    <hyperlink ref="J4" r:id="rId5" xr:uid="{65BF95D6-EB54-41F9-8886-7DFC774FFE44}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
001-0094, 001-0095, 001-0096 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E00982A-7A9B-43D1-9B5B-4F76D30F1C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C7232B-EA9B-4151-B2E2-AE258260E822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5982" uniqueCount="3000">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6024" uniqueCount="3019">
   <si>
     <t>ID</t>
   </si>
@@ -9040,6 +9040,63 @@
   </si>
   <si>
     <t>78-SS20PH102HM3/I</t>
+  </si>
+  <si>
+    <t>001-0094</t>
+  </si>
+  <si>
+    <t>001-0095</t>
+  </si>
+  <si>
+    <t>001-0096</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) Automotive MLCC 1uF, 10%, X7R, 50VDC</t>
+  </si>
+  <si>
+    <t>KAM21KR71H105KL</t>
+  </si>
+  <si>
+    <t>KYOCERA AVX</t>
+  </si>
+  <si>
+    <t>https://ele.kyocera.com/assets/products/capacitor/KGM_Series_e.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/KAM21KR71H105KL?qs=Jm2GQyTW%2FbhahfzttUK9QA%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 50V 10uF X7R 1210 10 % AEC-Q200</t>
+  </si>
+  <si>
+    <t>50V 10uF X7R</t>
+  </si>
+  <si>
+    <t>KAM32LR71H106KL</t>
+  </si>
+  <si>
+    <t>581-KAM32LR71H106KL</t>
+  </si>
+  <si>
+    <t>581-KAM21KR71H105KL</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/KAM32LR71H106KL?qs=sGAEpiMZZMuMW9TJLBQkXqLYvz3DzaXf%2FdVWcOcJzto%3D</t>
+  </si>
+  <si>
+    <t>KAM21BR71H104JM</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 50V 0.1uF X7R 0805 5% AEC-Q200</t>
+  </si>
+  <si>
+    <t>50V 0.1uF X7R</t>
+  </si>
+  <si>
+    <t>581-KAM21BR71H104JM</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/KAM21BR71H104JM?qs=sGAEpiMZZMuMW9TJLBQkXqLYvz3DzaXfcS9olcxY6vM%3D</t>
   </si>
 </sst>
 </file>
@@ -9209,7 +9266,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9262,8 +9319,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -9547,7 +9605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -13696,6 +13754,138 @@
         <v>62</v>
       </c>
       <c r="N94" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14">
+      <c r="A95" s="4" t="s">
+        <v>3000</v>
+      </c>
+      <c r="B95" t="s">
+        <v>3003</v>
+      </c>
+      <c r="C95" s="34" t="s">
+        <v>443</v>
+      </c>
+      <c r="D95" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E95" s="35" t="s">
+        <v>3004</v>
+      </c>
+      <c r="F95" s="36" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G95" s="33" t="s">
+        <v>3012</v>
+      </c>
+      <c r="H95" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I95" s="27" t="s">
+        <v>3006</v>
+      </c>
+      <c r="J95" s="32" t="s">
+        <v>3007</v>
+      </c>
+      <c r="K95" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L95" t="s">
+        <v>61</v>
+      </c>
+      <c r="M95" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="N95" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14">
+      <c r="A96" s="4" t="s">
+        <v>3001</v>
+      </c>
+      <c r="B96" t="s">
+        <v>3008</v>
+      </c>
+      <c r="C96" s="34" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D96" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="E96" s="35" t="s">
+        <v>3010</v>
+      </c>
+      <c r="F96" s="33" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G96" s="33" t="s">
+        <v>3011</v>
+      </c>
+      <c r="H96" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I96" s="27" t="s">
+        <v>3006</v>
+      </c>
+      <c r="J96" s="32" t="s">
+        <v>3013</v>
+      </c>
+      <c r="K96" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L96" t="s">
+        <v>61</v>
+      </c>
+      <c r="M96" s="7" t="s">
+        <v>702</v>
+      </c>
+      <c r="N96" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14">
+      <c r="A97" s="4" t="s">
+        <v>3002</v>
+      </c>
+      <c r="B97" t="s">
+        <v>3015</v>
+      </c>
+      <c r="C97" s="34" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D97" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E97" s="35" t="s">
+        <v>3014</v>
+      </c>
+      <c r="F97" s="33" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G97" s="33" t="s">
+        <v>3017</v>
+      </c>
+      <c r="H97" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I97" s="27" t="s">
+        <v>3006</v>
+      </c>
+      <c r="J97" t="s">
+        <v>3018</v>
+      </c>
+      <c r="K97" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L97" t="s">
+        <v>61</v>
+      </c>
+      <c r="M97" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="N97" t="s">
         <v>25</v>
       </c>
     </row>
@@ -13756,6 +13946,11 @@
     <hyperlink ref="J93" r:id="rId52" xr:uid="{02ABAA1D-5CBA-4945-9449-F11890AA00C1}"/>
     <hyperlink ref="I94" r:id="rId53" xr:uid="{CD066ABD-A9CF-4B23-B64F-6EFECB0682A9}"/>
     <hyperlink ref="J94" r:id="rId54" xr:uid="{DE191AC8-7CDC-47D8-8778-80293EDB2FDD}"/>
+    <hyperlink ref="I95" r:id="rId55" xr:uid="{CCA8EE89-F6B4-4DE6-8266-D2E2C7A801D9}"/>
+    <hyperlink ref="J95" r:id="rId56" xr:uid="{3EA9C5B0-8F07-472C-B534-F158D1D13832}"/>
+    <hyperlink ref="I96" r:id="rId57" xr:uid="{84DAD3FB-EB5D-446A-B122-0A99A60B6E95}"/>
+    <hyperlink ref="J96" r:id="rId58" xr:uid="{44B094DB-343C-49F4-A023-566CEE808AE0}"/>
+    <hyperlink ref="I97" r:id="rId59" xr:uid="{890D1BEC-53E9-4E41-AB45-508A74C3ACB5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -27961,22 +28156,22 @@
       <c r="A13" s="16" t="s">
         <v>2994</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="3" t="s">
         <v>2995</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="7" t="s">
         <v>2996</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="3" t="s">
         <v>2997</v>
       </c>
-      <c r="E13" s="35" t="s">
+      <c r="E13" s="17" t="s">
         <v>2998</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>1957</v>
       </c>
-      <c r="G13" s="35" t="s">
+      <c r="G13" s="17" t="s">
         <v>2999</v>
       </c>
       <c r="H13" s="7" t="s">

</xml_diff>

<commit_message>
001-0097, 001-0098, 001-0099, 001-0100, 001-0101, 001-0102, 001-0103, 001-0104 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F22F469-B048-42F6-8D06-3B2211C6DD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D670F-F1D6-4AB3-A5EB-F0ABEB79F458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10710" yWindow="0" windowWidth="10980" windowHeight="13770" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32295" yWindow="2355" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6095" uniqueCount="3050">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6207" uniqueCount="3102">
   <si>
     <t>ID</t>
   </si>
@@ -9192,6 +9192,162 @@
   </si>
   <si>
     <t>SMD3225-4P</t>
+  </si>
+  <si>
+    <t>001-0097</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 1.5pF 0402 0.5pF TOL 16V</t>
+  </si>
+  <si>
+    <t>16V 1.5pF C0G</t>
+  </si>
+  <si>
+    <t>710-885012005020</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012005020.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012005020?qs=0KOYDY2FL2%2FpnGt3CBSzcg%3D%3D</t>
+  </si>
+  <si>
+    <t>001-0098</t>
+  </si>
+  <si>
+    <t>001-0099</t>
+  </si>
+  <si>
+    <t>001-0100</t>
+  </si>
+  <si>
+    <t>001-0101</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 10pF 0402 5% 16V MLCC</t>
+  </si>
+  <si>
+    <t>16V 10pF C0G</t>
+  </si>
+  <si>
+    <t>710-885012005025</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012005025.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012005025?qs=0KOYDY2FL2%2F1u5tcR38OjQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 0.1uF 0402 20% 16V MLCC</t>
+  </si>
+  <si>
+    <t>16V 0.1uF X5R</t>
+  </si>
+  <si>
+    <t>710-885012105016</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012105016.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012105016?qs=0KOYDY2FL2%2FPbpf70bBQeA%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 0.1uF 0805 10% 50V MLCC</t>
+  </si>
+  <si>
+    <t>710-885012207098</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012207098?qs=0KOYDY2FL29sZCNyRsrK9g%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012207098.pdf</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 0.01uF 0402 10% 16V MLCC</t>
+  </si>
+  <si>
+    <t>001-0102</t>
+  </si>
+  <si>
+    <t>16V 10nF X5R</t>
+  </si>
+  <si>
+    <t>710-885012205031</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012205031.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012205031?qs=0KOYDY2FL28GOkIyNosgaQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 1uF 50 Vol 10%</t>
+  </si>
+  <si>
+    <t>885012005020</t>
+  </si>
+  <si>
+    <t>885012105016</t>
+  </si>
+  <si>
+    <t>885012005025</t>
+  </si>
+  <si>
+    <t>885012207098</t>
+  </si>
+  <si>
+    <t>885012205031</t>
+  </si>
+  <si>
+    <t>885012206126</t>
+  </si>
+  <si>
+    <t>710-885012206126</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012206126.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012206126?qs=amGC7iS6iy%2F%252BJOLb%2FSuwig%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 1uF 0402 20% 10V MLCC</t>
+  </si>
+  <si>
+    <t>001-0103</t>
+  </si>
+  <si>
+    <t>885012105012</t>
+  </si>
+  <si>
+    <t>710-885012105012</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012105012.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012105012?qs=0KOYDY2FL28qr2YJ9j3qRw%3D%3D</t>
+  </si>
+  <si>
+    <t>001-0104</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 10uF 50Vol 0.1</t>
+  </si>
+  <si>
+    <t>885012209073</t>
+  </si>
+  <si>
+    <t>710-885012209073</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012209073.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012209073?qs=sPbYRqrBIVm8PsM2ljQIMg%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -9361,7 +9517,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9418,6 +9574,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -9701,13 +9861,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
     <col min="2" max="2" width="29.6328125" customWidth="1"/>
     <col min="3" max="3" width="14.90625" customWidth="1"/>
     <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6328125" customWidth="1"/>
     <col min="7" max="7" width="15.453125" customWidth="1"/>
     <col min="8" max="8" width="12.453125" customWidth="1"/>
@@ -13982,6 +14143,358 @@
         <v>700</v>
       </c>
       <c r="N97" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14">
+      <c r="A98" s="4" t="s">
+        <v>3050</v>
+      </c>
+      <c r="B98" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C98" s="37" t="s">
+        <v>3052</v>
+      </c>
+      <c r="D98" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E98" s="38" t="s">
+        <v>3081</v>
+      </c>
+      <c r="F98" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G98" s="36" t="s">
+        <v>3053</v>
+      </c>
+      <c r="H98" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I98" s="27" t="s">
+        <v>3054</v>
+      </c>
+      <c r="J98" t="s">
+        <v>3055</v>
+      </c>
+      <c r="K98" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L98" t="s">
+        <v>61</v>
+      </c>
+      <c r="M98" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N98" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14">
+      <c r="A99" s="4" t="s">
+        <v>3056</v>
+      </c>
+      <c r="B99" t="s">
+        <v>3060</v>
+      </c>
+      <c r="C99" s="37" t="s">
+        <v>3061</v>
+      </c>
+      <c r="D99" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E99" s="38" t="s">
+        <v>3083</v>
+      </c>
+      <c r="F99" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G99" s="36" t="s">
+        <v>3062</v>
+      </c>
+      <c r="H99" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I99" s="27" t="s">
+        <v>3063</v>
+      </c>
+      <c r="J99" s="27" t="s">
+        <v>3064</v>
+      </c>
+      <c r="K99" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L99" t="s">
+        <v>61</v>
+      </c>
+      <c r="M99" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N99" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14">
+      <c r="A100" s="4" t="s">
+        <v>3057</v>
+      </c>
+      <c r="B100" t="s">
+        <v>3065</v>
+      </c>
+      <c r="C100" s="37" t="s">
+        <v>3066</v>
+      </c>
+      <c r="D100" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E100" s="38" t="s">
+        <v>3082</v>
+      </c>
+      <c r="F100" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G100" t="s">
+        <v>3067</v>
+      </c>
+      <c r="H100" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I100" t="s">
+        <v>3068</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>3069</v>
+      </c>
+      <c r="K100" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L100" t="s">
+        <v>61</v>
+      </c>
+      <c r="M100" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N100" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14">
+      <c r="A101" s="4" t="s">
+        <v>3058</v>
+      </c>
+      <c r="B101" t="s">
+        <v>3070</v>
+      </c>
+      <c r="C101" s="37" t="s">
+        <v>3016</v>
+      </c>
+      <c r="D101" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E101" s="38" t="s">
+        <v>3084</v>
+      </c>
+      <c r="F101" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G101" s="36" t="s">
+        <v>3071</v>
+      </c>
+      <c r="H101" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I101" t="s">
+        <v>3073</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>3072</v>
+      </c>
+      <c r="K101" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L101" t="s">
+        <v>61</v>
+      </c>
+      <c r="M101" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="N101" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14">
+      <c r="A102" s="4" t="s">
+        <v>3059</v>
+      </c>
+      <c r="B102" t="s">
+        <v>3074</v>
+      </c>
+      <c r="C102" s="37" t="s">
+        <v>3076</v>
+      </c>
+      <c r="D102" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E102" s="38" t="s">
+        <v>3085</v>
+      </c>
+      <c r="F102" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G102" s="36" t="s">
+        <v>3077</v>
+      </c>
+      <c r="H102" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I102" s="27" t="s">
+        <v>3078</v>
+      </c>
+      <c r="J102" s="32" t="s">
+        <v>3079</v>
+      </c>
+      <c r="K102" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L102" t="s">
+        <v>61</v>
+      </c>
+      <c r="M102" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N102" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14">
+      <c r="A103" s="4" t="s">
+        <v>3075</v>
+      </c>
+      <c r="B103" t="s">
+        <v>3080</v>
+      </c>
+      <c r="C103" s="17" t="s">
+        <v>443</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E103" s="38" t="s">
+        <v>3086</v>
+      </c>
+      <c r="F103" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G103" s="36" t="s">
+        <v>3087</v>
+      </c>
+      <c r="H103" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I103" s="2" t="s">
+        <v>3088</v>
+      </c>
+      <c r="J103" s="32" t="s">
+        <v>3089</v>
+      </c>
+      <c r="K103" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L103" t="s">
+        <v>61</v>
+      </c>
+      <c r="M103" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N103" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14">
+      <c r="A104" s="4" t="s">
+        <v>3091</v>
+      </c>
+      <c r="B104" t="s">
+        <v>3090</v>
+      </c>
+      <c r="C104" s="37" t="s">
+        <v>277</v>
+      </c>
+      <c r="D104" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E104" s="38" t="s">
+        <v>3092</v>
+      </c>
+      <c r="F104" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G104" s="39" t="s">
+        <v>3093</v>
+      </c>
+      <c r="H104" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I104" s="27" t="s">
+        <v>3094</v>
+      </c>
+      <c r="J104" s="32" t="s">
+        <v>3095</v>
+      </c>
+      <c r="K104" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L104" t="s">
+        <v>61</v>
+      </c>
+      <c r="M104" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N104" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14">
+      <c r="A105" s="4" t="s">
+        <v>3096</v>
+      </c>
+      <c r="B105" t="s">
+        <v>3097</v>
+      </c>
+      <c r="C105" s="17" t="s">
+        <v>3009</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="E105" s="38" t="s">
+        <v>3098</v>
+      </c>
+      <c r="F105" s="36" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G105" s="39" t="s">
+        <v>3099</v>
+      </c>
+      <c r="H105" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I105" s="27" t="s">
+        <v>3100</v>
+      </c>
+      <c r="J105" s="32" t="s">
+        <v>3101</v>
+      </c>
+      <c r="K105" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L105" t="s">
+        <v>61</v>
+      </c>
+      <c r="M105" s="7" t="s">
+        <v>702</v>
+      </c>
+      <c r="N105" t="s">
         <v>25</v>
       </c>
     </row>
@@ -14006,47 +14519,60 @@
     <hyperlink ref="I40" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
     <hyperlink ref="I41" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
     <hyperlink ref="I45" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="I58" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="J58" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="I59" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="J59" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="I60" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="J60" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="I61" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="J61" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="I62" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="J62" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="I67" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="J67" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="I68" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="J68" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="I69" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="J69" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="I70" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="J70" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="I71" r:id="rId37" xr:uid="{0B8C1C0C-47FA-451D-B2FE-12EFD0A111BF}"/>
-    <hyperlink ref="J71" r:id="rId38" xr:uid="{9FB12FE9-A0EE-496D-AFE6-FE36229B3E21}"/>
-    <hyperlink ref="J75" r:id="rId39" xr:uid="{4EB3F8F5-9523-4D51-98B0-69BB17DD7F5A}"/>
-    <hyperlink ref="J77" r:id="rId40" xr:uid="{3B031A79-4CEE-45C4-9A1F-B1D002630AFA}"/>
-    <hyperlink ref="I78" r:id="rId41" xr:uid="{93FF4324-911A-4833-81A9-4734C97681F3}"/>
-    <hyperlink ref="J78" r:id="rId42" xr:uid="{561B3DE3-61D1-42B0-B848-CBE9B1AFA9D1}"/>
-    <hyperlink ref="I79" r:id="rId43" xr:uid="{BE9E8745-188B-43B1-9452-32BEBE2AC112}"/>
-    <hyperlink ref="I87" r:id="rId44" xr:uid="{BBCF047A-9283-4540-8F64-F6AAC18C42BB}"/>
-    <hyperlink ref="J87" r:id="rId45" xr:uid="{85495087-0B60-4C63-9EAD-8FAFC16FDA87}"/>
-    <hyperlink ref="I88" r:id="rId46" xr:uid="{9D36823A-5DFC-4E8F-91FB-61378533EFF4}"/>
-    <hyperlink ref="J88" r:id="rId47" xr:uid="{56E53176-85EA-482A-8107-B53BC4B5A56E}"/>
-    <hyperlink ref="I89" r:id="rId48" xr:uid="{54C8C95D-2C8A-4B14-B3F8-1B69A2587372}"/>
-    <hyperlink ref="I82" r:id="rId49" xr:uid="{B234FDA3-9881-49C7-9757-E6B50F09E652}"/>
-    <hyperlink ref="I92" r:id="rId50" xr:uid="{629DD39D-5539-4595-B551-7C70898E50E5}"/>
-    <hyperlink ref="I93" r:id="rId51" xr:uid="{C9324AD1-D443-4B4A-88F6-7342BEEBC444}"/>
-    <hyperlink ref="J93" r:id="rId52" xr:uid="{02ABAA1D-5CBA-4945-9449-F11890AA00C1}"/>
-    <hyperlink ref="I94" r:id="rId53" xr:uid="{CD066ABD-A9CF-4B23-B64F-6EFECB0682A9}"/>
-    <hyperlink ref="J94" r:id="rId54" xr:uid="{DE191AC8-7CDC-47D8-8778-80293EDB2FDD}"/>
-    <hyperlink ref="I95" r:id="rId55" xr:uid="{CCA8EE89-F6B4-4DE6-8266-D2E2C7A801D9}"/>
-    <hyperlink ref="J95" r:id="rId56" xr:uid="{3EA9C5B0-8F07-472C-B534-F158D1D13832}"/>
-    <hyperlink ref="I96" r:id="rId57" xr:uid="{84DAD3FB-EB5D-446A-B122-0A99A60B6E95}"/>
-    <hyperlink ref="J96" r:id="rId58" xr:uid="{44B094DB-343C-49F4-A023-566CEE808AE0}"/>
-    <hyperlink ref="I97" r:id="rId59" xr:uid="{890D1BEC-53E9-4E41-AB45-508A74C3ACB5}"/>
+    <hyperlink ref="J58" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="I59" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="J59" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="I60" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="J60" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="I61" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="J61" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="I62" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="J62" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="I67" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="J67" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="I68" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="J68" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="I69" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="J69" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="I70" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="J70" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="I71" r:id="rId36" xr:uid="{0B8C1C0C-47FA-451D-B2FE-12EFD0A111BF}"/>
+    <hyperlink ref="J71" r:id="rId37" xr:uid="{9FB12FE9-A0EE-496D-AFE6-FE36229B3E21}"/>
+    <hyperlink ref="J75" r:id="rId38" xr:uid="{4EB3F8F5-9523-4D51-98B0-69BB17DD7F5A}"/>
+    <hyperlink ref="J77" r:id="rId39" xr:uid="{3B031A79-4CEE-45C4-9A1F-B1D002630AFA}"/>
+    <hyperlink ref="I78" r:id="rId40" xr:uid="{93FF4324-911A-4833-81A9-4734C97681F3}"/>
+    <hyperlink ref="J78" r:id="rId41" xr:uid="{561B3DE3-61D1-42B0-B848-CBE9B1AFA9D1}"/>
+    <hyperlink ref="I79" r:id="rId42" xr:uid="{BE9E8745-188B-43B1-9452-32BEBE2AC112}"/>
+    <hyperlink ref="I87" r:id="rId43" xr:uid="{BBCF047A-9283-4540-8F64-F6AAC18C42BB}"/>
+    <hyperlink ref="J87" r:id="rId44" xr:uid="{85495087-0B60-4C63-9EAD-8FAFC16FDA87}"/>
+    <hyperlink ref="I88" r:id="rId45" xr:uid="{9D36823A-5DFC-4E8F-91FB-61378533EFF4}"/>
+    <hyperlink ref="J88" r:id="rId46" xr:uid="{56E53176-85EA-482A-8107-B53BC4B5A56E}"/>
+    <hyperlink ref="I89" r:id="rId47" xr:uid="{54C8C95D-2C8A-4B14-B3F8-1B69A2587372}"/>
+    <hyperlink ref="I82" r:id="rId48" xr:uid="{B234FDA3-9881-49C7-9757-E6B50F09E652}"/>
+    <hyperlink ref="I92" r:id="rId49" xr:uid="{629DD39D-5539-4595-B551-7C70898E50E5}"/>
+    <hyperlink ref="I93" r:id="rId50" xr:uid="{C9324AD1-D443-4B4A-88F6-7342BEEBC444}"/>
+    <hyperlink ref="J93" r:id="rId51" xr:uid="{02ABAA1D-5CBA-4945-9449-F11890AA00C1}"/>
+    <hyperlink ref="I94" r:id="rId52" xr:uid="{CD066ABD-A9CF-4B23-B64F-6EFECB0682A9}"/>
+    <hyperlink ref="J94" r:id="rId53" xr:uid="{DE191AC8-7CDC-47D8-8778-80293EDB2FDD}"/>
+    <hyperlink ref="I95" r:id="rId54" xr:uid="{CCA8EE89-F6B4-4DE6-8266-D2E2C7A801D9}"/>
+    <hyperlink ref="J95" r:id="rId55" xr:uid="{3EA9C5B0-8F07-472C-B534-F158D1D13832}"/>
+    <hyperlink ref="I96" r:id="rId56" xr:uid="{84DAD3FB-EB5D-446A-B122-0A99A60B6E95}"/>
+    <hyperlink ref="J96" r:id="rId57" xr:uid="{44B094DB-343C-49F4-A023-566CEE808AE0}"/>
+    <hyperlink ref="I97" r:id="rId58" xr:uid="{890D1BEC-53E9-4E41-AB45-508A74C3ACB5}"/>
+    <hyperlink ref="I98" r:id="rId59" xr:uid="{02959CD1-6C86-4D79-AEAF-97CB61B96D25}"/>
+    <hyperlink ref="I99" r:id="rId60" xr:uid="{3688B733-FC93-4BD4-BD33-E91280D03ADE}"/>
+    <hyperlink ref="J99" r:id="rId61" xr:uid="{8F40B277-7A81-44F0-8336-1DAD2949332A}"/>
+    <hyperlink ref="J100" r:id="rId62" xr:uid="{DE00D900-0F4C-4258-946C-9BE0F3013002}"/>
+    <hyperlink ref="J101" r:id="rId63" xr:uid="{34919784-5679-4717-9885-2A1A0C412CE4}"/>
+    <hyperlink ref="I102" r:id="rId64" xr:uid="{470193F3-D16D-4EAC-841E-3D81FB5774A9}"/>
+    <hyperlink ref="J102" r:id="rId65" xr:uid="{2ED12714-63A2-41C3-AB62-1774DD1F70BA}"/>
+    <hyperlink ref="I58" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="I103" r:id="rId67" xr:uid="{4D721F85-2836-4ADB-B264-71CBD8B98BD8}"/>
+    <hyperlink ref="J103" r:id="rId68" xr:uid="{3925AD24-90B0-4A5C-A46D-F80F8E61579F}"/>
+    <hyperlink ref="I104" r:id="rId69" xr:uid="{478CCF2E-AB97-48E1-A38C-995964394AC8}"/>
+    <hyperlink ref="J104" r:id="rId70" xr:uid="{F9BBE179-DB54-4835-A14E-4454CA18A6AE}"/>
+    <hyperlink ref="I105" r:id="rId71" xr:uid="{ABB87B28-8AD2-4BF8-B4D7-500E78A25472}"/>
+    <hyperlink ref="J105" r:id="rId72" xr:uid="{F543587D-0A3E-429A-8125-C651D94CA2A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
010-0142, 010-0143, 010-0144, 010-0145, 010-0146, 010-0147, 010-0148, 010-0149, 015-0004 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D670F-F1D6-4AB3-A5EB-F0ABEB79F458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBCA921-DBC1-4B06-9069-00F4B7B41B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32295" yWindow="2355" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32295" yWindow="2355" windowWidth="14610" windowHeight="15585" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6207" uniqueCount="3102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6333" uniqueCount="3162">
   <si>
     <t>ID</t>
   </si>
@@ -9348,6 +9348,186 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012209073?qs=sPbYRqrBIVm8PsM2ljQIMg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0142</t>
+  </si>
+  <si>
+    <t>010-0143</t>
+  </si>
+  <si>
+    <t>010-0144</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS &lt;0.05 Ohms 0.1 W Jumper 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112116001</t>
+  </si>
+  <si>
+    <t>710-560112116001</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116001.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116001?qs=mELouGlnn3dlnHYj7TecuA%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 5.1 kOhms 5 % 0.25 W 0805 AEC-Q200</t>
+  </si>
+  <si>
+    <t>5.1kΩ 250mW  ±5%</t>
+  </si>
+  <si>
+    <t>560112120019</t>
+  </si>
+  <si>
+    <t>710-560112120019</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112120019.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112120019?qs=mELouGlnn3d1l%252BnKb9nSgA%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 330 Ohms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>330Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116020</t>
+  </si>
+  <si>
+    <t>710-560112116020</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116020.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116020?qs=mELouGlnn3dXlpeR%252Bp7gkg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0145</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 10 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112116005</t>
+  </si>
+  <si>
+    <t>710-560112116005</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116005.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116005?qs=mELouGlnn3dMVSPHwBGouA%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0146</t>
+  </si>
+  <si>
+    <t>010-0147</t>
+  </si>
+  <si>
+    <t>010-0148</t>
+  </si>
+  <si>
+    <t>010-0149</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116032?qs=mELouGlnn3dPZZEXKb4zAQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 1.8 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>1.8kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116032</t>
+  </si>
+  <si>
+    <t>710-560112116032</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116032.pdf</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 49.9 Ohms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>49.9Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116133</t>
+  </si>
+  <si>
+    <t>710-560112116133</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116133.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116133?qs=mELouGlnn3fu%2F7K9tg3bDw%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 4.02 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112116093</t>
+  </si>
+  <si>
+    <t>710-560112116093</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116093.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116093?qs=mELouGlnn3dikxUEmUbjog%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 10 Ohms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>10Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116013</t>
+  </si>
+  <si>
+    <t>710-560112116013</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116013.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116013?qs=mELouGlnn3f7quibYlpocQ%3D%3D</t>
+  </si>
+  <si>
+    <t>015-0004</t>
+  </si>
+  <si>
+    <t>Resistores de detección de corriente - SMD WRIS-PSMC 10mOhms 1% 2512 2W 100ppm/C</t>
+  </si>
+  <si>
+    <t>10mΩ 2W ±1%</t>
+  </si>
+  <si>
+    <t>580070763010</t>
+  </si>
+  <si>
+    <t>710-580070763010</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/580070763010.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/580070763010?qs=amGC7iS6iy%2FEZvIQbPzDXw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -9574,10 +9754,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -14153,19 +14333,19 @@
       <c r="B98" t="s">
         <v>3051</v>
       </c>
-      <c r="C98" s="37" t="s">
+      <c r="C98" s="17" t="s">
         <v>3052</v>
       </c>
       <c r="D98" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E98" s="38" t="s">
+      <c r="E98" s="36" t="s">
         <v>3081</v>
       </c>
-      <c r="F98" s="36" t="s">
+      <c r="F98" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G98" s="36" t="s">
+      <c r="G98" s="3" t="s">
         <v>3053</v>
       </c>
       <c r="H98" s="16" t="s">
@@ -14197,19 +14377,19 @@
       <c r="B99" t="s">
         <v>3060</v>
       </c>
-      <c r="C99" s="37" t="s">
+      <c r="C99" s="17" t="s">
         <v>3061</v>
       </c>
       <c r="D99" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E99" s="38" t="s">
+      <c r="E99" s="36" t="s">
         <v>3083</v>
       </c>
-      <c r="F99" s="36" t="s">
+      <c r="F99" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G99" s="36" t="s">
+      <c r="G99" s="3" t="s">
         <v>3062</v>
       </c>
       <c r="H99" s="16" t="s">
@@ -14241,16 +14421,16 @@
       <c r="B100" t="s">
         <v>3065</v>
       </c>
-      <c r="C100" s="37" t="s">
+      <c r="C100" s="17" t="s">
         <v>3066</v>
       </c>
       <c r="D100" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E100" s="38" t="s">
+      <c r="E100" s="36" t="s">
         <v>3082</v>
       </c>
-      <c r="F100" s="36" t="s">
+      <c r="F100" s="3" t="s">
         <v>2100</v>
       </c>
       <c r="G100" t="s">
@@ -14285,19 +14465,19 @@
       <c r="B101" t="s">
         <v>3070</v>
       </c>
-      <c r="C101" s="37" t="s">
+      <c r="C101" s="17" t="s">
         <v>3016</v>
       </c>
       <c r="D101" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="E101" s="38" t="s">
+      <c r="E101" s="36" t="s">
         <v>3084</v>
       </c>
-      <c r="F101" s="36" t="s">
+      <c r="F101" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G101" s="36" t="s">
+      <c r="G101" s="3" t="s">
         <v>3071</v>
       </c>
       <c r="H101" s="16" t="s">
@@ -14329,19 +14509,19 @@
       <c r="B102" t="s">
         <v>3074</v>
       </c>
-      <c r="C102" s="37" t="s">
+      <c r="C102" s="17" t="s">
         <v>3076</v>
       </c>
       <c r="D102" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E102" s="38" t="s">
+      <c r="E102" s="36" t="s">
         <v>3085</v>
       </c>
-      <c r="F102" s="36" t="s">
+      <c r="F102" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G102" s="36" t="s">
+      <c r="G102" s="3" t="s">
         <v>3077</v>
       </c>
       <c r="H102" s="16" t="s">
@@ -14379,13 +14559,13 @@
       <c r="D103" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E103" s="38" t="s">
+      <c r="E103" s="36" t="s">
         <v>3086</v>
       </c>
-      <c r="F103" s="36" t="s">
+      <c r="F103" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G103" s="36" t="s">
+      <c r="G103" s="3" t="s">
         <v>3087</v>
       </c>
       <c r="H103" s="16" t="s">
@@ -14417,19 +14597,19 @@
       <c r="B104" t="s">
         <v>3090</v>
       </c>
-      <c r="C104" s="37" t="s">
+      <c r="C104" s="17" t="s">
         <v>277</v>
       </c>
       <c r="D104" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E104" s="38" t="s">
+      <c r="E104" s="36" t="s">
         <v>3092</v>
       </c>
-      <c r="F104" s="36" t="s">
+      <c r="F104" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G104" s="39" t="s">
+      <c r="G104" s="31" t="s">
         <v>3093</v>
       </c>
       <c r="H104" s="16" t="s">
@@ -14467,13 +14647,13 @@
       <c r="D105" s="13" t="s">
         <v>520</v>
       </c>
-      <c r="E105" s="38" t="s">
+      <c r="E105" s="36" t="s">
         <v>3098</v>
       </c>
-      <c r="F105" s="36" t="s">
+      <c r="F105" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G105" s="39" t="s">
+      <c r="G105" s="31" t="s">
         <v>3099</v>
       </c>
       <c r="H105" s="16" t="s">
@@ -21378,10 +21558,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N142"/>
+  <dimension ref="A1:N151"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -27632,6 +27813,361 @@
       <c r="N142" t="s">
         <v>25</v>
       </c>
+    </row>
+    <row r="143" spans="1:14">
+      <c r="A143" s="16" t="s">
+        <v>3102</v>
+      </c>
+      <c r="B143" s="37" t="s">
+        <v>3105</v>
+      </c>
+      <c r="C143" s="17" t="s">
+        <v>893</v>
+      </c>
+      <c r="D143" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E143" s="38" t="s">
+        <v>3106</v>
+      </c>
+      <c r="F143" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G143" s="37" t="s">
+        <v>3107</v>
+      </c>
+      <c r="H143" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I143" s="27" t="s">
+        <v>3108</v>
+      </c>
+      <c r="J143" s="27" t="s">
+        <v>3109</v>
+      </c>
+      <c r="K143" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L143" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M143" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N143" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14">
+      <c r="A144" s="16" t="s">
+        <v>3103</v>
+      </c>
+      <c r="B144" s="37" t="s">
+        <v>3110</v>
+      </c>
+      <c r="C144" s="37" t="s">
+        <v>3111</v>
+      </c>
+      <c r="D144" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E144" s="38" t="s">
+        <v>3112</v>
+      </c>
+      <c r="F144" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G144" s="37" t="s">
+        <v>3113</v>
+      </c>
+      <c r="H144" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I144" s="27" t="s">
+        <v>3114</v>
+      </c>
+      <c r="J144" s="32" t="s">
+        <v>3115</v>
+      </c>
+      <c r="K144" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L144" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M144" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N144" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14">
+      <c r="A145" s="16" t="s">
+        <v>3104</v>
+      </c>
+      <c r="B145" s="37" t="s">
+        <v>3116</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>3117</v>
+      </c>
+      <c r="D145" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E145" s="38" t="s">
+        <v>3118</v>
+      </c>
+      <c r="F145" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G145" s="37" t="s">
+        <v>3119</v>
+      </c>
+      <c r="H145" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I145" s="27" t="s">
+        <v>3120</v>
+      </c>
+      <c r="J145" s="32" t="s">
+        <v>3121</v>
+      </c>
+      <c r="K145" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L145" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M145" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N145" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="146" spans="1:14">
+      <c r="A146" s="16" t="s">
+        <v>3122</v>
+      </c>
+      <c r="B146" s="37" t="s">
+        <v>3123</v>
+      </c>
+      <c r="C146" s="7" t="s">
+        <v>1149</v>
+      </c>
+      <c r="D146" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E146" s="38" t="s">
+        <v>3124</v>
+      </c>
+      <c r="F146" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G146" s="37" t="s">
+        <v>3125</v>
+      </c>
+      <c r="H146" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I146" s="27" t="s">
+        <v>3126</v>
+      </c>
+      <c r="J146" t="s">
+        <v>3127</v>
+      </c>
+      <c r="K146" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L146" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M146" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N146" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="147" spans="1:14">
+      <c r="A147" s="16" t="s">
+        <v>3128</v>
+      </c>
+      <c r="B147" s="37" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C147" s="17" t="s">
+        <v>3134</v>
+      </c>
+      <c r="D147" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E147" s="38" t="s">
+        <v>3135</v>
+      </c>
+      <c r="F147" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G147" s="37" t="s">
+        <v>3136</v>
+      </c>
+      <c r="H147" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I147" s="27" t="s">
+        <v>3137</v>
+      </c>
+      <c r="J147" s="27" t="s">
+        <v>3132</v>
+      </c>
+      <c r="K147" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L147" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M147" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N147" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="148" spans="1:14">
+      <c r="A148" s="16" t="s">
+        <v>3129</v>
+      </c>
+      <c r="B148" s="37" t="s">
+        <v>3138</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>3139</v>
+      </c>
+      <c r="D148" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E148" s="36" t="s">
+        <v>3140</v>
+      </c>
+      <c r="F148" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G148" t="s">
+        <v>3141</v>
+      </c>
+      <c r="H148" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I148" s="27" t="s">
+        <v>3142</v>
+      </c>
+      <c r="J148" s="32" t="s">
+        <v>3143</v>
+      </c>
+      <c r="K148" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L148" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M148" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N148" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="149" spans="1:14">
+      <c r="A149" s="16" t="s">
+        <v>3130</v>
+      </c>
+      <c r="B149" s="37" t="s">
+        <v>3144</v>
+      </c>
+      <c r="C149" s="16" t="s">
+        <v>1610</v>
+      </c>
+      <c r="D149" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E149" s="39" t="s">
+        <v>3145</v>
+      </c>
+      <c r="F149" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G149" s="37" t="s">
+        <v>3146</v>
+      </c>
+      <c r="H149" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I149" s="27" t="s">
+        <v>3147</v>
+      </c>
+      <c r="J149" s="32" t="s">
+        <v>3148</v>
+      </c>
+      <c r="K149" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L149" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M149" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N149" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="150" spans="1:14">
+      <c r="A150" s="16" t="s">
+        <v>3131</v>
+      </c>
+      <c r="B150" s="37" t="s">
+        <v>3149</v>
+      </c>
+      <c r="C150" s="16" t="s">
+        <v>3150</v>
+      </c>
+      <c r="D150" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E150" s="39" t="s">
+        <v>3151</v>
+      </c>
+      <c r="F150" s="37" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G150" s="37" t="s">
+        <v>3152</v>
+      </c>
+      <c r="H150" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I150" s="27" t="s">
+        <v>3153</v>
+      </c>
+      <c r="J150" s="32" t="s">
+        <v>3154</v>
+      </c>
+      <c r="K150" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L150" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M150" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N150" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="151" spans="1:14">
+      <c r="A151" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
@@ -27728,15 +28264,30 @@
     <hyperlink ref="J137" r:id="rId90" xr:uid="{270FAB0D-B47D-4805-A699-C4BB16679313}"/>
     <hyperlink ref="I140" r:id="rId91" xr:uid="{AF66F37C-DEF2-4C02-B09E-78216E8A0857}"/>
     <hyperlink ref="J140" r:id="rId92" xr:uid="{5C7EACC9-1558-4F25-8631-38E695251F20}"/>
+    <hyperlink ref="I143" r:id="rId93" xr:uid="{C01DAE4E-F612-4FC5-8D22-5944A3E92FB0}"/>
+    <hyperlink ref="J143" r:id="rId94" xr:uid="{06184D44-AC67-4E67-A84F-AA99CD34AEB6}"/>
+    <hyperlink ref="I144" r:id="rId95" xr:uid="{0BA127CF-9F17-46D3-8575-41BD9AD2CDB0}"/>
+    <hyperlink ref="J144" r:id="rId96" xr:uid="{4E510238-24C1-436C-B1B1-DC4BBBD46327}"/>
+    <hyperlink ref="I145" r:id="rId97" xr:uid="{4DAB6FCC-DE9F-47EE-8889-AF483417A869}"/>
+    <hyperlink ref="J145" r:id="rId98" xr:uid="{5B1AE306-EC71-4D08-9387-CBEBC35C11D8}"/>
+    <hyperlink ref="I146" r:id="rId99" xr:uid="{4917BA3D-010B-4FC0-897E-454B864E1931}"/>
+    <hyperlink ref="I147" r:id="rId100" xr:uid="{CA0F4A3B-5CA6-4B60-95A8-D5832F92DB0C}"/>
+    <hyperlink ref="J147" r:id="rId101" xr:uid="{E9DB0A36-8554-4D76-81C9-42407166BE48}"/>
+    <hyperlink ref="I148" r:id="rId102" xr:uid="{243AD2D2-4D58-4692-93A4-89A4B3090386}"/>
+    <hyperlink ref="J148" r:id="rId103" xr:uid="{081B7EBC-5724-44C6-B7A8-0F110E0A5EB2}"/>
+    <hyperlink ref="I149" r:id="rId104" xr:uid="{66E45401-3B0B-41F7-9778-7BDA8C0C1404}"/>
+    <hyperlink ref="J149" r:id="rId105" xr:uid="{1A42DE35-CA7D-4B83-ACC4-F85A80B83C4C}"/>
+    <hyperlink ref="I150" r:id="rId106" xr:uid="{866C2F71-4468-4B2A-8F29-42D5363F2AE6}"/>
+    <hyperlink ref="J150" r:id="rId107" xr:uid="{D030A4B2-39C9-4251-A1F3-D75C066D2B9B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId93"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId108"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="20.26953125" customWidth="1"/>
@@ -27918,6 +28469,50 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>3155</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3156</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3157</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>3158</v>
+      </c>
+      <c r="F5" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G5" t="s">
+        <v>3159</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>3160</v>
+      </c>
+      <c r="J5" t="s">
+        <v>3161</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>1647</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
@@ -27926,6 +28521,7 @@
     <hyperlink ref="I3" r:id="rId3" xr:uid="{EDE33321-C187-4A8F-8366-9AEDB9FF4C7B}"/>
     <hyperlink ref="I4" r:id="rId4" xr:uid="{DA619253-40A2-482C-A99F-F72A13182916}"/>
     <hyperlink ref="J4" r:id="rId5" xr:uid="{65BF95D6-EB54-41F9-8886-7DFC774FFE44}"/>
+    <hyperlink ref="I5" r:id="rId6" xr:uid="{E9BE5DD3-9340-403D-9879-EBA54F1D68BE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
070-0004, 070-0005, 043-0001, 055-0001 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B16B84C-A795-4F12-9527-5B4F35DED38B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E7BE8E-5349-4841-9AC6-E1B10AAFD1F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="16200" windowHeight="9970" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -24,13 +24,15 @@
     <sheet name="032 - Diode - TVS" sheetId="14" r:id="rId9"/>
     <sheet name="033 - Diode - LED" sheetId="12" r:id="rId10"/>
     <sheet name="040 - Fuses" sheetId="10" r:id="rId11"/>
-    <sheet name="045 - Crystal" sheetId="19" r:id="rId12"/>
-    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId13"/>
-    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId14"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId15"/>
-    <sheet name="090 - Processor" sheetId="18" r:id="rId16"/>
-    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId17"/>
-    <sheet name="110 - Connectors" sheetId="13" r:id="rId18"/>
+    <sheet name="043 - Transistors" sheetId="21" r:id="rId12"/>
+    <sheet name="045 - Crystal" sheetId="19" r:id="rId13"/>
+    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId14"/>
+    <sheet name="055 - Drivers" sheetId="20" r:id="rId15"/>
+    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId16"/>
+    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId17"/>
+    <sheet name="090 - Processor" sheetId="18" r:id="rId18"/>
+    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId19"/>
+    <sheet name="110 - Connectors" sheetId="13" r:id="rId20"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6333" uniqueCount="3163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6417" uniqueCount="3201">
   <si>
     <t>ID</t>
   </si>
@@ -9531,6 +9533,120 @@
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>055-0001</t>
+  </si>
+  <si>
+    <t>Controladores de puerta con aislamiento galvánico Automotive 5.7kVrms 10A single-channel i A 595-UCC21710QDWQ1</t>
+  </si>
+  <si>
+    <t>SOIC-16</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Drivers.SchLib</t>
+  </si>
+  <si>
+    <t>UCC21710QDWRQ1</t>
+  </si>
+  <si>
+    <t>595-UCC21710QDWRQ1</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/ucc21710-q1.pdf?ts=1780997053821&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FUCC21710-Q1</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/UCC21710QDWRQ1?qs=9r4v7xj2LnlqS59tMWgtnw%3D%3D</t>
+  </si>
+  <si>
+    <t>UCC21710</t>
+  </si>
+  <si>
+    <t>043-0001</t>
+  </si>
+  <si>
+    <t>MOSFET 150 V, N-Ch, 3.8 mOhms max, Automotive MOSFET, TOLT (10x15)</t>
+  </si>
+  <si>
+    <t>PG-HSOG-8-1</t>
+  </si>
+  <si>
+    <t>IAUTN15S6N025GATMA1</t>
+  </si>
+  <si>
+    <t>726-IAUTN15S6N025GAT</t>
+  </si>
+  <si>
+    <t>Infineon Technologies</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/70/1/Infineon_IAUTN15S6N025G_DataSheet_v01_00_EN.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Infineon-Technologies/IAUTN15S6N025GATMA1?qs=lxPAlgZqN%2Fyxd40SMd9ESg%3D%3D</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>IAUTN15S6N025</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Transistors.SchLib</t>
+  </si>
+  <si>
+    <t>070-0004</t>
+  </si>
+  <si>
+    <t>Convertidores DC/DC para montaje pasante 10W DC/DC Converter isolated, regulated in a PCB Mount Plastic Case</t>
+  </si>
+  <si>
+    <t>110V-24V</t>
+  </si>
+  <si>
+    <t>31.8x20.3x10.6mm</t>
+  </si>
+  <si>
+    <t>TEN 10-11015WIRH</t>
+  </si>
+  <si>
+    <t>495-TEN10-11015WIRH</t>
+  </si>
+  <si>
+    <t>https://www.tracopower.com/ten10wirh-datasheet</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TRACO-Power/TEN-10-11015WIRH?qs=A6eO%252BMLsxmQM8M6%2FnJVPNg%3D%3D</t>
+  </si>
+  <si>
+    <t>TEN 10-110</t>
+  </si>
+  <si>
+    <t>070-0005</t>
+  </si>
+  <si>
+    <t>Convertidores DC/DC para montaje pasante 2W 24-15VIN 5VOUT DC/DC</t>
+  </si>
+  <si>
+    <t>24V-(15,-5)V</t>
+  </si>
+  <si>
+    <t>19.5x9.8x12.5mm</t>
+  </si>
+  <si>
+    <t>MGJ2D241505SC</t>
+  </si>
+  <si>
+    <t>580-MGJ2D241505SC</t>
+  </si>
+  <si>
+    <t>Murata Power Solutions</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/76/1/kdc-mgj2.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Murata-Power-Solutions/MGJ2D241505SC?qs=xLDY6iXSiQZSXeU7bFDLTA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -16813,6 +16929,108 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FAFF3B6-AF11-4BFB-8078-829FF6F2F366}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>3172</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3173</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3180</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3174</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3175</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3177</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3176</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>3178</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>3179</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3181</v>
+      </c>
+      <c r="L2" s="34" t="s">
+        <v>3182</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3174</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{71BC0DAF-9651-41D4-BC90-0CA5C5CA063D}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{B8956BA2-569B-4007-9354-F99A76E81F8D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E5535EA-E186-4751-BC7F-9B3A0221302E}">
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -16961,7 +17179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -17211,7 +17429,109 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201D74E2-3547-4E9B-8216-09A22645AC2A}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>3163</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3164</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3165</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3167</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3168</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>3169</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>3170</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3171</v>
+      </c>
+      <c r="L2" t="s">
+        <v>3166</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3165</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{8F7A6184-A0A3-4957-BEC8-F3E55B833A4E}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{EFC059D7-FF37-4BE0-B7C4-41524A59BFAA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -17265,9 +17585,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="17.54296875" customWidth="1"/>
@@ -17449,17 +17769,109 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>3183</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3184</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3185</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3186</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3187</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" t="s">
+        <v>3188</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>3189</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>3190</v>
+      </c>
+      <c r="K5" t="s">
+        <v>3191</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M5" t="s">
+        <v>3191</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>3192</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3193</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3194</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3195</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3196</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3198</v>
+      </c>
+      <c r="G6" t="s">
+        <v>3197</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>3199</v>
+      </c>
+      <c r="J6" t="s">
+        <v>3200</v>
+      </c>
+      <c r="K6" t="s">
+        <v>3196</v>
+      </c>
+      <c r="L6" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M6" t="s">
+        <v>3196</v>
+      </c>
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{08280A44-0F58-4FDE-B5FD-3A95A0F423CB}"/>
     <hyperlink ref="J2" r:id="rId2" xr:uid="{85F326FF-BAE0-4072-815D-1EE4E7995C53}"/>
+    <hyperlink ref="I5" r:id="rId3" xr:uid="{38CEA448-03C1-4130-9D22-378144C1B83E}"/>
+    <hyperlink ref="J5" r:id="rId4" xr:uid="{178AE8D2-EC1F-4144-807A-F49730BDAEE7}"/>
+    <hyperlink ref="I6" r:id="rId5" xr:uid="{C6B22468-8A2D-4CA0-8E30-C5E1C054C475}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
   <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -17567,7 +17979,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18650,7 +19062,114 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>2906</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2907</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2908</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2909</v>
+      </c>
+      <c r="E2">
+        <v>860020675022</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2910</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2911</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2912</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2913</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2914</v>
+      </c>
+      <c r="L2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" t="s">
+        <v>2915</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="M3" s="7"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{BB2EDAB8-75EB-46D2-BA14-384BF06E1A6E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
   <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -21444,113 +21963,6 @@
     <hyperlink ref="I56" r:id="rId51" xr:uid="{CE941FB5-1D41-41B6-9CFD-C1256871C52E}"/>
     <hyperlink ref="J57" r:id="rId52" xr:uid="{72ED46D3-1227-48FD-9800-7E78EA501F81}"/>
     <hyperlink ref="I57" r:id="rId53" xr:uid="{30F29B76-2559-4C1E-A762-9F9E7C2882A4}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" t="s">
-        <v>2906</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2907</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2908</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2909</v>
-      </c>
-      <c r="E2">
-        <v>860020675022</v>
-      </c>
-      <c r="F2" t="s">
-        <v>2910</v>
-      </c>
-      <c r="G2" t="s">
-        <v>2911</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>2912</v>
-      </c>
-      <c r="J2" t="s">
-        <v>2913</v>
-      </c>
-      <c r="K2" t="s">
-        <v>2914</v>
-      </c>
-      <c r="L2" t="s">
-        <v>61</v>
-      </c>
-      <c r="M2" t="s">
-        <v>2915</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="M3" s="7"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{BB2EDAB8-75EB-46D2-BA14-384BF06E1A6E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
010-0150, 010-0151, 010-0152, 090-0002, 110-0062 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944AA604-5C9C-4A07-B4A8-289EF1B0937A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDDD5F2-53E9-4AE3-BB92-BF21129E6B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,16 @@
     <sheet name="032 - Diode - TVS" sheetId="14" r:id="rId10"/>
     <sheet name="033 - Diode - LED" sheetId="12" r:id="rId11"/>
     <sheet name="040 - Fuses" sheetId="10" r:id="rId12"/>
-    <sheet name="043 - Transistors" sheetId="21" r:id="rId13"/>
-    <sheet name="045 - Crystal" sheetId="19" r:id="rId14"/>
-    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId15"/>
-    <sheet name="055 - Drivers" sheetId="20" r:id="rId16"/>
-    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId17"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId18"/>
-    <sheet name="090 - Processor" sheetId="18" r:id="rId19"/>
-    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId20"/>
-    <sheet name="110 - Connectors" sheetId="13" r:id="rId21"/>
+    <sheet name="042 - NTC" sheetId="23" r:id="rId13"/>
+    <sheet name="043 - Transistors" sheetId="21" r:id="rId14"/>
+    <sheet name="045 - Crystal" sheetId="19" r:id="rId15"/>
+    <sheet name="050 - ICs - Analog" sheetId="2" r:id="rId16"/>
+    <sheet name="055 - Drivers" sheetId="20" r:id="rId17"/>
+    <sheet name="060 - ICs - Digital" sheetId="3" r:id="rId18"/>
+    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId19"/>
+    <sheet name="090 - Processor" sheetId="18" r:id="rId20"/>
+    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId21"/>
+    <sheet name="110 - Connectors" sheetId="13" r:id="rId22"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6472" uniqueCount="3228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6557" uniqueCount="3263">
   <si>
     <t>ID</t>
   </si>
@@ -9729,6 +9730,111 @@
   </si>
   <si>
     <t>CAP SMD 1812</t>
+  </si>
+  <si>
+    <t>010-0150</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD CRGP 2512 15R 1% SMD Resistor</t>
+  </si>
+  <si>
+    <t>15Ω 2W ±1%</t>
+  </si>
+  <si>
+    <t>2512</t>
+  </si>
+  <si>
+    <t>CRGP2512F15R</t>
+  </si>
+  <si>
+    <t>279-CRGP2512F15R</t>
+  </si>
+  <si>
+    <t>https://www.te.com/commerce/DocumentDelivery/DDEController?Action=srchrtrv&amp;DocNm=9-1773463-9&amp;DocType=Data%20Sheet&amp;DocLang=English&amp;PartCntxt=2176331-3&amp;DocFormat=pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TE-Connectivity-Holsworthy/CRGP2512F15R?qs=sGAEpiMZZMtlubZbdhIBIOInyB5Ysv8smEFBCggATNk%3D</t>
+  </si>
+  <si>
+    <t>010-0151</t>
+  </si>
+  <si>
+    <t>010-0152</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 0.75W 6.8ohms 1% High Power AEC-Q200</t>
+  </si>
+  <si>
+    <t>6.8Ω 750mW ±1%</t>
+  </si>
+  <si>
+    <t>CRCW06036R80FKEAHP</t>
+  </si>
+  <si>
+    <t>71-CRCW06036R80FKEAH</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/CRCW06036R80FKEAHP?qs=KWN%252BoghGvh0VLghfFgThPw%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 0.75W 8.2ohms 1% High Power AEC-Q200</t>
+  </si>
+  <si>
+    <t>8.2Ω 750mW ±1%</t>
+  </si>
+  <si>
+    <t>CRCW06038R20FKEAHP</t>
+  </si>
+  <si>
+    <t>71-CRCW06038R20FKEAH</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/CRCW06038R20FKEAHP?qs=40TFAHZMFveezrMfyoByGQ%3D%3D</t>
+  </si>
+  <si>
+    <t>090-0002</t>
+  </si>
+  <si>
+    <t>Equipos y placas de desarrollo - TMS320 C2000 F28379D DELFIN O LAUNCHPAD</t>
+  </si>
+  <si>
+    <t>LAUNCHXL-F28379D</t>
+  </si>
+  <si>
+    <t>595-LAUNCHXL-F28379D</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ug/sprui77c/sprui77c.pdf?ts=1639427205104&amp;ref_url=https%253A%252F%252Fwww.google.com%252F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/LAUNCHXL-F28379D?qs=8%252Br4Hz5Xir%252BwQNYYjOfeVA%3D%3D</t>
+  </si>
+  <si>
+    <t>110-0062</t>
+  </si>
+  <si>
+    <t>SSK03-MPH-254-B20</t>
+  </si>
+  <si>
+    <t>Same Sky</t>
+  </si>
+  <si>
+    <t>179-SSK03MPH254B20</t>
+  </si>
+  <si>
+    <t>20P</t>
+  </si>
+  <si>
+    <t>Alojamientos de cables y cabecera 2.54mm Male Header, 2X20pin, Straight, PA6T, Gold Flash</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/6118/1/ssk03_mph_254.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Same-Sky/SSK03-MPH-254-B20?qs=G4MbTVxgV4GvjhUhLLGrSQ%3D%3D</t>
+  </si>
+  <si>
+    <t>CONN 20P</t>
   </si>
 </sst>
 </file>
@@ -9779,12 +9885,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -9796,24 +9904,28 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -9829,17 +9941,20 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -9957,9 +10072,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -14887,10 +15002,10 @@
       <c r="B106" t="s">
         <v>3220</v>
       </c>
-      <c r="C106" s="37" t="s">
+      <c r="C106" s="17" t="s">
         <v>3221</v>
       </c>
-      <c r="D106" s="38" t="s">
+      <c r="D106" s="13" t="s">
         <v>3222</v>
       </c>
       <c r="E106" s="36" t="s">
@@ -14899,7 +15014,7 @@
       <c r="F106" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G106" s="39" t="s">
+      <c r="G106" s="31" t="s">
         <v>3224</v>
       </c>
       <c r="H106" s="16" t="s">
@@ -14917,10 +15032,10 @@
       <c r="L106" t="s">
         <v>61</v>
       </c>
-      <c r="M106" s="40" t="s">
+      <c r="M106" s="7" t="s">
         <v>3227</v>
       </c>
-      <c r="N106" s="40" t="s">
+      <c r="N106" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -18083,6 +18198,60 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB954362-0CE9-4363-A149-F8AA1E8DAAF4}">
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FAFF3B6-AF11-4BFB-8078-829FF6F2F366}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18184,7 +18353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E5535EA-E186-4751-BC7F-9B3A0221302E}">
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18333,7 +18502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18583,7 +18752,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201D74E2-3547-4E9B-8216-09A22645AC2A}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18685,7 +18854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
   <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -18739,7 +18908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -19025,114 +19194,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" s="33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="33" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="33" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="33" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="33" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="33" t="s">
-        <v>3019</v>
-      </c>
-      <c r="I1" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>3020</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3021</v>
-      </c>
-      <c r="C2">
-        <v>64</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3022</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3023</v>
-      </c>
-      <c r="F2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" t="s">
-        <v>3024</v>
-      </c>
-      <c r="H2" t="s">
-        <v>3162</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>3025</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>3026</v>
-      </c>
-      <c r="L2" t="s">
-        <v>3023</v>
-      </c>
-      <c r="M2" t="s">
-        <v>3027</v>
-      </c>
-      <c r="N2" t="s">
-        <v>3022</v>
-      </c>
-      <c r="O2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" xr:uid="{F8A04A1C-92B7-4CCD-8C95-726A110347D5}"/>
-    <hyperlink ref="K2" r:id="rId2" xr:uid="{2F912663-1CD4-41BE-AE9B-6D2CA04D31B2}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
   <dimension ref="A1:N3"/>
@@ -19285,6 +19346,164 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="33" t="s">
+        <v>3019</v>
+      </c>
+      <c r="I1" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>3020</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3021</v>
+      </c>
+      <c r="C2">
+        <v>64</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3022</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3023</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3024</v>
+      </c>
+      <c r="H2" t="s">
+        <v>3162</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>3025</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>3026</v>
+      </c>
+      <c r="L2" t="s">
+        <v>3023</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3027</v>
+      </c>
+      <c r="N2" t="s">
+        <v>3022</v>
+      </c>
+      <c r="O2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>3248</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3249</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3250</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3251</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>3252</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>3253</v>
+      </c>
+      <c r="L3" t="s">
+        <v>3250</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3027</v>
+      </c>
+      <c r="N3" t="s">
+        <v>3250</v>
+      </c>
+      <c r="O3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{F8A04A1C-92B7-4CCD-8C95-726A110347D5}"/>
+    <hyperlink ref="K2" r:id="rId2" xr:uid="{2F912663-1CD4-41BE-AE9B-6D2CA04D31B2}"/>
+    <hyperlink ref="J3" r:id="rId3" xr:uid="{5A7F225D-EAAF-407C-A3F5-CF931A93B345}"/>
+    <hyperlink ref="K3" r:id="rId4" xr:uid="{A443CB7E-9DAC-4B30-B6D7-ABE633033E6D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -20367,9 +20586,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="5" max="5" width="16.36328125" bestFit="1" customWidth="1"/>
@@ -23102,6 +23321,47 @@
         <v>2322</v>
       </c>
       <c r="N62" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
+      <c r="A63" s="16" t="s">
+        <v>3254</v>
+      </c>
+      <c r="B63" t="s">
+        <v>3259</v>
+      </c>
+      <c r="C63" s="39" t="s">
+        <v>3258</v>
+      </c>
+      <c r="D63" s="16" t="s">
+        <v>2543</v>
+      </c>
+      <c r="E63" t="s">
+        <v>3255</v>
+      </c>
+      <c r="F63" t="s">
+        <v>3256</v>
+      </c>
+      <c r="G63" t="s">
+        <v>3257</v>
+      </c>
+      <c r="H63" t="s">
+        <v>21</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>3260</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>3261</v>
+      </c>
+      <c r="K63" s="17" t="s">
+        <v>3262</v>
+      </c>
+      <c r="L63" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="N63" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -23161,6 +23421,8 @@
     <hyperlink ref="I56" r:id="rId51" xr:uid="{CE941FB5-1D41-41B6-9CFD-C1256871C52E}"/>
     <hyperlink ref="J57" r:id="rId52" xr:uid="{72ED46D3-1227-48FD-9800-7E78EA501F81}"/>
     <hyperlink ref="I57" r:id="rId53" xr:uid="{30F29B76-2559-4C1E-A762-9F9E7C2882A4}"/>
+    <hyperlink ref="I63" r:id="rId54" xr:uid="{6A963C34-C9E4-46D1-9088-09C203C63186}"/>
+    <hyperlink ref="J63" r:id="rId55" xr:uid="{29B6CE96-A331-4903-A5B6-DD5273C7B49A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23272,7 +23534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N151"/>
+  <dimension ref="A1:N154"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -28746,8 +29008,8 @@
       <c r="C125" s="17" t="s">
         <v>1559</v>
       </c>
-      <c r="D125" s="3">
-        <v>2512</v>
+      <c r="D125" s="40" t="s">
+        <v>3231</v>
       </c>
       <c r="E125" s="17" t="s">
         <v>1560</v>
@@ -29881,7 +30143,139 @@
       </c>
     </row>
     <row r="151" spans="1:14">
-      <c r="A151" s="16"/>
+      <c r="A151" s="16" t="s">
+        <v>3228</v>
+      </c>
+      <c r="B151" s="37" t="s">
+        <v>3229</v>
+      </c>
+      <c r="C151" s="16" t="s">
+        <v>3230</v>
+      </c>
+      <c r="D151" s="38" t="s">
+        <v>3231</v>
+      </c>
+      <c r="E151" s="39" t="s">
+        <v>3232</v>
+      </c>
+      <c r="F151" s="37" t="s">
+        <v>1524</v>
+      </c>
+      <c r="G151" s="37" t="s">
+        <v>3233</v>
+      </c>
+      <c r="H151" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I151" s="27" t="s">
+        <v>3234</v>
+      </c>
+      <c r="J151" s="32" t="s">
+        <v>3235</v>
+      </c>
+      <c r="K151" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L151" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M151" s="17" t="s">
+        <v>1647</v>
+      </c>
+      <c r="N151" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="152" spans="1:14">
+      <c r="A152" s="16" t="s">
+        <v>3236</v>
+      </c>
+      <c r="B152" s="37" t="s">
+        <v>3238</v>
+      </c>
+      <c r="C152" s="16" t="s">
+        <v>3239</v>
+      </c>
+      <c r="D152" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E152" s="39" t="s">
+        <v>3240</v>
+      </c>
+      <c r="F152" s="37" t="s">
+        <v>945</v>
+      </c>
+      <c r="G152" s="37" t="s">
+        <v>3241</v>
+      </c>
+      <c r="H152" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I152" s="27" t="s">
+        <v>2928</v>
+      </c>
+      <c r="J152" t="s">
+        <v>3242</v>
+      </c>
+      <c r="K152" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="L152" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M152" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N152" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="153" spans="1:14">
+      <c r="A153" s="16" t="s">
+        <v>3237</v>
+      </c>
+      <c r="B153" s="37" t="s">
+        <v>3243</v>
+      </c>
+      <c r="C153" s="16" t="s">
+        <v>3244</v>
+      </c>
+      <c r="D153" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E153" s="39" t="s">
+        <v>3245</v>
+      </c>
+      <c r="F153" s="37" t="s">
+        <v>945</v>
+      </c>
+      <c r="G153" s="37" t="s">
+        <v>3246</v>
+      </c>
+      <c r="H153" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I153" s="27" t="s">
+        <v>2928</v>
+      </c>
+      <c r="J153" s="27" t="s">
+        <v>3247</v>
+      </c>
+      <c r="K153" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="L153" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M153" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N153" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="154" spans="1:14">
+      <c r="A154" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
@@ -29993,9 +30387,14 @@
     <hyperlink ref="J149" r:id="rId105" xr:uid="{1A42DE35-CA7D-4B83-ACC4-F85A80B83C4C}"/>
     <hyperlink ref="I150" r:id="rId106" xr:uid="{866C2F71-4468-4B2A-8F29-42D5363F2AE6}"/>
     <hyperlink ref="J150" r:id="rId107" xr:uid="{D030A4B2-39C9-4251-A1F3-D75C066D2B9B}"/>
+    <hyperlink ref="I151" r:id="rId108" xr:uid="{3CCC961A-FF6C-4434-BC16-DDC86909A33F}"/>
+    <hyperlink ref="J151" r:id="rId109" xr:uid="{C97E27C0-F3AB-4B5F-8915-58EC85F19F0D}"/>
+    <hyperlink ref="I152" r:id="rId110" xr:uid="{6971B994-F382-4D08-B0E3-89DECACB1BB6}"/>
+    <hyperlink ref="I153" r:id="rId111" xr:uid="{C3A39571-7B63-4B1B-8B0B-6C12C2D3193F}"/>
+    <hyperlink ref="J153" r:id="rId112" xr:uid="{53C0A29A-1A44-4CAA-BD58-4A236F43C0F3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId108"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId113"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
062-0001, 062-0002, 001-0107, 001-0108, 001-0109 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F13589-66E7-4F6B-A953-78148688FE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7DBB5-03D0-475B-B814-DAAE6467A581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -31,10 +31,11 @@
     <sheet name="051 - ICs - Digital" sheetId="24" r:id="rId16"/>
     <sheet name="055 - Drivers" sheetId="20" r:id="rId17"/>
     <sheet name="060 - Sensor" sheetId="3" r:id="rId18"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId19"/>
-    <sheet name="090 - Processor" sheetId="18" r:id="rId20"/>
-    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId21"/>
-    <sheet name="110 - Connectors" sheetId="13" r:id="rId22"/>
+    <sheet name="062 - Amplifiers" sheetId="25" r:id="rId19"/>
+    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId20"/>
+    <sheet name="090 - Processor" sheetId="18" r:id="rId21"/>
+    <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId22"/>
+    <sheet name="110 - Connectors" sheetId="13" r:id="rId23"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6601" uniqueCount="3289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6685" uniqueCount="3329">
   <si>
     <t>ID</t>
   </si>
@@ -9913,6 +9914,126 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/7461090?qs=sGAEpiMZZMvlX3nhDDO4AGfuriVUnyWatNc5gc2eHA0%3D</t>
+  </si>
+  <si>
+    <t>062-0001</t>
+  </si>
+  <si>
+    <t>AMC1200BDUBR</t>
+  </si>
+  <si>
+    <t>595-AMC1200BDUBR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/amc1200.pdf?ts=1781612882045&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FAMC1200%253FkeyMatch%253DAMC1200%2526tisearch%253Duniversal_search%2526usecase%253DGPN-ALT</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/AMC1200BDUBR?qs=4whTb%2F0XQMjhZwrxk0lf%2FQ%3D%3D</t>
+  </si>
+  <si>
+    <t>TLV6001UIDBVR</t>
+  </si>
+  <si>
+    <t>595-TLV6001UIDBVR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/tlv6001.pdf?ts=1781607824916&amp;ref_url=https%253A%252F%252Fcz.mouser.com%252F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/TLV6001UIDBVR?qs=8N88piwwHEgntIgM8jjJ5Q%3D%3D</t>
+  </si>
+  <si>
+    <t>SOP-8</t>
+  </si>
+  <si>
+    <t>Amplificadores de aislamiento 4kV peak Iso Amp A 5 95-AMC1200BDUB A 59 A 595-AMC1200BDUB</t>
+  </si>
+  <si>
+    <t>eUSR_SchLibrary/eUSR_SchLibrary - Amplifiers.SchLib</t>
+  </si>
+  <si>
+    <t>AMC1200B</t>
+  </si>
+  <si>
+    <t>TLV6001</t>
+  </si>
+  <si>
+    <t>SOT-23-5</t>
+  </si>
+  <si>
+    <t>062-0002</t>
+  </si>
+  <si>
+    <t>Amplificadores operacionales - Op Amps Single 5.5-V 1-MHz R RIO operational a A A 595-TLV6001UIDBVT</t>
+  </si>
+  <si>
+    <t>GRT1885C1E103FA02D</t>
+  </si>
+  <si>
+    <t>81-GRT1885C1E103FA2D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/76/2/GRT1885C1E103FA02_01A.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Murata-Electronics/GRT1885C1E103FA02D?qs=xZ%2FP%252Ba9zWqaqiXqJj78%252Bmg%3D%3D</t>
+  </si>
+  <si>
+    <t>VJ0603D471KCXAJ</t>
+  </si>
+  <si>
+    <t>Vishay</t>
+  </si>
+  <si>
+    <t>77-VJ0603D471KCXAJ</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/45258/vjhifreqseries.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Vitramon/VJ0603D471KCXAJ?qs=oomPkbqnLXekRyIlVWaYLQ%3D%3D</t>
+  </si>
+  <si>
+    <t>C0603C512F5GACTU</t>
+  </si>
+  <si>
+    <t>KEMET</t>
+  </si>
+  <si>
+    <t>80-C0603C512F5G</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/72/1/C0603C512F5GACTU.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KEMET/C0603C512F5GACTU?qs=Fn3VdHBzkcmgqbeAGPfrXg%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 0.01 uF 25 VDC 1% 0603 C0G (NP0) AEC-Q200</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) VJ0603 HIFREQ 471 0.1 non-magnetic copper non-magnetic copper 25V unmarked 7" reel</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 50V 5100pF 0603 C0G 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25V 10nF NP0</t>
+  </si>
+  <si>
+    <t>25V 470pF NP0</t>
+  </si>
+  <si>
+    <t>25V 10nF NP0</t>
+  </si>
+  <si>
+    <t>001-0107</t>
+  </si>
+  <si>
+    <t>001-0108</t>
+  </si>
+  <si>
+    <t>001-0109</t>
   </si>
 </sst>
 </file>
@@ -10091,7 +10212,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10150,10 +10271,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -10437,7 +10555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N107"/>
+  <dimension ref="A1:N110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -15159,6 +15277,138 @@
         <v>3227</v>
       </c>
       <c r="N107" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14">
+      <c r="A108" s="4" t="s">
+        <v>3326</v>
+      </c>
+      <c r="B108" t="s">
+        <v>3320</v>
+      </c>
+      <c r="C108" t="s">
+        <v>3323</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E108" t="s">
+        <v>3306</v>
+      </c>
+      <c r="F108" t="s">
+        <v>585</v>
+      </c>
+      <c r="G108" t="s">
+        <v>3307</v>
+      </c>
+      <c r="H108" t="s">
+        <v>21</v>
+      </c>
+      <c r="I108" s="2" t="s">
+        <v>3308</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>3309</v>
+      </c>
+      <c r="K108" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L108" t="s">
+        <v>61</v>
+      </c>
+      <c r="M108" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N108" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14">
+      <c r="A109" s="4" t="s">
+        <v>3327</v>
+      </c>
+      <c r="B109" t="s">
+        <v>3321</v>
+      </c>
+      <c r="C109" t="s">
+        <v>3324</v>
+      </c>
+      <c r="D109" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E109" t="s">
+        <v>3310</v>
+      </c>
+      <c r="F109" t="s">
+        <v>3311</v>
+      </c>
+      <c r="G109" t="s">
+        <v>3312</v>
+      </c>
+      <c r="H109" t="s">
+        <v>21</v>
+      </c>
+      <c r="I109" s="2" t="s">
+        <v>3313</v>
+      </c>
+      <c r="J109" s="2" t="s">
+        <v>3314</v>
+      </c>
+      <c r="K109" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L109" t="s">
+        <v>61</v>
+      </c>
+      <c r="M109" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N109" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14">
+      <c r="A110" s="4" t="s">
+        <v>3328</v>
+      </c>
+      <c r="B110" t="s">
+        <v>3322</v>
+      </c>
+      <c r="C110" t="s">
+        <v>3325</v>
+      </c>
+      <c r="D110" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E110" t="s">
+        <v>3315</v>
+      </c>
+      <c r="F110" t="s">
+        <v>3316</v>
+      </c>
+      <c r="G110" t="s">
+        <v>3317</v>
+      </c>
+      <c r="H110" t="s">
+        <v>21</v>
+      </c>
+      <c r="I110" s="2" t="s">
+        <v>3318</v>
+      </c>
+      <c r="J110" s="2" t="s">
+        <v>3319</v>
+      </c>
+      <c r="K110" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L110" t="s">
+        <v>61</v>
+      </c>
+      <c r="M110" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N110" t="s">
         <v>25</v>
       </c>
     </row>
@@ -15240,6 +15490,12 @@
     <hyperlink ref="I106" r:id="rId73" xr:uid="{BD618E63-4947-48D9-B209-8DCC58D284A8}"/>
     <hyperlink ref="J106" r:id="rId74" xr:uid="{C6D1135A-ABDE-44F6-88F2-FD4FF685F9BD}"/>
     <hyperlink ref="J107" r:id="rId75" xr:uid="{1FF336D1-9AD9-43B7-B5A0-A1ECC5C35A05}"/>
+    <hyperlink ref="I108" r:id="rId76" xr:uid="{46D4B59D-8E89-4DFA-8C9B-D3898FC3F9F3}"/>
+    <hyperlink ref="J108" r:id="rId77" xr:uid="{16223393-80B2-4745-8EA0-0A4239D2EC41}"/>
+    <hyperlink ref="I109" r:id="rId78" xr:uid="{55DEE86C-7DBE-4CD7-A07A-510E08868177}"/>
+    <hyperlink ref="J109" r:id="rId79" xr:uid="{0CE792E4-F174-4E91-B551-7288414F4023}"/>
+    <hyperlink ref="I110" r:id="rId80" xr:uid="{D7BF0419-A302-4F7D-9852-5D8A83AABBD7}"/>
+    <hyperlink ref="J110" r:id="rId81" xr:uid="{DA72DF56-54CF-4031-AB23-9AEE808CCA42}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19081,6 +19337,306 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4185B0A-D162-4EBC-935B-7159E365DD54}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>3289</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3299</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3298</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3290</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3291</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>3292</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>3293</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3301</v>
+      </c>
+      <c r="L2" t="s">
+        <v>3300</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3301</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>3304</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3305</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3303</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3294</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3295</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3296</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>3297</v>
+      </c>
+      <c r="K3" t="s">
+        <v>3302</v>
+      </c>
+      <c r="L3" t="s">
+        <v>3300</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3303</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{0AE24270-4D5D-4E12-981B-AA2533208AEE}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{339478FA-7B81-4702-B5E2-22F306F57121}"/>
+    <hyperlink ref="I3" r:id="rId3" xr:uid="{28D99F1F-302C-4204-9911-77A7F0CFE035}"/>
+    <hyperlink ref="J3" r:id="rId4" xr:uid="{BCBD2BA5-6C89-4F65-A990-3E3D7A05A9E7}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>2906</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2907</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2908</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2909</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>3205</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2910</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2911</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2912</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2913</v>
+      </c>
+      <c r="K2" t="s">
+        <v>2914</v>
+      </c>
+      <c r="L2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" t="s">
+        <v>2915</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>3201</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3203</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3204</v>
+      </c>
+      <c r="E3" s="36" t="s">
+        <v>3206</v>
+      </c>
+      <c r="F3" t="s">
+        <v>2910</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3207</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3208</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>3209</v>
+      </c>
+      <c r="K3" t="s">
+        <v>2914</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3210</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{BB2EDAB8-75EB-46D2-BA14-384BF06E1A6E}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{8F6B3EB5-F217-4353-ABA9-F461982FB5ED}"/>
+    <hyperlink ref="J3" r:id="rId3" xr:uid="{E90B210E-79B4-494B-B985-7D11C4705F7B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -19366,158 +19922,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" t="s">
-        <v>2906</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2907</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2908</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2909</v>
-      </c>
-      <c r="E2" s="36" t="s">
-        <v>3205</v>
-      </c>
-      <c r="F2" t="s">
-        <v>2910</v>
-      </c>
-      <c r="G2" t="s">
-        <v>2911</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>2912</v>
-      </c>
-      <c r="J2" t="s">
-        <v>2913</v>
-      </c>
-      <c r="K2" t="s">
-        <v>2914</v>
-      </c>
-      <c r="L2" t="s">
-        <v>61</v>
-      </c>
-      <c r="M2" t="s">
-        <v>2915</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
-        <v>3201</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3202</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3203</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3204</v>
-      </c>
-      <c r="E3" s="36" t="s">
-        <v>3206</v>
-      </c>
-      <c r="F3" t="s">
-        <v>2910</v>
-      </c>
-      <c r="G3" t="s">
-        <v>3207</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>3208</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>3209</v>
-      </c>
-      <c r="K3" t="s">
-        <v>2914</v>
-      </c>
-      <c r="L3" t="s">
-        <v>61</v>
-      </c>
-      <c r="M3" t="s">
-        <v>3210</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="16" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{BB2EDAB8-75EB-46D2-BA14-384BF06E1A6E}"/>
-    <hyperlink ref="I3" r:id="rId2" xr:uid="{8F6B3EB5-F217-4353-ABA9-F461982FB5ED}"/>
-    <hyperlink ref="J3" r:id="rId3" xr:uid="{E90B210E-79B4-494B-B985-7D11C4705F7B}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
   <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -19675,7 +20080,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -20758,7 +21163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
   <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
@@ -23547,19 +23952,19 @@
       <c r="B64" t="s">
         <v>3283</v>
       </c>
-      <c r="C64" s="39" t="s">
+      <c r="C64" s="16" t="s">
         <v>2488</v>
       </c>
       <c r="D64" s="16" t="s">
         <v>3284</v>
       </c>
-      <c r="E64" s="40" t="s">
+      <c r="E64" s="20" t="s">
         <v>3285</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>2100</v>
       </c>
-      <c r="G64" s="38" t="s">
+      <c r="G64" s="3" t="s">
         <v>3286</v>
       </c>
       <c r="H64" t="s">
@@ -23571,7 +23976,7 @@
       <c r="J64" s="2" t="s">
         <v>3288</v>
       </c>
-      <c r="K64" s="41" t="s">
+      <c r="K64" s="17" t="s">
         <v>2429</v>
       </c>
       <c r="L64" s="7" t="s">

</xml_diff>

<commit_message>
010-0153, 010-0154, 010-0155 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7DBB5-03D0-475B-B814-DAAE6467A581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580C0203-3800-43DF-8E8C-CB21C43739CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6685" uniqueCount="3329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6727" uniqueCount="3352">
   <si>
     <t>ID</t>
   </si>
@@ -10034,6 +10034,75 @@
   </si>
   <si>
     <t>001-0109</t>
+  </si>
+  <si>
+    <t>010-0153</t>
+  </si>
+  <si>
+    <t>010-0154</t>
+  </si>
+  <si>
+    <t>010-0155</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors MCU 0805-15 0.1% P1 1K65</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 3.3Kohm 0.1% 15ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>RES SMD 12 OHM 0.25% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>1.65kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>3.3kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>12Ω 250mW  0.25%</t>
+  </si>
+  <si>
+    <t>MCU08050E1651BP100</t>
+  </si>
+  <si>
+    <t>594-MCU08050E1651BP1</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/28700/mcx0x0xpre.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Beyschlag/MCU08050E1651BP100?qs=sGAEpiMZZMvdGkrng054t2c0lhweLxbk6HRvs42FTBI%3D</t>
+  </si>
+  <si>
+    <t>ERA-6APB332V</t>
+  </si>
+  <si>
+    <t>Panasonic</t>
+  </si>
+  <si>
+    <t>667-ERA-6APB332V</t>
+  </si>
+  <si>
+    <t>https://industrial.panasonic.com/cdbs/www-data/pdf/RDM0000/AOA0000C307.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6APB332V?qs=sGAEpiMZZMvdGkrng054t7Q%2FBjLwFmgicQi9zKDLbrs%3D</t>
+  </si>
+  <si>
+    <t>RT1206CRC0712RL</t>
+  </si>
+  <si>
+    <t>RT1206CRC0712RL-ND</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>https://www.digikey.es/es/models/5937613?tab=null</t>
+  </si>
+  <si>
+    <t>https://www.digikey.es/es/products/detail/yageo/RT1206CRC0712RL/5937613</t>
   </si>
 </sst>
 </file>
@@ -10212,7 +10281,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10271,7 +10340,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -15334,7 +15402,7 @@
       <c r="C109" t="s">
         <v>3324</v>
       </c>
-      <c r="D109" s="38" t="s">
+      <c r="D109" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E109" t="s">
@@ -15378,7 +15446,7 @@
       <c r="C110" t="s">
         <v>3325</v>
       </c>
-      <c r="D110" s="38" t="s">
+      <c r="D110" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E110" t="s">
@@ -24165,7 +24233,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N154"/>
+  <dimension ref="A1:N159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -30906,7 +30974,139 @@
       </c>
     </row>
     <row r="154" spans="1:14">
-      <c r="A154" s="16"/>
+      <c r="A154" s="16" t="s">
+        <v>3329</v>
+      </c>
+      <c r="B154" t="s">
+        <v>3332</v>
+      </c>
+      <c r="C154" t="s">
+        <v>3335</v>
+      </c>
+      <c r="D154" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E154" t="s">
+        <v>3338</v>
+      </c>
+      <c r="F154" t="s">
+        <v>3311</v>
+      </c>
+      <c r="G154" t="s">
+        <v>3339</v>
+      </c>
+      <c r="H154" t="s">
+        <v>21</v>
+      </c>
+      <c r="I154" s="2" t="s">
+        <v>3340</v>
+      </c>
+      <c r="J154" s="2" t="s">
+        <v>3341</v>
+      </c>
+      <c r="K154" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L154" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M154" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N154" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14">
+      <c r="A155" s="16" t="s">
+        <v>3330</v>
+      </c>
+      <c r="B155" t="s">
+        <v>3333</v>
+      </c>
+      <c r="C155" t="s">
+        <v>3336</v>
+      </c>
+      <c r="D155" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E155" t="s">
+        <v>3342</v>
+      </c>
+      <c r="F155" t="s">
+        <v>3343</v>
+      </c>
+      <c r="G155" t="s">
+        <v>3344</v>
+      </c>
+      <c r="H155" t="s">
+        <v>21</v>
+      </c>
+      <c r="I155" s="2" t="s">
+        <v>3345</v>
+      </c>
+      <c r="J155" s="2" t="s">
+        <v>3346</v>
+      </c>
+      <c r="K155" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L155" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M155" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N155" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="156" spans="1:14">
+      <c r="A156" s="16" t="s">
+        <v>3331</v>
+      </c>
+      <c r="B156" t="s">
+        <v>3334</v>
+      </c>
+      <c r="C156" t="s">
+        <v>3337</v>
+      </c>
+      <c r="D156" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="E156" t="s">
+        <v>3347</v>
+      </c>
+      <c r="F156" t="s">
+        <v>60</v>
+      </c>
+      <c r="G156" t="s">
+        <v>3348</v>
+      </c>
+      <c r="H156" t="s">
+        <v>3349</v>
+      </c>
+      <c r="I156" t="s">
+        <v>3350</v>
+      </c>
+      <c r="J156" s="2" t="s">
+        <v>3351</v>
+      </c>
+      <c r="K156" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L156" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M156" s="7" t="s">
+        <v>1645</v>
+      </c>
+      <c r="N156" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14">
+      <c r="F159" s="21"/>
     </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
@@ -31023,9 +31223,14 @@
     <hyperlink ref="I152" r:id="rId110" xr:uid="{6971B994-F382-4D08-B0E3-89DECACB1BB6}"/>
     <hyperlink ref="I153" r:id="rId111" xr:uid="{C3A39571-7B63-4B1B-8B0B-6C12C2D3193F}"/>
     <hyperlink ref="J153" r:id="rId112" xr:uid="{53C0A29A-1A44-4CAA-BD58-4A236F43C0F3}"/>
+    <hyperlink ref="I154" r:id="rId113" xr:uid="{EC84B0AF-9E78-4228-A4D8-C52EEB67EF3E}"/>
+    <hyperlink ref="J154" r:id="rId114" xr:uid="{293A3F3E-9607-4CA6-999A-FBB3D073E270}"/>
+    <hyperlink ref="I155" r:id="rId115" xr:uid="{819E07D4-A0E4-475C-ACC0-622501017E74}"/>
+    <hyperlink ref="J155" r:id="rId116" xr:uid="{9D7A02D8-02AB-40F9-A4C3-999EDC72ED54}"/>
+    <hyperlink ref="J156" r:id="rId117" xr:uid="{C7F72D9E-B22F-4AFF-9CFB-3A851699B586}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId113"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId118"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
001-0110, 001-0111, 001-0112, 001-0113, 010-0156, 010-0157, 010-0158, 010-0159, 020-0001, 020-0002, 070-0006, 070-0007, 070-0008 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{400EDE90-C96D-4FA7-A343-F0BE4401D0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5FD5C94-E2A0-464E-ABDF-65CDE4E48212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
     <sheet name="055 - Drivers" sheetId="20" r:id="rId17"/>
     <sheet name="060 - Sensor" sheetId="3" r:id="rId18"/>
     <sheet name="062 - Amplifiers" sheetId="25" r:id="rId19"/>
-    <sheet name="070 - Power Supply - DCDC" sheetId="8" r:id="rId20"/>
+    <sheet name="070 - Power Supply" sheetId="8" r:id="rId20"/>
     <sheet name="090 - Processor" sheetId="18" r:id="rId21"/>
     <sheet name="100 - Electromechanicals" sheetId="15" r:id="rId22"/>
     <sheet name="110 - Connectors" sheetId="13" r:id="rId23"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6727" uniqueCount="3352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6909" uniqueCount="3448">
   <si>
     <t>ID</t>
   </si>
@@ -10103,6 +10103,294 @@
   </si>
   <si>
     <t>50V 5.1nF NP0</t>
+  </si>
+  <si>
+    <t>885012206052</t>
+  </si>
+  <si>
+    <t>710-885012206052</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012206052.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012206052?qs=0KOYDY2FL2%2F2JKabApojcQ%3D%3D</t>
+  </si>
+  <si>
+    <t>885012107014</t>
+  </si>
+  <si>
+    <t>710-885012107014</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012107014.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012107014?qs=0KOYDY2FL28i0pwNdARIlg%3D%3D</t>
+  </si>
+  <si>
+    <t>885012206046</t>
+  </si>
+  <si>
+    <t>710-885012206046</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012206046.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012206046?qs=0KOYDY2FL2%252B89gr6HvTBXA%3D%3D</t>
+  </si>
+  <si>
+    <t>885012106029</t>
+  </si>
+  <si>
+    <t>710-885012106029</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012106029.pdf</t>
+  </si>
+  <si>
+    <t>001-0110</t>
+  </si>
+  <si>
+    <t>001-0111</t>
+  </si>
+  <si>
+    <t>001-0112</t>
+  </si>
+  <si>
+    <t>001-0113</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 1uF 0603 10% 16V MLCC</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 10uF 0805 20% 16V MLCC</t>
+  </si>
+  <si>
+    <t>16V 10uF X5R</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 0.1uF 0603 10% 16V MLCC</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012106029?qs=amGC7iS6iy%252BgG3I4L92Nqg%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 2.2uF 16V 10%</t>
+  </si>
+  <si>
+    <t>560112110142</t>
+  </si>
+  <si>
+    <t>710-560112110142</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112110142.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112110142?qs=mELouGlnn3daEwPMtfpdeg%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 118 kOhms 1 % 0.1 W 0402 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112110099</t>
+  </si>
+  <si>
+    <t>710-560112110099</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112110099.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112110099?qs=mELouGlnn3eF8MLEVMJrCw%3D%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 22.1 kOhms 1 % 0.1 W 0402 AEC-Q200</t>
+  </si>
+  <si>
+    <t>CRCW040269K8FKED</t>
+  </si>
+  <si>
+    <t>71-CRCW0402-69.8K-E3</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay/CRCW040269K8FKED?qs=sGAEpiMZZMtlubZbdhIBICni6BQV4SfY1e7wNtp2Znw%3D</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 1/10 Watt 69.8Kohms 1%</t>
+  </si>
+  <si>
+    <t>118kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>010-0156</t>
+  </si>
+  <si>
+    <t>010-0157</t>
+  </si>
+  <si>
+    <t>010-0158</t>
+  </si>
+  <si>
+    <t>22.1kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>69.8kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>74438336100</t>
+  </si>
+  <si>
+    <t>710-74438336100</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/74438336100.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/74438336100?qs=iC14BvcgY%2F3tj5fn6qP7Hg%3D%3D</t>
+  </si>
+  <si>
+    <t>74438357082</t>
+  </si>
+  <si>
+    <t>710-74438357082</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/74438357082.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/74438357082?qs=AQlKX63v8RvaY%2FvJVfZzHA%3D%3D</t>
+  </si>
+  <si>
+    <t>IND</t>
+  </si>
+  <si>
+    <t>Inductores de potencia (SMD) WE-MAPI 10uH 1.2A DCR=322mOhms AEC-Q200</t>
+  </si>
+  <si>
+    <t>10uH 1.65A 322mOhm</t>
+  </si>
+  <si>
+    <t>SMD;3x3mm</t>
+  </si>
+  <si>
+    <t>IND SMD 3x3</t>
+  </si>
+  <si>
+    <t>020-0001</t>
+  </si>
+  <si>
+    <t>020-0002</t>
+  </si>
+  <si>
+    <t>8.2uH 2.8A 86mOhm</t>
+  </si>
+  <si>
+    <t>SMD;4.1x4.1mm</t>
+  </si>
+  <si>
+    <t>IND SMD 4.1x4.1</t>
+  </si>
+  <si>
+    <t>Inductores de potencia (SMD) WE-MAPI 8.2uH 2.8A DCR=86mOhms AEC-Q200</t>
+  </si>
+  <si>
+    <t>070-0006</t>
+  </si>
+  <si>
+    <t>070-0007</t>
+  </si>
+  <si>
+    <t>070-0008</t>
+  </si>
+  <si>
+    <t>TLV705165YFPR</t>
+  </si>
+  <si>
+    <t>595-TLV705165YFPR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/tlv705.pdf?ts=1781649192737&amp;ref_url=https%253A%252F%252Fwww.ti.com</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/TLV705165YFPR?qs=rrS6PyfT74d8bhzeUZaAoA%3D%3D</t>
+  </si>
+  <si>
+    <t>LMR51410YFDBVR</t>
+  </si>
+  <si>
+    <t>595-LMR51410YFDBVR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/lmr51410.pdf?ts=1781684561920&amp;ref_url=https%253A%252F%252Fwww.mouser.de%252F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/LMR51410YFDBVR?qs=i8QVZAFTkqTUiBodeYrDsw%3D%3D</t>
+  </si>
+  <si>
+    <t>LM2776DBVT</t>
+  </si>
+  <si>
+    <t>595-LM2776DBVT</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/lm2776.pdf?ts=1781716279536&amp;ref_url=https%253A%252F%252Fwww.mouser.es%252F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/LM2776DBVT?qs=GJ%2F2ZGcr5uMLAYYW9ugYkg%3D%3D</t>
+  </si>
+  <si>
+    <t>(4/42)V-(0.8/28)V</t>
+  </si>
+  <si>
+    <t>Reguladores de tensión de conmutación SIMPLE SWITCHER 4V t o 42V 1A synchronou</t>
+  </si>
+  <si>
+    <t>Reguladores de voltaje LDO 200-mA high-PSRR l o w-IQ low-dropout v A 595-TLV705165YFPT</t>
+  </si>
+  <si>
+    <t>(2/5.5)V-1.65V</t>
+  </si>
+  <si>
+    <t>DSBGA-4</t>
+  </si>
+  <si>
+    <t>TLV705165</t>
+  </si>
+  <si>
+    <t>LMR51410</t>
+  </si>
+  <si>
+    <t>(2.7/5.5)V-(-2.7/-5.5)V</t>
+  </si>
+  <si>
+    <t>Reguladores de tensión de conmutación Switched Capacitor I nverter A 595-LM277 A 595-LM2776DBVR</t>
+  </si>
+  <si>
+    <t>LM2776</t>
+  </si>
+  <si>
+    <t>010-0159</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 100 kOhms 1 % 0.1 W 0402 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112110019</t>
+  </si>
+  <si>
+    <t>710-560112110019</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112110019.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112110019?qs=mELouGlnn3eOtqJeFyZVpA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -10623,7 +10911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N110"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -15477,6 +15765,182 @@
         <v>62</v>
       </c>
       <c r="N110" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14">
+      <c r="A111" s="4" t="s">
+        <v>3367</v>
+      </c>
+      <c r="B111" t="s">
+        <v>3371</v>
+      </c>
+      <c r="C111" t="s">
+        <v>2988</v>
+      </c>
+      <c r="D111" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E111" s="36" t="s">
+        <v>3352</v>
+      </c>
+      <c r="F111" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G111" t="s">
+        <v>3353</v>
+      </c>
+      <c r="H111" t="s">
+        <v>21</v>
+      </c>
+      <c r="I111" s="2" t="s">
+        <v>3354</v>
+      </c>
+      <c r="J111" s="2" t="s">
+        <v>3355</v>
+      </c>
+      <c r="K111" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L111" t="s">
+        <v>61</v>
+      </c>
+      <c r="M111" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N111" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14">
+      <c r="A112" s="4" t="s">
+        <v>3368</v>
+      </c>
+      <c r="B112" t="s">
+        <v>3372</v>
+      </c>
+      <c r="C112" t="s">
+        <v>3373</v>
+      </c>
+      <c r="D112" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E112" s="36" t="s">
+        <v>3356</v>
+      </c>
+      <c r="F112" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G112" t="s">
+        <v>3357</v>
+      </c>
+      <c r="H112" t="s">
+        <v>21</v>
+      </c>
+      <c r="I112" s="2" t="s">
+        <v>3358</v>
+      </c>
+      <c r="J112" s="2" t="s">
+        <v>3359</v>
+      </c>
+      <c r="K112" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L112" t="s">
+        <v>61</v>
+      </c>
+      <c r="M112" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="N112" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14">
+      <c r="A113" s="4" t="s">
+        <v>3369</v>
+      </c>
+      <c r="B113" t="s">
+        <v>3374</v>
+      </c>
+      <c r="C113" t="s">
+        <v>2982</v>
+      </c>
+      <c r="D113" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E113" s="36" t="s">
+        <v>3360</v>
+      </c>
+      <c r="F113" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G113" t="s">
+        <v>3361</v>
+      </c>
+      <c r="H113" t="s">
+        <v>21</v>
+      </c>
+      <c r="I113" s="2" t="s">
+        <v>3362</v>
+      </c>
+      <c r="J113" s="2" t="s">
+        <v>3363</v>
+      </c>
+      <c r="K113" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L113" t="s">
+        <v>61</v>
+      </c>
+      <c r="M113" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N113" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14">
+      <c r="A114" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="B114" t="s">
+        <v>3376</v>
+      </c>
+      <c r="C114" t="s">
+        <v>155</v>
+      </c>
+      <c r="D114" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E114" s="36" t="s">
+        <v>3364</v>
+      </c>
+      <c r="F114" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G114" t="s">
+        <v>3365</v>
+      </c>
+      <c r="H114" t="s">
+        <v>21</v>
+      </c>
+      <c r="I114" s="2" t="s">
+        <v>3366</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>3375</v>
+      </c>
+      <c r="K114" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L114" t="s">
+        <v>61</v>
+      </c>
+      <c r="M114" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N114" t="s">
         <v>25</v>
       </c>
     </row>
@@ -15564,8 +16028,17 @@
     <hyperlink ref="J109" r:id="rId79" xr:uid="{0CE792E4-F174-4E91-B551-7288414F4023}"/>
     <hyperlink ref="I110" r:id="rId80" xr:uid="{D7BF0419-A302-4F7D-9852-5D8A83AABBD7}"/>
     <hyperlink ref="J110" r:id="rId81" xr:uid="{DA72DF56-54CF-4031-AB23-9AEE808CCA42}"/>
+    <hyperlink ref="I111" r:id="rId82" xr:uid="{AD5C5368-A948-45EC-8368-303EF16B76C4}"/>
+    <hyperlink ref="J111" r:id="rId83" xr:uid="{12677E4F-CC0C-474A-AF70-3FA3FD23CCC8}"/>
+    <hyperlink ref="I112" r:id="rId84" xr:uid="{6738B4F6-C20E-4F28-A5E0-DA4B845CD87C}"/>
+    <hyperlink ref="J112" r:id="rId85" xr:uid="{203E6C20-5030-4C57-A692-AE145EF9A648}"/>
+    <hyperlink ref="I113" r:id="rId86" xr:uid="{6BF8DD46-F79B-4225-A5CE-0178FA8E1FD1}"/>
+    <hyperlink ref="J113" r:id="rId87" xr:uid="{888ED7A4-81F2-44BF-ACB2-1634B14D367A}"/>
+    <hyperlink ref="I114" r:id="rId88" xr:uid="{4DE3B0C7-2537-4971-98DE-9A56EF44C421}"/>
+    <hyperlink ref="J114" r:id="rId89" xr:uid="{FB1B8B94-45EA-4535-BE3A-72D28A8B6781}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId90"/>
 </worksheet>
 </file>
 
@@ -19706,7 +20179,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="17.54296875" customWidth="1"/>
@@ -19976,6 +20449,138 @@
         <v>25</v>
       </c>
     </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>3417</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3434</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3435</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3436</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3420</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
+        <v>3421</v>
+      </c>
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>3422</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>3423</v>
+      </c>
+      <c r="K7" t="s">
+        <v>3437</v>
+      </c>
+      <c r="L7" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M7" t="s">
+        <v>3436</v>
+      </c>
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>3418</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3433</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3432</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2120</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3424</v>
+      </c>
+      <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>3427</v>
+      </c>
+      <c r="K8" t="s">
+        <v>3438</v>
+      </c>
+      <c r="L8" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M8" t="s">
+        <v>2120</v>
+      </c>
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>3419</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3440</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3439</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2120</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3428</v>
+      </c>
+      <c r="F9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" t="s">
+        <v>3429</v>
+      </c>
+      <c r="H9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" t="s">
+        <v>3430</v>
+      </c>
+      <c r="J9" t="s">
+        <v>3431</v>
+      </c>
+      <c r="K9" t="s">
+        <v>3441</v>
+      </c>
+      <c r="L9" t="s">
+        <v>1689</v>
+      </c>
+      <c r="M9" t="s">
+        <v>2120</v>
+      </c>
+      <c r="N9" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
@@ -19984,9 +20589,13 @@
     <hyperlink ref="I5" r:id="rId3" xr:uid="{38CEA448-03C1-4130-9D22-378144C1B83E}"/>
     <hyperlink ref="J5" r:id="rId4" xr:uid="{178AE8D2-EC1F-4144-807A-F49730BDAEE7}"/>
     <hyperlink ref="I6" r:id="rId5" xr:uid="{C6B22468-8A2D-4CA0-8E30-C5E1C054C475}"/>
+    <hyperlink ref="I7" r:id="rId6" xr:uid="{46E13713-695D-493D-96DD-70A916E207CE}"/>
+    <hyperlink ref="J7" r:id="rId7" xr:uid="{CE7C033B-E1D3-4982-B98D-45472DE55249}"/>
+    <hyperlink ref="J8" r:id="rId8" xr:uid="{EA27946F-BAF3-48A3-B1E1-735BC730E575}"/>
+    <hyperlink ref="I8" r:id="rId9" xr:uid="{E0BD2FA6-2C87-41A3-AA17-DD7C10DA47E6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -24233,7 +24842,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N159"/>
+  <dimension ref="A1:N160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -31105,8 +31714,181 @@
         <v>25</v>
       </c>
     </row>
+    <row r="157" spans="1:14">
+      <c r="A157" s="16" t="s">
+        <v>3393</v>
+      </c>
+      <c r="B157" t="s">
+        <v>3381</v>
+      </c>
+      <c r="C157" s="16" t="s">
+        <v>3392</v>
+      </c>
+      <c r="D157" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E157" s="36" t="s">
+        <v>3377</v>
+      </c>
+      <c r="F157" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G157" t="s">
+        <v>3378</v>
+      </c>
+      <c r="H157" t="s">
+        <v>21</v>
+      </c>
+      <c r="I157" s="2" t="s">
+        <v>3379</v>
+      </c>
+      <c r="J157" t="s">
+        <v>3380</v>
+      </c>
+      <c r="K157" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L157" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M157" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N157" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14">
+      <c r="A158" s="16" t="s">
+        <v>3394</v>
+      </c>
+      <c r="B158" t="s">
+        <v>3386</v>
+      </c>
+      <c r="C158" s="16" t="s">
+        <v>3396</v>
+      </c>
+      <c r="D158" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E158" s="36" t="s">
+        <v>3382</v>
+      </c>
+      <c r="F158" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G158" t="s">
+        <v>3383</v>
+      </c>
+      <c r="H158" t="s">
+        <v>21</v>
+      </c>
+      <c r="I158" s="2" t="s">
+        <v>3384</v>
+      </c>
+      <c r="J158" t="s">
+        <v>3385</v>
+      </c>
+      <c r="K158" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L158" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M158" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N158" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="159" spans="1:14">
-      <c r="F159" s="21"/>
+      <c r="A159" s="16" t="s">
+        <v>3395</v>
+      </c>
+      <c r="B159" t="s">
+        <v>3391</v>
+      </c>
+      <c r="C159" s="16" t="s">
+        <v>3397</v>
+      </c>
+      <c r="D159" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E159" t="s">
+        <v>3387</v>
+      </c>
+      <c r="F159" t="s">
+        <v>3311</v>
+      </c>
+      <c r="G159" t="s">
+        <v>3388</v>
+      </c>
+      <c r="H159" t="s">
+        <v>21</v>
+      </c>
+      <c r="I159" s="2" t="s">
+        <v>3389</v>
+      </c>
+      <c r="J159" s="2" t="s">
+        <v>3390</v>
+      </c>
+      <c r="K159" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L159" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M159" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N159" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14">
+      <c r="A160" s="16" t="s">
+        <v>3442</v>
+      </c>
+      <c r="B160" t="s">
+        <v>3443</v>
+      </c>
+      <c r="C160" s="16" t="s">
+        <v>929</v>
+      </c>
+      <c r="D160" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E160" s="20" t="s">
+        <v>3444</v>
+      </c>
+      <c r="F160" s="16" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G160" s="16" t="s">
+        <v>3445</v>
+      </c>
+      <c r="H160" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I160" s="27" t="s">
+        <v>3446</v>
+      </c>
+      <c r="J160" t="s">
+        <v>3447</v>
+      </c>
+      <c r="K160" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L160" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M160" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N160" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
@@ -31228,9 +32010,13 @@
     <hyperlink ref="I155" r:id="rId115" xr:uid="{819E07D4-A0E4-475C-ACC0-622501017E74}"/>
     <hyperlink ref="J155" r:id="rId116" xr:uid="{9D7A02D8-02AB-40F9-A4C3-999EDC72ED54}"/>
     <hyperlink ref="J156" r:id="rId117" xr:uid="{C7F72D9E-B22F-4AFF-9CFB-3A851699B586}"/>
+    <hyperlink ref="I158" r:id="rId118" xr:uid="{A3CABA41-1EF9-4C9F-AE07-C02EA7FCF75E}"/>
+    <hyperlink ref="I159" r:id="rId119" xr:uid="{D5889C02-ED09-4327-9DFB-0BBF24BA4AA7}"/>
+    <hyperlink ref="J159" r:id="rId120" xr:uid="{5E88809D-3319-44CA-AC1F-18CC618C3A0A}"/>
+    <hyperlink ref="I160" r:id="rId121" xr:uid="{38247BF1-5599-4165-BFEC-26629D789AC3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId118"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId122"/>
 </worksheet>
 </file>
 
@@ -31478,7 +32264,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C6B0FD-D8A3-44EC-9532-03DDA232F922}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -31525,8 +32311,103 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>3411</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3407</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3408</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3409</v>
+      </c>
+      <c r="E2" s="36" t="s">
+        <v>3398</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3399</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>3400</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>3401</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3406</v>
+      </c>
+      <c r="L2" t="s">
+        <v>2904</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>3410</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>3412</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3416</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3413</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3414</v>
+      </c>
+      <c r="E3" s="36" t="s">
+        <v>3402</v>
+      </c>
+      <c r="F3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3403</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3404</v>
+      </c>
+      <c r="J3" t="s">
+        <v>3405</v>
+      </c>
+      <c r="K3" t="s">
+        <v>3406</v>
+      </c>
+      <c r="L3" t="s">
+        <v>2904</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>3415</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{07883802-B058-47F9-BBB3-C06E82952829}"/>
+    <hyperlink ref="J2" r:id="rId2" xr:uid="{62DD0F89-540D-4537-B7A5-4B172FA10C23}"/>
+    <hyperlink ref="I3" r:id="rId3" xr:uid="{A45B5B86-5ADB-44B4-BF96-CFB1161AF6C6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
001-0114, 001-0115, 001-0116 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C5A904-14E0-40B9-B0A1-5757D9C583FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE01584E-F2A1-4EBB-B809-BEEF27A38C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6922" uniqueCount="3450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6950" uniqueCount="3463">
   <si>
     <t>ID</t>
   </si>
@@ -10397,6 +10397,45 @@
   </si>
   <si>
     <t>0Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>ZRB18AR61E106KE01L</t>
+  </si>
+  <si>
+    <t>81-ZRB18AR61E106KE1L</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Murata-Electronics/ZRB18AR61E106KE01L?qs=sGAEpiMZZMsh%252B1woXyUXj%2Fze%252BJJ8bUKCZuLWV6qOmdQ%3D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/76/2/ZRB18AR61E106KE01_02A.pdf</t>
+  </si>
+  <si>
+    <t>885012206071</t>
+  </si>
+  <si>
+    <t>710-885012206071</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/885012206071.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/885012206071?qs=0KOYDY2FL2%2FEBQkuHgvarg%3D%3D</t>
+  </si>
+  <si>
+    <t>25V 0.1uF X7R</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 0603 25VDC 10uF 10% X5R</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 0.1uF 0603 10% 25V MLCC</t>
+  </si>
+  <si>
+    <t>001-0114</t>
+  </si>
+  <si>
+    <t>001-0115</t>
   </si>
 </sst>
 </file>
@@ -10575,7 +10614,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10634,8 +10673,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -10919,7 +10956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N114"/>
+  <dimension ref="A1:N116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -15949,6 +15986,94 @@
         <v>62</v>
       </c>
       <c r="N114" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
+      <c r="A115" s="4" t="s">
+        <v>3461</v>
+      </c>
+      <c r="B115" t="s">
+        <v>3459</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="D115" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>3450</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>3451</v>
+      </c>
+      <c r="H115" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I115" s="2" t="s">
+        <v>3452</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>3453</v>
+      </c>
+      <c r="K115" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="L115" t="s">
+        <v>61</v>
+      </c>
+      <c r="M115" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N115" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
+      <c r="A116" s="4" t="s">
+        <v>3462</v>
+      </c>
+      <c r="B116" t="s">
+        <v>3460</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>3458</v>
+      </c>
+      <c r="D116" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E116" s="36" t="s">
+        <v>3454</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G116" t="s">
+        <v>3455</v>
+      </c>
+      <c r="H116" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I116" s="2" t="s">
+        <v>3456</v>
+      </c>
+      <c r="J116" s="2" t="s">
+        <v>3457</v>
+      </c>
+      <c r="K116" s="3" t="s">
+        <v>3458</v>
+      </c>
+      <c r="L116" t="s">
+        <v>61</v>
+      </c>
+      <c r="M116" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N116" t="s">
         <v>25</v>
       </c>
     </row>
@@ -16044,9 +16169,11 @@
     <hyperlink ref="J113" r:id="rId87" xr:uid="{888ED7A4-81F2-44BF-ACB2-1634B14D367A}"/>
     <hyperlink ref="I114" r:id="rId88" xr:uid="{4DE3B0C7-2537-4971-98DE-9A56EF44C421}"/>
     <hyperlink ref="J114" r:id="rId89" xr:uid="{FB1B8B94-45EA-4535-BE3A-72D28A8B6781}"/>
+    <hyperlink ref="J115" r:id="rId90" xr:uid="{88671F05-A2EE-487E-BF71-2F48DB15577D}"/>
+    <hyperlink ref="I115" r:id="rId91" xr:uid="{42FBB82F-FA0A-49B4-BEC5-E4E89D6CB366}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId90"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId92"/>
 </worksheet>
 </file>
 
@@ -31908,7 +32035,7 @@
       <c r="C161" s="16" t="s">
         <v>3449</v>
       </c>
-      <c r="D161" s="38" t="s">
+      <c r="D161" s="20" t="s">
         <v>59</v>
       </c>
       <c r="E161">
@@ -31917,10 +32044,10 @@
       <c r="F161" s="16" t="s">
         <v>2100</v>
       </c>
-      <c r="G161" s="39" t="s">
+      <c r="G161" s="16" t="s">
         <v>3107</v>
       </c>
-      <c r="H161" s="39" t="s">
+      <c r="H161" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I161" s="27" t="s">

</xml_diff>

<commit_message>
023-0002, 004-0002, 001-0117, 001-0118 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE23959-6875-40F2-AEF9-9D4DBB8E573D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7643704E-0F7D-4704-8899-B926297121C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46695" yWindow="2355" windowWidth="14610" windowHeight="15585" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6964" uniqueCount="3470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7020" uniqueCount="3502">
   <si>
     <t>ID</t>
   </si>
@@ -10457,6 +10457,102 @@
   </si>
   <si>
     <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) WCAP-CSGP 100pF 0402 5% 16V MLCC</t>
+  </si>
+  <si>
+    <t>1812VC105KAT2A</t>
+  </si>
+  <si>
+    <t>581-1812VC105KAT2A</t>
+  </si>
+  <si>
+    <t>https://datasheets.kyocera-avx.com/AVX-HV_MLCC.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/1812VC105KAT2A?qs=sGAEpiMZZMvsSlwiRhF8qtsBU8Zhqm2RiX3yQof58UA8TRVHqLE0IA%3D%3D</t>
+  </si>
+  <si>
+    <t>C4532X7T2E684M160KA</t>
+  </si>
+  <si>
+    <t>810-C4532X7T2E684M6K</t>
+  </si>
+  <si>
+    <t>https://product.tdk.com/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_commercial_highvoltage_en.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TDK/C4532X7T2E684M160KA?qs=sGAEpiMZZMvsSlwiRhF8qtKev7nvVKumgcECMxBqJildLuXsoVBqzA%3D%3D</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 250V 1uF X7R 1812 10 %</t>
+  </si>
+  <si>
+    <t>250V 1uF X7R</t>
+  </si>
+  <si>
+    <t>250V 680nF X7T</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 1812 250V 0.68uF X7T 20% T: 1.6mm</t>
+  </si>
+  <si>
+    <t>001-0117</t>
+  </si>
+  <si>
+    <t>001-0118</t>
+  </si>
+  <si>
+    <t>004-0002</t>
+  </si>
+  <si>
+    <t>Condensadores de seguridad 500volts 680pF 20% LS=15mm</t>
+  </si>
+  <si>
+    <t>1.5kV 680pF Y1</t>
+  </si>
+  <si>
+    <t>THT;W5.5xL18mm</t>
+  </si>
+  <si>
+    <t>P295BE681M500A</t>
+  </si>
+  <si>
+    <t>80-P295BE681M500A</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/72/1/KEM_F3088_P295_Y1_500.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KEMET/P295BE681M500A?qs=zoGAYOF739DgwL35ue4hHg%3D%3D</t>
+  </si>
+  <si>
+    <t>CAP_15Px12.5H</t>
+  </si>
+  <si>
+    <t>023-0002</t>
+  </si>
+  <si>
+    <t>Cebadores / filtros de modo común Filter Component</t>
+  </si>
+  <si>
+    <t>325uH 3.3A 35 %</t>
+  </si>
+  <si>
+    <t>11x11x8.8</t>
+  </si>
+  <si>
+    <t>TCK-050</t>
+  </si>
+  <si>
+    <t>495-TCK-050</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/1230/1/tck_050_datasheet.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TRACO-Power/TCK-050?qs=ckJk83FOD0VjpXDswRrv6g%3D%3D</t>
+  </si>
+  <si>
+    <t>IND_CMM_THT_11x11mm</t>
   </si>
 </sst>
 </file>
@@ -10635,7 +10731,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10694,6 +10790,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -10977,7 +11075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N117"/>
+  <dimension ref="A1:N119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -16139,6 +16237,94 @@
         <v>698</v>
       </c>
       <c r="N117" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14">
+      <c r="A118" s="4" t="s">
+        <v>3482</v>
+      </c>
+      <c r="B118" t="s">
+        <v>3478</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>3479</v>
+      </c>
+      <c r="D118" s="13" t="s">
+        <v>3222</v>
+      </c>
+      <c r="E118" t="s">
+        <v>3470</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>3471</v>
+      </c>
+      <c r="H118" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I118" s="27" t="s">
+        <v>3472</v>
+      </c>
+      <c r="J118" s="32" t="s">
+        <v>3473</v>
+      </c>
+      <c r="K118" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L118" t="s">
+        <v>61</v>
+      </c>
+      <c r="M118" s="7" t="s">
+        <v>3227</v>
+      </c>
+      <c r="N118" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14">
+      <c r="A119" s="4" t="s">
+        <v>3483</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>3481</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>3480</v>
+      </c>
+      <c r="D119" s="13" t="s">
+        <v>3222</v>
+      </c>
+      <c r="E119" t="s">
+        <v>3474</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="G119" s="3" t="s">
+        <v>3475</v>
+      </c>
+      <c r="H119" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I119" s="27" t="s">
+        <v>3476</v>
+      </c>
+      <c r="J119" s="32" t="s">
+        <v>3477</v>
+      </c>
+      <c r="K119" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L119" t="s">
+        <v>61</v>
+      </c>
+      <c r="M119" s="7" t="s">
+        <v>3227</v>
+      </c>
+      <c r="N119" t="s">
         <v>25</v>
       </c>
     </row>
@@ -16238,9 +16424,13 @@
     <hyperlink ref="I115" r:id="rId91" xr:uid="{42FBB82F-FA0A-49B4-BEC5-E4E89D6CB366}"/>
     <hyperlink ref="I117" r:id="rId92" xr:uid="{23D714D4-7CC4-4BAB-A4CC-6A79467AD22E}"/>
     <hyperlink ref="J117" r:id="rId93" xr:uid="{0C0CFB93-4989-4142-A8A1-5426DCB29DF6}"/>
+    <hyperlink ref="I118" r:id="rId94" xr:uid="{E8F66462-23F8-4357-86E4-F00E1DDD00BD}"/>
+    <hyperlink ref="J118" r:id="rId95" xr:uid="{0DDD8FD6-EB7C-4099-AC8D-546E7FFB975A}"/>
+    <hyperlink ref="I119" r:id="rId96" xr:uid="{3E85D3AE-5734-420B-B08C-558D7D7AE59C}"/>
+    <hyperlink ref="J119" r:id="rId97" xr:uid="{4F7D3F8C-8C44-41BA-BBA8-939E653CA2D5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId94"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId98"/>
 </worksheet>
 </file>
 
@@ -25029,14 +25219,56 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="E3" s="36"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="A3" t="s">
+        <v>3484</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3485</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>3486</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>3487</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3488</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>3316</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3489</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="27" t="s">
+        <v>3490</v>
+      </c>
+      <c r="J3" s="27" t="s">
+        <v>3491</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3492</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{A3195937-552B-4025-8C26-81ADB44BFFC2}"/>
     <hyperlink ref="J2" r:id="rId2" xr:uid="{52A98722-6674-4772-ABA0-DFA6125FAC08}"/>
+    <hyperlink ref="I3" r:id="rId3" xr:uid="{349067E1-E702-4B84-8148-B4C1A22F177F}"/>
+    <hyperlink ref="J3" r:id="rId4" xr:uid="{C828D96D-14A3-4C4F-A35B-A9CD2A9F5BC8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32661,7 +32893,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D956EFE-E955-4E62-8478-2294E6413DC1}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -32752,9 +32984,56 @@
         <v>25</v>
       </c>
     </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>3493</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3494</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>3495</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>3496</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3497</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>3498</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="27" t="s">
+        <v>3499</v>
+      </c>
+      <c r="J3" s="32" t="s">
+        <v>3500</v>
+      </c>
+      <c r="K3" t="s">
+        <v>2903</v>
+      </c>
+      <c r="L3" t="s">
+        <v>2904</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3501</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{1A9E4CB0-A8E7-4FC1-A9A7-FA5E28311F4C}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{56FF5CE4-5A16-43B7-A444-8540568671A8}"/>
+    <hyperlink ref="J3" r:id="rId3" xr:uid="{5A2C53EE-4AA9-4D60-B6B6-16BED3AC487F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
010-0161, 010-0162, 010-0163, 010-0164, 001-0119, 001-0120 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7643704E-0F7D-4704-8899-B926297121C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE71E387-20A1-4B98-8AE0-E7021B06AE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46695" yWindow="2355" windowWidth="14610" windowHeight="15585" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46695" yWindow="2355" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7020" uniqueCount="3502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7105" uniqueCount="3543">
   <si>
     <t>ID</t>
   </si>
@@ -10553,6 +10553,129 @@
   </si>
   <si>
     <t>IND_CMM_THT_11x11mm</t>
+  </si>
+  <si>
+    <t>010-0161</t>
+  </si>
+  <si>
+    <t>010-0162</t>
+  </si>
+  <si>
+    <t>010-0163</t>
+  </si>
+  <si>
+    <t>010-0164</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors CHIP RESISTOR Precision</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 1.8Kohm 0.1% 10ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors RP 2A 20R 0.1% 15PPM CUT LENGTH</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 2.2Kohm 0.1% 15ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>1MΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>1.8kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>20Ω 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>2.2kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>CRT1206-BW-1004ELF</t>
+  </si>
+  <si>
+    <t>652-CRT1206BW1004ELF</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/40/1/CRT.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Bourns/CRT1206-BW-1004ELF?qs=sGAEpiMZZMvdGkrng054t9uZ12tsVZVXUwFPKPuMiMw%3D</t>
+  </si>
+  <si>
+    <t>ERA-6ARB182V</t>
+  </si>
+  <si>
+    <t>667-ERA-6ARB182V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6ARB182V?qs=sGAEpiMZZMvdGkrng054t7Q%2FBjLwFmgiTwW2qqIgdzU%3D</t>
+  </si>
+  <si>
+    <t>RP73D2A20RBTG</t>
+  </si>
+  <si>
+    <t>TE</t>
+  </si>
+  <si>
+    <t>279-RP73D2A20RBTG</t>
+  </si>
+  <si>
+    <t>https://www.te.com/commerce/DocumentDelivery/DDEController?Action=showdoc&amp;DocId=Data+Sheet%7F1773272%7FL%7Fpdf%7FEnglish%7FENG_DS_1773272_L.pdf%7F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TE-Connectivity-Holsworthy/RP73D2A20RBTG?qs=sGAEpiMZZMvdGkrng054t9WFtWtrbdtG%2F6%2Fjgh8ECZ8%3D</t>
+  </si>
+  <si>
+    <t>ERA-6APB222V</t>
+  </si>
+  <si>
+    <t>667-ERA-6APB222V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6APB222V?qs=sGAEpiMZZMvdGkrng054t7Q%2FBjLwFmgixWLzItBYhMc%3D</t>
+  </si>
+  <si>
+    <t>001-0119</t>
+  </si>
+  <si>
+    <t>001-0120</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 25V 10pF C0G 0402 0. 1pF</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 0603 330pF 25volts C0G 1%</t>
+  </si>
+  <si>
+    <t>25V 10pF NP0</t>
+  </si>
+  <si>
+    <t>25V 330pF NP0</t>
+  </si>
+  <si>
+    <t>04023A100BAT2A</t>
+  </si>
+  <si>
+    <t>581-04023A100BAT2A</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/5926/1/C0GNP0_Dielectric.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/04023A100BAT2A?qs=Op3aA%252BNiUY5yU4vAZ7xiKg%3D%3D</t>
+  </si>
+  <si>
+    <t>VJ0603A331FXXCW1BC</t>
+  </si>
+  <si>
+    <t>77-VJ0603A331FXXCBC</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/28548/vjw1bcbascomseries.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Vitramon/VJ0603A331FXXCW1BC?qs=%2Fh0R4aLiLgPLKHvkP5P%252BKw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -10731,7 +10854,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10790,8 +10913,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -11075,7 +11197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -16325,6 +16447,94 @@
         <v>3227</v>
       </c>
       <c r="N119" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
+      <c r="A120" s="4" t="s">
+        <v>3529</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>3531</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>3533</v>
+      </c>
+      <c r="D120" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E120" t="s">
+        <v>3535</v>
+      </c>
+      <c r="F120" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G120" t="s">
+        <v>3536</v>
+      </c>
+      <c r="H120" t="s">
+        <v>21</v>
+      </c>
+      <c r="I120" s="2" t="s">
+        <v>3537</v>
+      </c>
+      <c r="J120" s="2" t="s">
+        <v>3538</v>
+      </c>
+      <c r="K120" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L120" t="s">
+        <v>61</v>
+      </c>
+      <c r="M120" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="N120" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
+      <c r="A121" s="4" t="s">
+        <v>3530</v>
+      </c>
+      <c r="B121" t="s">
+        <v>3532</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>3534</v>
+      </c>
+      <c r="D121" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E121" t="s">
+        <v>3539</v>
+      </c>
+      <c r="F121" t="s">
+        <v>3311</v>
+      </c>
+      <c r="G121" t="s">
+        <v>3540</v>
+      </c>
+      <c r="H121" t="s">
+        <v>21</v>
+      </c>
+      <c r="I121" t="s">
+        <v>3541</v>
+      </c>
+      <c r="J121" s="2" t="s">
+        <v>3542</v>
+      </c>
+      <c r="K121" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L121" t="s">
+        <v>61</v>
+      </c>
+      <c r="M121" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N121" t="s">
         <v>25</v>
       </c>
     </row>
@@ -16428,9 +16638,12 @@
     <hyperlink ref="J118" r:id="rId95" xr:uid="{0DDD8FD6-EB7C-4099-AC8D-546E7FFB975A}"/>
     <hyperlink ref="I119" r:id="rId96" xr:uid="{3E85D3AE-5734-420B-B08C-558D7D7AE59C}"/>
     <hyperlink ref="J119" r:id="rId97" xr:uid="{4F7D3F8C-8C44-41BA-BBA8-939E653CA2D5}"/>
+    <hyperlink ref="I120" r:id="rId98" xr:uid="{C96C48DA-EDC8-49C8-AF84-EC04D1CADF1F}"/>
+    <hyperlink ref="J120" r:id="rId99" xr:uid="{82BD7645-36AC-4B87-A6AC-DC24E52B487C}"/>
+    <hyperlink ref="J121" r:id="rId100" xr:uid="{8D158E67-4FC0-4FA4-904D-A0664134DB5C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId98"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId101"/>
 </worksheet>
 </file>
 
@@ -25228,7 +25441,7 @@
       <c r="C3" s="3" t="s">
         <v>3486</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="3" t="s">
         <v>3487</v>
       </c>
       <c r="E3" t="s">
@@ -25276,7 +25489,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N161"/>
+  <dimension ref="A1:N165"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -32337,8 +32550,8 @@
       <c r="D161" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E161">
-        <v>560112116001</v>
+      <c r="E161" s="36" t="s">
+        <v>3106</v>
       </c>
       <c r="F161" s="16" t="s">
         <v>2100</v>
@@ -32365,6 +32578,182 @@
         <v>57</v>
       </c>
       <c r="N161" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="162" spans="1:14">
+      <c r="A162" s="16" t="s">
+        <v>3502</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>3506</v>
+      </c>
+      <c r="C162" s="16" t="s">
+        <v>3510</v>
+      </c>
+      <c r="D162" s="38" t="s">
+        <v>249</v>
+      </c>
+      <c r="E162" t="s">
+        <v>3514</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>1516</v>
+      </c>
+      <c r="G162" s="3" t="s">
+        <v>3515</v>
+      </c>
+      <c r="H162" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I162" s="27" t="s">
+        <v>3516</v>
+      </c>
+      <c r="J162" s="32" t="s">
+        <v>3517</v>
+      </c>
+      <c r="K162" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L162" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M162" s="7" t="s">
+        <v>1645</v>
+      </c>
+      <c r="N162" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="163" spans="1:14">
+      <c r="A163" s="16" t="s">
+        <v>3503</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>3507</v>
+      </c>
+      <c r="C163" s="16" t="s">
+        <v>3511</v>
+      </c>
+      <c r="D163" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E163" t="s">
+        <v>3518</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G163" s="3" t="s">
+        <v>3519</v>
+      </c>
+      <c r="H163" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I163" s="27" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J163" s="32" t="s">
+        <v>3520</v>
+      </c>
+      <c r="K163" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L163" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M163" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N163" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="164" spans="1:14">
+      <c r="A164" s="16" t="s">
+        <v>3504</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>3508</v>
+      </c>
+      <c r="C164" s="16" t="s">
+        <v>3512</v>
+      </c>
+      <c r="D164" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E164" t="s">
+        <v>3521</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>3522</v>
+      </c>
+      <c r="G164" s="3" t="s">
+        <v>3523</v>
+      </c>
+      <c r="H164" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I164" s="27" t="s">
+        <v>3524</v>
+      </c>
+      <c r="J164" s="32" t="s">
+        <v>3525</v>
+      </c>
+      <c r="K164" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L164" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M164" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N164" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="165" spans="1:14">
+      <c r="A165" s="16" t="s">
+        <v>3505</v>
+      </c>
+      <c r="B165" t="s">
+        <v>3509</v>
+      </c>
+      <c r="C165" s="16" t="s">
+        <v>3513</v>
+      </c>
+      <c r="D165" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E165" t="s">
+        <v>3526</v>
+      </c>
+      <c r="F165" s="3" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G165" s="3" t="s">
+        <v>3527</v>
+      </c>
+      <c r="H165" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I165" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J165" t="s">
+        <v>3528</v>
+      </c>
+      <c r="K165" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L165" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M165" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N165" t="s">
         <v>25</v>
       </c>
     </row>
@@ -32494,9 +32883,15 @@
     <hyperlink ref="I160" r:id="rId121" xr:uid="{38247BF1-5599-4165-BFEC-26629D789AC3}"/>
     <hyperlink ref="I161" r:id="rId122" xr:uid="{7C28565D-C222-4AEC-81A3-9D2C8C79A1A1}"/>
     <hyperlink ref="J161" r:id="rId123" xr:uid="{3A2D1BFE-71D6-460D-8752-1790B0BCD8EB}"/>
+    <hyperlink ref="I162" r:id="rId124" xr:uid="{4463DBEE-380B-4841-92E5-B0899C1AD050}"/>
+    <hyperlink ref="J162" r:id="rId125" xr:uid="{62FCC9B6-C758-4F6B-B770-33EEFB677F26}"/>
+    <hyperlink ref="I163" r:id="rId126" xr:uid="{B69945C4-5E62-46A4-B52C-B5FBF9EDB912}"/>
+    <hyperlink ref="J163" r:id="rId127" xr:uid="{E16CCBB4-7842-4D7A-96FB-5BD6FA1E6421}"/>
+    <hyperlink ref="I164" r:id="rId128" xr:uid="{7CE4EE78-4CA5-4B21-8D4B-AA08BC8B3267}"/>
+    <hyperlink ref="J164" r:id="rId129" xr:uid="{4DF264B3-7BEB-4A01-9BB8-A7BE1607E581}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId124"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId130"/>
 </worksheet>
 </file>
 
@@ -32994,7 +33389,7 @@
       <c r="C3" s="31" t="s">
         <v>3495</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="31" t="s">
         <v>3496</v>
       </c>
       <c r="E3" t="s">

</xml_diff>

<commit_message>
001-0121, 010-0167, 010-0168, 010-0169 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE110CB-2630-4579-9C13-EC515E231E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA4BEBE-085A-4A84-AC25-2280EFC350FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7146" uniqueCount="3566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7202" uniqueCount="3591">
   <si>
     <t>ID</t>
   </si>
@@ -10745,6 +10745,81 @@
   </si>
   <si>
     <t>010-0166</t>
+  </si>
+  <si>
+    <t>010-0167</t>
+  </si>
+  <si>
+    <t>010-0168</t>
+  </si>
+  <si>
+    <t>010-0169</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 Thin film chip resistor</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 3Kohm 0.1% 15ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 0805 33Kohm 0.1% 15ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>16.5kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>3kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>33kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>ERA-6ARB1652V</t>
+  </si>
+  <si>
+    <t>667-ERA-6ARB1652V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6ARB1652V?qs=sGAEpiMZZMvdGkrng054t%2FDNinWxsEFqx8wKlfWZmnLEWdfrAdOy9w%3D%3D</t>
+  </si>
+  <si>
+    <t>ERA-6APB302V</t>
+  </si>
+  <si>
+    <t>667-ERA-6APB302V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6APB302V?qs=sGAEpiMZZMvdGkrng054t7Q%2FBjLwFmgiNXNWyxy63ps%3D</t>
+  </si>
+  <si>
+    <t>ERA-6APB333V</t>
+  </si>
+  <si>
+    <t>667-ERA-6APB333V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6APB333V?qs=sGAEpiMZZMvdGkrng054t7Q%2FBjLwFmgi3idxPYTcWw0%3D</t>
+  </si>
+  <si>
+    <t>001-0121</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 25V 1500pF C0G 0603 1%</t>
+  </si>
+  <si>
+    <t>16V 1.5nF NP0</t>
+  </si>
+  <si>
+    <t>C0603C152F3GECTU</t>
+  </si>
+  <si>
+    <t>80-C0603C152F3GEC</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/508/1/KEM_C1091_C0G_ESD.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KEMET/C0603C152F3GECTU?qs=Mv7BduZupUh%252Bk5D8ZWarTg%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -11265,7 +11340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N121"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -16603,6 +16678,50 @@
         <v>62</v>
       </c>
       <c r="N121" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14">
+      <c r="A122" s="4" t="s">
+        <v>3584</v>
+      </c>
+      <c r="B122" t="s">
+        <v>3585</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>3586</v>
+      </c>
+      <c r="D122" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E122" t="s">
+        <v>3587</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>3316</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>3588</v>
+      </c>
+      <c r="H122" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I122" s="27" t="s">
+        <v>3589</v>
+      </c>
+      <c r="J122" s="27" t="s">
+        <v>3590</v>
+      </c>
+      <c r="K122" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L122" t="s">
+        <v>61</v>
+      </c>
+      <c r="M122" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N122" t="s">
         <v>25</v>
       </c>
     </row>
@@ -16709,9 +16828,11 @@
     <hyperlink ref="I120" r:id="rId98" xr:uid="{C96C48DA-EDC8-49C8-AF84-EC04D1CADF1F}"/>
     <hyperlink ref="J120" r:id="rId99" xr:uid="{82BD7645-36AC-4B87-A6AC-DC24E52B487C}"/>
     <hyperlink ref="J121" r:id="rId100" xr:uid="{8D158E67-4FC0-4FA4-904D-A0664134DB5C}"/>
+    <hyperlink ref="I122" r:id="rId101" xr:uid="{5646A60C-F082-4812-AAFF-C09F7BC184F6}"/>
+    <hyperlink ref="J122" r:id="rId102" xr:uid="{E13F1BFA-1BC5-4864-9D2F-0D97B5F47657}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId101"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId103"/>
 </worksheet>
 </file>
 
@@ -25601,7 +25722,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N167"/>
+  <dimension ref="A1:N170"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -32954,6 +33075,138 @@
         <v>1645</v>
       </c>
       <c r="N167" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="168" spans="1:14">
+      <c r="A168" s="16" t="s">
+        <v>3566</v>
+      </c>
+      <c r="B168" s="16" t="s">
+        <v>3569</v>
+      </c>
+      <c r="C168" s="16" t="s">
+        <v>3572</v>
+      </c>
+      <c r="D168" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E168" t="s">
+        <v>3575</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G168" s="3" t="s">
+        <v>3576</v>
+      </c>
+      <c r="H168" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I168" s="27" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J168" s="27" t="s">
+        <v>3577</v>
+      </c>
+      <c r="K168" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L168" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M168" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N168" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="169" spans="1:14">
+      <c r="A169" s="16" t="s">
+        <v>3567</v>
+      </c>
+      <c r="B169" s="16" t="s">
+        <v>3570</v>
+      </c>
+      <c r="C169" s="16" t="s">
+        <v>3573</v>
+      </c>
+      <c r="D169" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E169" t="s">
+        <v>3578</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G169" s="3" t="s">
+        <v>3579</v>
+      </c>
+      <c r="H169" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I169" s="27" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J169" t="s">
+        <v>3580</v>
+      </c>
+      <c r="K169" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L169" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M169" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N169" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="170" spans="1:14">
+      <c r="A170" s="16" t="s">
+        <v>3568</v>
+      </c>
+      <c r="B170" t="s">
+        <v>3571</v>
+      </c>
+      <c r="C170" s="16" t="s">
+        <v>3574</v>
+      </c>
+      <c r="D170" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E170" t="s">
+        <v>3581</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G170" s="3" t="s">
+        <v>3582</v>
+      </c>
+      <c r="H170" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I170" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J170" t="s">
+        <v>3583</v>
+      </c>
+      <c r="K170" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L170" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M170" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N170" t="s">
         <v>25</v>
       </c>
     </row>
@@ -33092,9 +33345,12 @@
     <hyperlink ref="I166" r:id="rId130" display="https://www.mouser.com/catalog/specsheets/KOA_Speer_RN73R__8_20_24.pdf?_gl=1*23gnzt*_gcl_aw*R0NMLjE3ODA5NDM2MTUuQ2owS0NRancwSm5SQmhESkFSSXNBTG9iblhiTVZmV3NWb0pqSGVpNWRkTXk2SzRuNEhwRGVRWXYxa0dMT0s1N0VWSjRWQlE1eFhBYUoxd2FBa3NuRUFMd193Y0I.*_gcl_au*MjAyMjI4MzgwOS4xNzc1NDk0ODAwLjEzNzM0NjYwNTMuMTc4MTk0MzEyNS4xNzgxOTQ0MDMw*_ga*Nzg3Njk5NTY0LjE3NDY2Mzg0MjI.*_ga_15W4STQT4T*czE3ODE5NDMwOTckbzk3JGcxJHQxNzgxOTQ0MDQwJGo0MCRsMCRoMA.." xr:uid="{637208B5-2C9A-4EEB-9CE7-9AEB37AC38F3}"/>
     <hyperlink ref="J166" r:id="rId131" xr:uid="{C0A169AF-232E-42CF-80E5-11600433186C}"/>
     <hyperlink ref="J167" r:id="rId132" xr:uid="{42A48B33-700F-4889-AE6E-DC32FECC2541}"/>
+    <hyperlink ref="I168" r:id="rId133" xr:uid="{5017C3EA-65D9-46AF-AF8E-218938D0A3B7}"/>
+    <hyperlink ref="J168" r:id="rId134" xr:uid="{18E306B2-279B-447D-8479-574435B55633}"/>
+    <hyperlink ref="I169" r:id="rId135" xr:uid="{0DCBF918-6691-4999-BB88-8B4F9C447EAB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId133"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId136"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
010-0170, 010-0171, 050-0005 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA4BEBE-085A-4A84-AC25-2280EFC350FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F02F2F-84B1-4490-AC16-5CF383DE7186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7202" uniqueCount="3591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7244" uniqueCount="3613">
   <si>
     <t>ID</t>
   </si>
@@ -10820,6 +10820,72 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/KEMET/C0603C152F3GECTU?qs=Mv7BduZupUh%252Bk5D8ZWarTg%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0170</t>
+  </si>
+  <si>
+    <t>010-0171</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 1 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 28 kOhms 1 % 0.1 W 0402 AEC-Q200</t>
+  </si>
+  <si>
+    <t>1kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>2.8kΩ 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116014</t>
+  </si>
+  <si>
+    <t>710-560112116014</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116014.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116014?qs=sGAEpiMZZMvdGkrng054txLI%2FDB4oIKD92viHLDiYpSVemZawWv4yQ%3D%3D</t>
+  </si>
+  <si>
+    <t>560112110228</t>
+  </si>
+  <si>
+    <t>710-560112110228</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112110228.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112110228?qs=mELouGlnn3ckGB3GQT9Puw%3D%3D</t>
+  </si>
+  <si>
+    <t>050-0005</t>
+  </si>
+  <si>
+    <t>Comparadores analógicos Dual Differential A 595-TLC372CPW A 595- A 595-TLC372CPW</t>
+  </si>
+  <si>
+    <t>TSSOP-8</t>
+  </si>
+  <si>
+    <t>TLC372CPWR</t>
+  </si>
+  <si>
+    <t>595-TLC372CPWR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/tlc372.pdf?ts=1782158413305&amp;ref_url=https%253A%252F%252Fwww.mouser.es%252F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/TLC372CPWR?qs=Zu35EjizYSQJQcLjIiS2wQ%3D%3D</t>
+  </si>
+  <si>
+    <t>TLC372C</t>
   </si>
 </sst>
 </file>
@@ -20168,7 +20234,7 @@
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="93.81640625" customWidth="1"/>
+    <col min="2" max="2" width="43.7265625" customWidth="1"/>
     <col min="5" max="5" width="16.1796875" customWidth="1"/>
     <col min="6" max="6" width="17.81640625" customWidth="1"/>
     <col min="7" max="7" width="16.7265625" customWidth="1"/>
@@ -20240,10 +20306,10 @@
         <v>18</v>
       </c>
       <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
         <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -20284,10 +20350,10 @@
         <v>39</v>
       </c>
       <c r="F3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" t="s">
         <v>40</v>
-      </c>
-      <c r="G3" t="s">
-        <v>41</v>
       </c>
       <c r="H3" t="s">
         <v>21</v>
@@ -20328,10 +20394,10 @@
         <v>18</v>
       </c>
       <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
         <v>1652</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
       </c>
       <c r="H4" t="s">
         <v>69</v>
@@ -20372,10 +20438,10 @@
         <v>39</v>
       </c>
       <c r="F5" t="s">
+        <v>1658</v>
+      </c>
+      <c r="G5" t="s">
         <v>1657</v>
-      </c>
-      <c r="G5" t="s">
-        <v>1658</v>
       </c>
       <c r="H5" t="s">
         <v>69</v>
@@ -20399,17 +20465,64 @@
         <v>25</v>
       </c>
     </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>3605</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>3606</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3607</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3608</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>3609</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>3610</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>3611</v>
+      </c>
+      <c r="K6" t="s">
+        <v>3612</v>
+      </c>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>3607</v>
+      </c>
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="9" spans="1:14">
       <c r="L9" s="21"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" xr:uid="{78125F11-BE4E-4312-8E61-0550889BB81F}"/>
     <hyperlink ref="I2" r:id="rId2" xr:uid="{1CFCC581-B5E5-4159-8EE1-35A941FCD4DF}"/>
     <hyperlink ref="J4" r:id="rId3" xr:uid="{BD7BCD4B-25F3-483F-8F98-D146F94F5AAF}"/>
+    <hyperlink ref="I6" r:id="rId4" xr:uid="{9E4B6332-A551-48B7-BFF0-45B7D65C08A2}"/>
+    <hyperlink ref="J6" r:id="rId5" xr:uid="{2277AFAF-7670-400C-9F4A-5D96406C91FF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -25722,7 +25835,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N170"/>
+  <dimension ref="A1:N172"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -33207,6 +33320,94 @@
         <v>1646</v>
       </c>
       <c r="N170" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="171" spans="1:14">
+      <c r="A171" s="16" t="s">
+        <v>3591</v>
+      </c>
+      <c r="B171" s="16" t="s">
+        <v>3593</v>
+      </c>
+      <c r="C171" s="16" t="s">
+        <v>3595</v>
+      </c>
+      <c r="D171" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E171" s="36" t="s">
+        <v>3597</v>
+      </c>
+      <c r="F171" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G171" t="s">
+        <v>3598</v>
+      </c>
+      <c r="H171" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I171" t="s">
+        <v>3599</v>
+      </c>
+      <c r="J171" s="2" t="s">
+        <v>3600</v>
+      </c>
+      <c r="K171" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L171" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M171" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N171" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="172" spans="1:14">
+      <c r="A172" s="16" t="s">
+        <v>3592</v>
+      </c>
+      <c r="B172" t="s">
+        <v>3594</v>
+      </c>
+      <c r="C172" s="16" t="s">
+        <v>3596</v>
+      </c>
+      <c r="D172" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E172" s="36" t="s">
+        <v>3601</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G172" t="s">
+        <v>3602</v>
+      </c>
+      <c r="H172" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I172" s="27" t="s">
+        <v>3603</v>
+      </c>
+      <c r="J172" s="2" t="s">
+        <v>3604</v>
+      </c>
+      <c r="K172" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L172" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M172" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N172" t="s">
         <v>25</v>
       </c>
     </row>
@@ -33348,9 +33549,12 @@
     <hyperlink ref="I168" r:id="rId133" xr:uid="{5017C3EA-65D9-46AF-AF8E-218938D0A3B7}"/>
     <hyperlink ref="J168" r:id="rId134" xr:uid="{18E306B2-279B-447D-8479-574435B55633}"/>
     <hyperlink ref="I169" r:id="rId135" xr:uid="{0DCBF918-6691-4999-BB88-8B4F9C447EAB}"/>
+    <hyperlink ref="J171" r:id="rId136" xr:uid="{DCF772DB-BDD0-4B1A-9FFA-545D6848BA75}"/>
+    <hyperlink ref="I172" r:id="rId137" xr:uid="{FA50CF1F-CE1E-48C4-AFFC-FEFE4E08F6BD}"/>
+    <hyperlink ref="J172" r:id="rId138" xr:uid="{B2371745-8711-4172-950E-289F49877CF4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId136"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId139"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
010-0173, 010-0172, 050-0006 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F02F2F-84B1-4490-AC16-5CF383DE7186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6286F60-DE9F-4D2F-AACF-1202290F46B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7244" uniqueCount="3613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7286" uniqueCount="3633">
   <si>
     <t>ID</t>
   </si>
@@ -10886,6 +10886,66 @@
   </si>
   <si>
     <t>TLC372C</t>
+  </si>
+  <si>
+    <t>560112116009</t>
+  </si>
+  <si>
+    <t>710-560112116009</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116009.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116009?qs=sGAEpiMZZMvdGkrng054txLI%2FDB4oIKDTCqaE%2Fpesdwv2JWXHdCmlQ%3D%3D</t>
+  </si>
+  <si>
+    <t>TNPW060317K6BEEA</t>
+  </si>
+  <si>
+    <t>71-TNPW060317K6BEEA</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/28758/tnpw_e3.pdf</t>
+  </si>
+  <si>
+    <t>17.6kΩ 210mW ±1%</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 100 Ohms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>Thin Film Resistors 17.6Kohms .1% 25ppm</t>
+  </si>
+  <si>
+    <t>010-0172</t>
+  </si>
+  <si>
+    <t>010-0173</t>
+  </si>
+  <si>
+    <t>050-0006</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/sn74act10-q1.pdf?ts=1755166715768&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fsitesearch%252Fen-us%252Fdocs%252Funiversalsearch.tsp%253FlangPref%253Den-US%2526nr%253D2%2526searchTerm%253DSN74ACT10WBQARQ1</t>
+  </si>
+  <si>
+    <t>Puertas lógicas Automotive 3-ch 3- i nput 1.5V to 6V 24</t>
+  </si>
+  <si>
+    <t>SN74ACT10QPWRG4Q1</t>
+  </si>
+  <si>
+    <t>595-N74ACT10QPWRG4Q1</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Texas-Instruments/SN74ACT10QPWRG4Q1?qs=sGAEpiMZZMutXGli8Ay4kFDTtzDUNYkmI6wEEhUY5cY%3D</t>
+  </si>
+  <si>
+    <t>SN74ACT10-Q1</t>
+  </si>
+  <si>
+    <t>TSSOP-14</t>
   </si>
 </sst>
 </file>
@@ -20509,6 +20569,50 @@
         <v>25</v>
       </c>
     </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>3625</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>3627</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3632</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3628</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>3629</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="27" t="s">
+        <v>3626</v>
+      </c>
+      <c r="J7" s="27" t="s">
+        <v>3630</v>
+      </c>
+      <c r="K7" t="s">
+        <v>3631</v>
+      </c>
+      <c r="L7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" t="s">
+        <v>3632</v>
+      </c>
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="9" spans="1:14">
       <c r="L9" s="21"/>
     </row>
@@ -20520,9 +20624,10 @@
     <hyperlink ref="J4" r:id="rId3" xr:uid="{BD7BCD4B-25F3-483F-8F98-D146F94F5AAF}"/>
     <hyperlink ref="I6" r:id="rId4" xr:uid="{9E4B6332-A551-48B7-BFF0-45B7D65C08A2}"/>
     <hyperlink ref="J6" r:id="rId5" xr:uid="{2277AFAF-7670-400C-9F4A-5D96406C91FF}"/>
+    <hyperlink ref="I7" r:id="rId6" xr:uid="{4EE7BCCF-17ED-4BF0-90C6-97AD9B6D2A45}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -25835,7 +25940,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N172"/>
+  <dimension ref="A1:N174"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -33408,6 +33513,94 @@
         <v>1644</v>
       </c>
       <c r="N172" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="173" spans="1:14">
+      <c r="A173" s="16" t="s">
+        <v>3623</v>
+      </c>
+      <c r="B173" s="16" t="s">
+        <v>3621</v>
+      </c>
+      <c r="C173" s="16" t="s">
+        <v>1334</v>
+      </c>
+      <c r="D173" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E173" s="36" t="s">
+        <v>3613</v>
+      </c>
+      <c r="F173" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G173" t="s">
+        <v>3614</v>
+      </c>
+      <c r="H173" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I173" t="s">
+        <v>3615</v>
+      </c>
+      <c r="J173" s="2" t="s">
+        <v>3616</v>
+      </c>
+      <c r="K173" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L173" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M173" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N173" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="174" spans="1:14">
+      <c r="A174" s="16" t="s">
+        <v>3624</v>
+      </c>
+      <c r="B174" s="16" t="s">
+        <v>3622</v>
+      </c>
+      <c r="C174" s="16" t="s">
+        <v>3620</v>
+      </c>
+      <c r="D174" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E174" t="s">
+        <v>3617</v>
+      </c>
+      <c r="F174" s="3" t="s">
+        <v>3311</v>
+      </c>
+      <c r="G174" s="3" t="s">
+        <v>3618</v>
+      </c>
+      <c r="H174" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I174" t="s">
+        <v>3619</v>
+      </c>
+      <c r="J174" t="s">
+        <v>3619</v>
+      </c>
+      <c r="K174" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L174" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M174" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N174" t="s">
         <v>25</v>
       </c>
     </row>
@@ -33552,9 +33745,10 @@
     <hyperlink ref="J171" r:id="rId136" xr:uid="{DCF772DB-BDD0-4B1A-9FFA-545D6848BA75}"/>
     <hyperlink ref="I172" r:id="rId137" xr:uid="{FA50CF1F-CE1E-48C4-AFFC-FEFE4E08F6BD}"/>
     <hyperlink ref="J172" r:id="rId138" xr:uid="{B2371745-8711-4172-950E-289F49877CF4}"/>
+    <hyperlink ref="J173" r:id="rId139" xr:uid="{3A21D11A-C4F5-4700-844C-E488B5091D30}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId139"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId140"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
001-0123, 020-0003, 031-0013, 040-0021 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A36233-08C0-4E66-9885-4DBBF9911E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D470915-6B92-45F6-8D0F-A398B9E7A2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40305" yWindow="3975" windowWidth="16200" windowHeight="9975" firstSheet="19" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32280" yWindow="2235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7398" uniqueCount="3683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7467" uniqueCount="3720">
   <si>
     <t>ID</t>
   </si>
@@ -11097,6 +11097,117 @@
   </si>
   <si>
     <t>NCV8114</t>
+  </si>
+  <si>
+    <t>110-0065</t>
+  </si>
+  <si>
+    <t>Conectores para automoción 35P HEADER AMPSEAL ASSEMBLY</t>
+  </si>
+  <si>
+    <t>35P</t>
+  </si>
+  <si>
+    <t>THT 4mm</t>
+  </si>
+  <si>
+    <t>1-776163-1</t>
+  </si>
+  <si>
+    <t>571-1-776163-1</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/80/26/ENG_CD_776163_K1.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TE-Connectivity-AMP/1-776163-1?qs=VKrXD49J9EqcsUPRwW8PqQ%3D%3D</t>
+  </si>
+  <si>
+    <t>CONN 1-776163-1</t>
+  </si>
+  <si>
+    <t>Diodos y rectificadores Schottky 3A 60V</t>
+  </si>
+  <si>
+    <t>031-0013</t>
+  </si>
+  <si>
+    <t>MBRS360T3G</t>
+  </si>
+  <si>
+    <t>863-MBRS360T3G</t>
+  </si>
+  <si>
+    <t>https://www.onsemi.com/pdf/datasheet/mbrs360t3-d.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/onsemi/MBRS360T3G?qs=3JMERSakebpuPnGIg0cvPA%3D%3D</t>
+  </si>
+  <si>
+    <t>001-0123</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 10 uF 50 VDC 10% 0805 X5R</t>
+  </si>
+  <si>
+    <t>GRM21BR61H106KE43K</t>
+  </si>
+  <si>
+    <t>81-GRM21BR61H106KE3K</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/76/1/GRM21BR61H106KE43_01A.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Murata-Electronics/GRM21BR61H106KE43K?qs=xZ%2FP%252Ba9zWqbh3%252B96jyTKxw%3D%3D</t>
+  </si>
+  <si>
+    <t>020-0003</t>
+  </si>
+  <si>
+    <t>Inductores de potencia (SMD) WE-LHMI Powr SMD7030 10uH 3.0A 85mOhm</t>
+  </si>
+  <si>
+    <t>10uH 3A ±20%</t>
+  </si>
+  <si>
+    <t>SMD;7.3x6.6mm</t>
+  </si>
+  <si>
+    <t>IND SMD 7.3x6.6</t>
+  </si>
+  <si>
+    <t>74437346100</t>
+  </si>
+  <si>
+    <t>710-74437346100</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/74437346100.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/74437346100?qs=cFlH0mFHHFqNHncV%252BuVFvQ%3D%3D</t>
+  </si>
+  <si>
+    <t>040-0021</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 2.5A Fast Acting 1206 SinglFuse</t>
+  </si>
+  <si>
+    <t>2.5A</t>
+  </si>
+  <si>
+    <t>SF-1206F250-2</t>
+  </si>
+  <si>
+    <t>652-SF-1206F250-2</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/40/1/sf_1206f48eb4f2c90e165f58a72ff000066632f.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Bourns/SF-1206F250-2?qs=GIQXYiEeHGDcWHFyUr2UTQ%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -11281,7 +11392,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11344,6 +11455,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -11627,7 +11739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N123"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -17053,6 +17165,50 @@
         <v>3227</v>
       </c>
       <c r="N123" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14">
+      <c r="A124" s="39" t="s">
+        <v>3698</v>
+      </c>
+      <c r="B124" s="16" t="s">
+        <v>3699</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E124" t="s">
+        <v>3700</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>3701</v>
+      </c>
+      <c r="H124" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I124" s="27" t="s">
+        <v>3702</v>
+      </c>
+      <c r="J124" s="32" t="s">
+        <v>3703</v>
+      </c>
+      <c r="K124" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L124" t="s">
+        <v>61</v>
+      </c>
+      <c r="M124" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="N124" t="s">
         <v>25</v>
       </c>
     </row>
@@ -17163,9 +17319,11 @@
     <hyperlink ref="J122" r:id="rId102" xr:uid="{E13F1BFA-1BC5-4864-9D2F-0D97B5F47657}"/>
     <hyperlink ref="I123" r:id="rId103" xr:uid="{958FF4C4-BE0E-4556-B03B-7C4DCD6D04F9}"/>
     <hyperlink ref="J123" r:id="rId104" xr:uid="{FF54A4A3-2741-4A5A-9D1A-3F5746177EAD}"/>
+    <hyperlink ref="I124" r:id="rId105" xr:uid="{3BC617E5-C20D-4B7A-B6F8-6DE6572A7AA0}"/>
+    <hyperlink ref="J124" r:id="rId106" xr:uid="{69468929-3CB4-4434-AED4-E3828EC8E37D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId105"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId107"/>
 </worksheet>
 </file>
 
@@ -19278,7 +19436,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="13" max="13" width="13.36328125" customWidth="1"/>
@@ -20218,6 +20376,50 @@
         <v>1746</v>
       </c>
       <c r="N21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" t="s">
+        <v>3713</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>3714</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>3715</v>
+      </c>
+      <c r="D22" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3716</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>1516</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>3717</v>
+      </c>
+      <c r="H22" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I22" s="27" t="s">
+        <v>3718</v>
+      </c>
+      <c r="J22" s="32" t="s">
+        <v>3719</v>
+      </c>
+      <c r="K22" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L22" t="s">
+        <v>55</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N22" t="s">
         <v>25</v>
       </c>
     </row>
@@ -20240,6 +20442,8 @@
     <hyperlink ref="I20" r:id="rId14" xr:uid="{6C9DFF48-0956-4B25-8972-EC0656F1483E}"/>
     <hyperlink ref="J20" r:id="rId15" xr:uid="{6EF40273-C6D8-4BC3-9EF6-1B4C76903848}"/>
     <hyperlink ref="J21" r:id="rId16" xr:uid="{FFB17F08-401F-47B0-899B-612CD8B9FB6B}"/>
+    <hyperlink ref="I22" r:id="rId17" xr:uid="{1372C46B-1234-4FDC-9A5A-49F3F36A3112}"/>
+    <hyperlink ref="J22" r:id="rId18" xr:uid="{5B608490-0175-4BFB-8CEB-749053C4E8DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23255,7 +23459,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="5" max="5" width="16.36328125" bestFit="1" customWidth="1"/>
@@ -26120,6 +26324,50 @@
         <v>7461117</v>
       </c>
       <c r="N65" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
+      <c r="A66" s="16" t="s">
+        <v>3683</v>
+      </c>
+      <c r="B66" s="16" t="s">
+        <v>3684</v>
+      </c>
+      <c r="C66" s="16" t="s">
+        <v>3685</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>3686</v>
+      </c>
+      <c r="E66" t="s">
+        <v>3687</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>2192</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>3688</v>
+      </c>
+      <c r="H66" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I66" s="27" t="s">
+        <v>3689</v>
+      </c>
+      <c r="J66" s="32" t="s">
+        <v>3690</v>
+      </c>
+      <c r="K66" s="17" t="s">
+        <v>3691</v>
+      </c>
+      <c r="L66" s="7" t="s">
+        <v>2572</v>
+      </c>
+      <c r="M66" t="s">
+        <v>3687</v>
+      </c>
+      <c r="N66" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -26182,6 +26430,8 @@
     <hyperlink ref="J63" r:id="rId54" xr:uid="{29B6CE96-A331-4903-A5B6-DD5273C7B49A}"/>
     <hyperlink ref="I64" r:id="rId55" xr:uid="{5CA52475-6941-42F8-9AA3-C5156AF91DB1}"/>
     <hyperlink ref="J64" r:id="rId56" xr:uid="{0176710A-1D50-48A9-9ACC-C0E8F9C09246}"/>
+    <hyperlink ref="I66" r:id="rId57" xr:uid="{F4FD0F61-138E-4DBE-8F6A-3A26376F772A}"/>
+    <hyperlink ref="J66" r:id="rId58" xr:uid="{F9BBC9A3-5DDE-4132-B9F9-18EE393B61F2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -34535,7 +34785,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C6B0FD-D8A3-44EC-9532-03DDA232F922}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -34667,6 +34917,50 @@
         <v>3415</v>
       </c>
       <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>3704</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>3705</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3706</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3707</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>3709</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>3710</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="27" t="s">
+        <v>3711</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>3712</v>
+      </c>
+      <c r="K4" t="s">
+        <v>3406</v>
+      </c>
+      <c r="L4" t="s">
+        <v>2904</v>
+      </c>
+      <c r="M4" s="17" t="s">
+        <v>3708</v>
+      </c>
+      <c r="N4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -34676,9 +34970,11 @@
     <hyperlink ref="I2" r:id="rId1" xr:uid="{07883802-B058-47F9-BBB3-C06E82952829}"/>
     <hyperlink ref="J2" r:id="rId2" xr:uid="{62DD0F89-540D-4537-B7A5-4B172FA10C23}"/>
     <hyperlink ref="I3" r:id="rId3" xr:uid="{A45B5B86-5ADB-44B4-BF96-CFB1161AF6C6}"/>
+    <hyperlink ref="I4" r:id="rId4" xr:uid="{172DE15B-CE66-4479-BB47-E78881F87955}"/>
+    <hyperlink ref="J4" r:id="rId5" xr:uid="{554E337A-6092-4CB5-BAAD-9E740E529981}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -35244,7 +35540,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2008B-4BF4-4C9A-883A-FEE5873AEAF4}">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14" ht="16" customHeight="1">
@@ -35816,6 +36112,50 @@
         <v>1994</v>
       </c>
       <c r="N13" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="16" t="s">
+        <v>3693</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>3692</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>1997</v>
+      </c>
+      <c r="D14" s="40" t="s">
+        <v>2047</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3694</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>1858</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>3695</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" s="27" t="s">
+        <v>3696</v>
+      </c>
+      <c r="J14" s="32" t="s">
+        <v>3697</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>1918</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>1910</v>
+      </c>
+      <c r="M14" t="s">
+        <v>2047</v>
+      </c>
+      <c r="N14" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -35834,6 +36174,8 @@
     <hyperlink ref="I11" r:id="rId10" xr:uid="{E8167B89-7FBA-4877-BC25-3D4C05ED8AA6}"/>
     <hyperlink ref="I12" r:id="rId11" xr:uid="{C4B46D5B-BD3F-4DBC-A61E-40C494B3D177}"/>
     <hyperlink ref="J13" r:id="rId12" xr:uid="{0C7D58F5-DE06-4F14-BC9F-F6688DDA76B4}"/>
+    <hyperlink ref="I14" r:id="rId13" xr:uid="{69D5D5EE-78C1-424D-8FB6-5CEE6BF86BEE}"/>
+    <hyperlink ref="J14" r:id="rId14" xr:uid="{E4E8D2D8-B131-437F-A58D-DE6AA7E926D6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
010-0184, 010-0185, 010-0186 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA813EBF-8389-4C81-B2ED-461B0C1711E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5621C71C-6C41-47E7-A527-FED67CACD76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37332" yWindow="2100" windowWidth="11724" windowHeight="12336" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25812" yWindow="1992" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7718" uniqueCount="3841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7774" uniqueCount="3867">
   <si>
     <t>ID</t>
   </si>
@@ -11571,6 +11571,84 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/TE-Connectivity-Holsworthy/RQ73C1J20KBTD?qs=gZXFycFWdAPzh65iaC%2FK3A%3D%3D</t>
+  </si>
+  <si>
+    <t>001-0128</t>
+  </si>
+  <si>
+    <t>Condensadores de cerámica multicapa (MLCC- SMD/SMT) 4300 pF 25 VDC 2% 0603 C0G (NP0)</t>
+  </si>
+  <si>
+    <t>25V 4.3nF NP0</t>
+  </si>
+  <si>
+    <t>GRM1885C1E432GA01J</t>
+  </si>
+  <si>
+    <t>81-GRM1885C1E432GA1J</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/76/1/GRM1885C1E432GA01-01A.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Murata-Electronics/GRM1885C1E432GA01J?qs=QzBtWTOodeWyXLs1jqPc7Q%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0184</t>
+  </si>
+  <si>
+    <t>Resistores de película fina - SMD 0805 16Kohm 0.1% 10ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>ERA-6ARB163V</t>
+  </si>
+  <si>
+    <t>667-ERA-6ARB163V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6ARB163V?qs=sGAEpiMZZMtlubZbdhIBIJiMSTY83nT4nukUMCYb38k%3D</t>
+  </si>
+  <si>
+    <t>010-0185</t>
+  </si>
+  <si>
+    <t>Resistores de película fina - SMD 0805 24Kohm 0.1% 15ppm AEC-Q200</t>
+  </si>
+  <si>
+    <t>16kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>24kΩ 125mW ±0.1%</t>
+  </si>
+  <si>
+    <t>ERA-6APB243V</t>
+  </si>
+  <si>
+    <t>667-ERA-6APB243V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Panasonic/ERA-6APB243V?qs=ob%252BdNz2%252BYEgwblk2D2VCQQ%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0186</t>
+  </si>
+  <si>
+    <t>Resistores de película fina - SMD RQ 0805 12K1 0.1% 10PPM 5K RL</t>
+  </si>
+  <si>
+    <t>12kΩ 200mW ±0.1%</t>
+  </si>
+  <si>
+    <t>RQ73C2A12K1BTD</t>
+  </si>
+  <si>
+    <t>279-RQ73C2A12K1BTD</t>
+  </si>
+  <si>
+    <t>https://www.te.com/en/product-9-2176380-9.html</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/TE-Connectivity-Holsworthy/RQ73C2A12K1BTD?qs=gZXFycFWdAO8owZcKCpcmw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -12094,7 +12172,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N128"/>
+  <dimension ref="A1:N129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -17740,6 +17818,50 @@
         <v>62</v>
       </c>
       <c r="N128" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
+      <c r="A129" s="38" t="s">
+        <v>3841</v>
+      </c>
+      <c r="B129" s="16" t="s">
+        <v>3842</v>
+      </c>
+      <c r="C129" s="16" t="s">
+        <v>3843</v>
+      </c>
+      <c r="D129" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E129" t="s">
+        <v>3844</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>3845</v>
+      </c>
+      <c r="H129" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I129" s="26" t="s">
+        <v>3846</v>
+      </c>
+      <c r="J129" s="31" t="s">
+        <v>3847</v>
+      </c>
+      <c r="K129" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L129" t="s">
+        <v>61</v>
+      </c>
+      <c r="M129" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N129" t="s">
         <v>25</v>
       </c>
     </row>
@@ -17859,9 +17981,11 @@
     <hyperlink ref="J126" r:id="rId111" xr:uid="{348E15E9-2492-4FC3-9ADB-2287FB61453A}"/>
     <hyperlink ref="I128" r:id="rId112" xr:uid="{7E9F6B16-E367-4F43-A463-251B6118FB6C}"/>
     <hyperlink ref="J128" r:id="rId113" xr:uid="{6D13DE09-35E1-44E8-A161-CF565B19ADED}"/>
+    <hyperlink ref="I129" r:id="rId114" xr:uid="{FB710C94-A4D0-4FF6-A673-D2144CBFEE83}"/>
+    <hyperlink ref="J129" r:id="rId115" xr:uid="{9DCA9E08-FCEB-4C24-B9BD-2A4EB3937E26}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId114"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId116"/>
 </worksheet>
 </file>
 
@@ -27451,7 +27575,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N184"/>
+  <dimension ref="A1:N187"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -35512,7 +35636,7 @@
       <c r="A184" s="16" t="s">
         <v>3834</v>
       </c>
-      <c r="B184" s="39" t="s">
+      <c r="B184" s="16" t="s">
         <v>3835</v>
       </c>
       <c r="C184" s="16" t="s">
@@ -35521,16 +35645,16 @@
       <c r="D184" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E184" s="39" t="s">
+      <c r="E184" s="16" t="s">
         <v>3837</v>
       </c>
-      <c r="F184" s="40" t="s">
+      <c r="F184" s="30" t="s">
         <v>1524</v>
       </c>
-      <c r="G184" s="40" t="s">
+      <c r="G184" s="30" t="s">
         <v>3838</v>
       </c>
-      <c r="H184" s="39" t="s">
+      <c r="H184" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I184" s="26" t="s">
@@ -35549,6 +35673,138 @@
         <v>57</v>
       </c>
       <c r="N184" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="185" spans="1:14">
+      <c r="A185" s="16" t="s">
+        <v>3848</v>
+      </c>
+      <c r="B185" s="39" t="s">
+        <v>3849</v>
+      </c>
+      <c r="C185" s="16" t="s">
+        <v>3855</v>
+      </c>
+      <c r="D185" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E185" s="39" t="s">
+        <v>3850</v>
+      </c>
+      <c r="F185" s="40" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G185" s="40" t="s">
+        <v>3851</v>
+      </c>
+      <c r="H185" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I185" s="26" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J185" s="31" t="s">
+        <v>3852</v>
+      </c>
+      <c r="K185" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L185" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M185" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N185" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="186" spans="1:14">
+      <c r="A186" s="16" t="s">
+        <v>3853</v>
+      </c>
+      <c r="B186" s="39" t="s">
+        <v>3854</v>
+      </c>
+      <c r="C186" s="16" t="s">
+        <v>3856</v>
+      </c>
+      <c r="D186" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E186" s="39" t="s">
+        <v>3857</v>
+      </c>
+      <c r="F186" s="40" t="s">
+        <v>3342</v>
+      </c>
+      <c r="G186" s="40" t="s">
+        <v>3858</v>
+      </c>
+      <c r="H186" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I186" s="26" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J186" s="31" t="s">
+        <v>3859</v>
+      </c>
+      <c r="K186" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L186" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M186" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N186" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="187" spans="1:14">
+      <c r="A187" s="16" t="s">
+        <v>3860</v>
+      </c>
+      <c r="B187" s="39" t="s">
+        <v>3861</v>
+      </c>
+      <c r="C187" s="16" t="s">
+        <v>3862</v>
+      </c>
+      <c r="D187" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E187" s="39" t="s">
+        <v>3863</v>
+      </c>
+      <c r="F187" s="40" t="s">
+        <v>1524</v>
+      </c>
+      <c r="G187" s="40" t="s">
+        <v>3864</v>
+      </c>
+      <c r="H187" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I187" s="26" t="s">
+        <v>3865</v>
+      </c>
+      <c r="J187" s="31" t="s">
+        <v>3866</v>
+      </c>
+      <c r="K187" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L187" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M187" s="17" t="s">
+        <v>1646</v>
+      </c>
+      <c r="N187" t="s">
         <v>25</v>
       </c>
     </row>
@@ -35712,9 +35968,15 @@
     <hyperlink ref="J183" r:id="rId155" xr:uid="{3A9AF27C-EAA3-4F8D-B05D-139594372A97}"/>
     <hyperlink ref="I184" r:id="rId156" xr:uid="{D00616E2-05E3-4C0D-936C-236760B22307}"/>
     <hyperlink ref="J184" r:id="rId157" xr:uid="{7D0F9E12-2745-498A-B01D-8E33966F5A6D}"/>
+    <hyperlink ref="I185" r:id="rId158" xr:uid="{76F8280B-4CF8-4448-8C9A-3185533245A6}"/>
+    <hyperlink ref="J185" r:id="rId159" xr:uid="{F8240B68-10A9-44E1-9FC1-E1BCA6E4C641}"/>
+    <hyperlink ref="I186" r:id="rId160" xr:uid="{160C0D78-3243-4318-9D23-9CF9CA067F85}"/>
+    <hyperlink ref="J186" r:id="rId161" xr:uid="{6E7208C2-303A-4F5A-A973-294BBF656D01}"/>
+    <hyperlink ref="I187" r:id="rId162" xr:uid="{DEEBED7E-17D0-4EAC-BAFF-84DAFFF8847D}"/>
+    <hyperlink ref="J187" r:id="rId163" xr:uid="{4D207532-6F36-4B9E-ABE1-BC18363AB4D3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId158"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId164"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
010-0187, 010-0188, 010-0189, 010-0190 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5621C71C-6C41-47E7-A527-FED67CACD76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D26F753-56DD-4AAA-A5A3-CE78084B7F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25812" yWindow="1992" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25812" yWindow="1992" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7774" uniqueCount="3867">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7830" uniqueCount="3893">
   <si>
     <t>ID</t>
   </si>
@@ -11649,6 +11649,84 @@
   </si>
   <si>
     <t>https://www.mouser.es/ProductDetail/TE-Connectivity-Holsworthy/RQ73C2A12K1BTD?qs=gZXFycFWdAO8owZcKCpcmw%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0187</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 470 Ohms 5 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>470Ω 100mW ±5%</t>
+  </si>
+  <si>
+    <t>560112116031</t>
+  </si>
+  <si>
+    <t>710-560112116031</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116031.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116031?qs=sGAEpiMZZMvdGkrng054t2cqbZCzJY7Nc63jNcSJ2mNzAJgQFdfNBw%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0188</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 4.7 kOhms 5 % 0.1 W 0402 AEC-Q200</t>
+  </si>
+  <si>
+    <t>4.7kΩ 100mW ±5%</t>
+  </si>
+  <si>
+    <t>560112110018</t>
+  </si>
+  <si>
+    <t>710-560112110018</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112110018.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112110018?qs=sGAEpiMZZMvdGkrng054txLI%2FDB4oIKDXtogfAbE0Wc%252BspLjErwG3g%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0189</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 1 kOhms 1 % 0.25 W 1206 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112132038</t>
+  </si>
+  <si>
+    <t>710-560112132038</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112132038.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112132038?qs=sGAEpiMZZMvdGkrng054txLI%2FDB4oIKDY2lGR1OfVmrCt7nE4RR%2Faw%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0190</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors WRIS-RSKS 100 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>560112116004</t>
+  </si>
+  <si>
+    <t>710-560112116004</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116004.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Wurth-Elektronik/560112116004?qs=sGAEpiMZZMvdGkrng054txLI%2FDB4oIKDB%252BmfBE1ySSGuQklCN21gzA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -11825,7 +11903,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11887,8 +11965,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -27575,7 +27655,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N187"/>
+  <dimension ref="A1:N191"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -35680,7 +35760,7 @@
       <c r="A185" s="16" t="s">
         <v>3848</v>
       </c>
-      <c r="B185" s="39" t="s">
+      <c r="B185" s="16" t="s">
         <v>3849</v>
       </c>
       <c r="C185" s="16" t="s">
@@ -35689,16 +35769,16 @@
       <c r="D185" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="E185" s="39" t="s">
+      <c r="E185" s="16" t="s">
         <v>3850</v>
       </c>
-      <c r="F185" s="40" t="s">
+      <c r="F185" s="30" t="s">
         <v>3342</v>
       </c>
-      <c r="G185" s="40" t="s">
+      <c r="G185" s="30" t="s">
         <v>3851</v>
       </c>
-      <c r="H185" s="39" t="s">
+      <c r="H185" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I185" s="26" t="s">
@@ -35724,7 +35804,7 @@
       <c r="A186" s="16" t="s">
         <v>3853</v>
       </c>
-      <c r="B186" s="39" t="s">
+      <c r="B186" s="16" t="s">
         <v>3854</v>
       </c>
       <c r="C186" s="16" t="s">
@@ -35733,16 +35813,16 @@
       <c r="D186" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="E186" s="39" t="s">
+      <c r="E186" s="16" t="s">
         <v>3857</v>
       </c>
-      <c r="F186" s="40" t="s">
+      <c r="F186" s="30" t="s">
         <v>3342</v>
       </c>
-      <c r="G186" s="40" t="s">
+      <c r="G186" s="30" t="s">
         <v>3858</v>
       </c>
-      <c r="H186" s="39" t="s">
+      <c r="H186" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I186" s="26" t="s">
@@ -35768,7 +35848,7 @@
       <c r="A187" s="16" t="s">
         <v>3860</v>
       </c>
-      <c r="B187" s="39" t="s">
+      <c r="B187" s="16" t="s">
         <v>3861</v>
       </c>
       <c r="C187" s="16" t="s">
@@ -35777,16 +35857,16 @@
       <c r="D187" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="E187" s="39" t="s">
+      <c r="E187" s="16" t="s">
         <v>3863</v>
       </c>
-      <c r="F187" s="40" t="s">
+      <c r="F187" s="30" t="s">
         <v>1524</v>
       </c>
-      <c r="G187" s="40" t="s">
+      <c r="G187" s="30" t="s">
         <v>3864</v>
       </c>
-      <c r="H187" s="39" t="s">
+      <c r="H187" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I187" s="26" t="s">
@@ -35805,6 +35885,182 @@
         <v>1646</v>
       </c>
       <c r="N187" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="188" spans="1:14">
+      <c r="A188" s="16" t="s">
+        <v>3867</v>
+      </c>
+      <c r="B188" t="s">
+        <v>3868</v>
+      </c>
+      <c r="C188" s="16" t="s">
+        <v>3869</v>
+      </c>
+      <c r="D188" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E188" s="39" t="s">
+        <v>3870</v>
+      </c>
+      <c r="F188" s="40" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G188" s="41" t="s">
+        <v>3871</v>
+      </c>
+      <c r="H188" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I188" s="2" t="s">
+        <v>3872</v>
+      </c>
+      <c r="J188" s="2" t="s">
+        <v>3873</v>
+      </c>
+      <c r="K188" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L188" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M188" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N188" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="189" spans="1:14">
+      <c r="A189" s="16" t="s">
+        <v>3874</v>
+      </c>
+      <c r="B189" t="s">
+        <v>3875</v>
+      </c>
+      <c r="C189" s="16" t="s">
+        <v>3876</v>
+      </c>
+      <c r="D189" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E189" s="39" t="s">
+        <v>3877</v>
+      </c>
+      <c r="F189" s="40" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G189" s="40" t="s">
+        <v>3878</v>
+      </c>
+      <c r="H189" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I189" s="26" t="s">
+        <v>3879</v>
+      </c>
+      <c r="J189" s="31" t="s">
+        <v>3880</v>
+      </c>
+      <c r="K189" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L189" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M189" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N189" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="190" spans="1:14">
+      <c r="A190" s="16" t="s">
+        <v>3881</v>
+      </c>
+      <c r="B190" t="s">
+        <v>3882</v>
+      </c>
+      <c r="C190" s="16" t="s">
+        <v>921</v>
+      </c>
+      <c r="D190" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="E190" s="39" t="s">
+        <v>3883</v>
+      </c>
+      <c r="F190" s="40" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G190" s="40" t="s">
+        <v>3884</v>
+      </c>
+      <c r="H190" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I190" s="26" t="s">
+        <v>3885</v>
+      </c>
+      <c r="J190" s="31" t="s">
+        <v>3886</v>
+      </c>
+      <c r="K190" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L190" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M190" s="7" t="s">
+        <v>1645</v>
+      </c>
+      <c r="N190" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="191" spans="1:14">
+      <c r="A191" s="16" t="s">
+        <v>3887</v>
+      </c>
+      <c r="B191" t="s">
+        <v>3888</v>
+      </c>
+      <c r="C191" s="16" t="s">
+        <v>929</v>
+      </c>
+      <c r="D191" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E191" s="39" t="s">
+        <v>3889</v>
+      </c>
+      <c r="F191" s="40" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G191" s="40" t="s">
+        <v>3890</v>
+      </c>
+      <c r="H191" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I191" s="26" t="s">
+        <v>3891</v>
+      </c>
+      <c r="J191" s="31" t="s">
+        <v>3892</v>
+      </c>
+      <c r="K191" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L191" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M191" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N191" t="s">
         <v>25</v>
       </c>
     </row>
@@ -35974,9 +36230,17 @@
     <hyperlink ref="J186" r:id="rId161" xr:uid="{6E7208C2-303A-4F5A-A973-294BBF656D01}"/>
     <hyperlink ref="I187" r:id="rId162" xr:uid="{DEEBED7E-17D0-4EAC-BAFF-84DAFFF8847D}"/>
     <hyperlink ref="J187" r:id="rId163" xr:uid="{4D207532-6F36-4B9E-ABE1-BC18363AB4D3}"/>
+    <hyperlink ref="I188" r:id="rId164" xr:uid="{2870986C-1953-4DC5-9B89-873E713D299E}"/>
+    <hyperlink ref="J188" r:id="rId165" xr:uid="{A9897C76-A247-4FC9-9EB7-688C646664B8}"/>
+    <hyperlink ref="I189" r:id="rId166" xr:uid="{03119699-A4ED-41E9-802A-E01A41195490}"/>
+    <hyperlink ref="J189" r:id="rId167" xr:uid="{0B59B227-55EE-4290-A209-1475B1D01884}"/>
+    <hyperlink ref="I190" r:id="rId168" xr:uid="{066E29AC-27BD-48CF-96FC-427AF0B4A004}"/>
+    <hyperlink ref="J190" r:id="rId169" xr:uid="{0416598A-C30A-47A1-9871-D973FB462120}"/>
+    <hyperlink ref="I191" r:id="rId170" xr:uid="{1A8D28AA-426F-4991-A638-E362EF62E8B7}"/>
+    <hyperlink ref="J191" r:id="rId171" xr:uid="{0D368A4C-5099-4A8A-AFA4-4A14478071B4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId164"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId172"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
010-0191, 043-0002, 040-0022, 040-0023, 040-024 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F727296F-CB30-45AB-BA47-6B0C293B0C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAB7F5D-6061-446B-84BA-07CEACF1C04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25812" yWindow="1992" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7858" uniqueCount="3904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7924" uniqueCount="3937">
   <si>
     <t>ID</t>
   </si>
@@ -11761,6 +11761,105 @@
   </si>
   <si>
     <t>VAR SMD 1206</t>
+  </si>
+  <si>
+    <t>043-0002</t>
+  </si>
+  <si>
+    <t>MOSFET P</t>
+  </si>
+  <si>
+    <t>MOSFET -30V Vds 20V Vgs SOT-23</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>SI2303CDS-T1-GE3</t>
+  </si>
+  <si>
+    <t>781-SI2303CDS-T1-GE3</t>
+  </si>
+  <si>
+    <t>https://www.vishay.com/docs/69991/si2303cd.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Vishay-Semiconductors/SI2303CDS-T1-GE3?qs=IRuQNBqMOckJHxNXLRBkmw%3D%3D</t>
+  </si>
+  <si>
+    <t>010-0191</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 220 Ohms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>220Ω 100mW ±1%</t>
+  </si>
+  <si>
+    <t>560112116126</t>
+  </si>
+  <si>
+    <t>710-560112116126</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/560112116126.pdf</t>
+  </si>
+  <si>
+    <t>040-0022</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 1206 0.2AMPS SMD</t>
+  </si>
+  <si>
+    <t>200mA</t>
+  </si>
+  <si>
+    <t>https://datasheets.kyocera-avx.com/AccuGuard2.pdf</t>
+  </si>
+  <si>
+    <t>F1206B0R20FSTR</t>
+  </si>
+  <si>
+    <t>581-F1206B0R20FSTR</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/F1206B0R20FSTR?qs=qfFDQzOiitCIvTCyICvztA%3D%3D</t>
+  </si>
+  <si>
+    <t>040-0023</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 63V 1A FA HALIDE FREE SLIM</t>
+  </si>
+  <si>
+    <t>0466001.NRHF</t>
+  </si>
+  <si>
+    <t>576-0466001.NRHF</t>
+  </si>
+  <si>
+    <t>https://www.littelfuse.com/assetdocs/littelfuse_fuse_466_datasheet?assetguid=dbe9bcd7-6072-4adf-bf5b-d33e52a6b90f</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/Littelfuse/0466001.NRHF?qs=n5MbhIql%252BRl7ALFy%2FbHisA%3D%3D</t>
+  </si>
+  <si>
+    <t>040-0024</t>
+  </si>
+  <si>
+    <t>Fusibles de montaje en superficie 1206 0.5AMPS SMD</t>
+  </si>
+  <si>
+    <t>500mA</t>
+  </si>
+  <si>
+    <t>F1206B0R50FSTR</t>
+  </si>
+  <si>
+    <t>581-F1206B0R50FSTR</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/ProductDetail/KYOCERA-AVX/F1206B0R50FSTR?qs=hZPoALHhU4OC%2FuvTP6tvGA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -11937,7 +12036,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11999,6 +12098,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -20359,7 +20462,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="13" max="13" width="13.36328125" customWidth="1"/>
@@ -21343,6 +21446,138 @@
         <v>1701</v>
       </c>
       <c r="N22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" t="s">
+        <v>3918</v>
+      </c>
+      <c r="B23" s="42" t="s">
+        <v>3919</v>
+      </c>
+      <c r="C23" s="42" t="s">
+        <v>3920</v>
+      </c>
+      <c r="D23" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E23" s="42" t="s">
+        <v>3922</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>3005</v>
+      </c>
+      <c r="G23" s="40" t="s">
+        <v>3923</v>
+      </c>
+      <c r="H23" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I23" t="s">
+        <v>3921</v>
+      </c>
+      <c r="J23" t="s">
+        <v>3924</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L23" t="s">
+        <v>55</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" t="s">
+        <v>3925</v>
+      </c>
+      <c r="B24" s="42" t="s">
+        <v>3926</v>
+      </c>
+      <c r="C24" s="42" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D24" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E24" s="42" t="s">
+        <v>3927</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G24" s="40" t="s">
+        <v>3928</v>
+      </c>
+      <c r="H24" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" s="26" t="s">
+        <v>3929</v>
+      </c>
+      <c r="J24" s="26" t="s">
+        <v>3930</v>
+      </c>
+      <c r="K24" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L24" t="s">
+        <v>55</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" t="s">
+        <v>3931</v>
+      </c>
+      <c r="B25" s="42" t="s">
+        <v>3932</v>
+      </c>
+      <c r="C25" s="42" t="s">
+        <v>3933</v>
+      </c>
+      <c r="D25" s="7">
+        <v>1206</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>3934</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G25" s="40" t="s">
+        <v>3935</v>
+      </c>
+      <c r="H25" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I25" s="26" t="s">
+        <v>3921</v>
+      </c>
+      <c r="J25" s="31" t="s">
+        <v>3936</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L25" t="s">
+        <v>55</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N25" t="s">
         <v>25</v>
       </c>
     </row>
@@ -21367,6 +21602,10 @@
     <hyperlink ref="J21" r:id="rId16" xr:uid="{FFB17F08-401F-47B0-899B-612CD8B9FB6B}"/>
     <hyperlink ref="I22" r:id="rId17" xr:uid="{1372C46B-1234-4FDC-9A5A-49F3F36A3112}"/>
     <hyperlink ref="J22" r:id="rId18" xr:uid="{5B608490-0175-4BFB-8CEB-749053C4E8DA}"/>
+    <hyperlink ref="I24" r:id="rId19" xr:uid="{8860E270-1EA1-413E-81F7-FE643E5ACB08}"/>
+    <hyperlink ref="J24" r:id="rId20" xr:uid="{0EEBF3D2-D854-4F60-9074-0417D1F60860}"/>
+    <hyperlink ref="I25" r:id="rId21" xr:uid="{C43E42B6-8EB7-4520-ABCA-F6BA4656E176}"/>
+    <hyperlink ref="J25" r:id="rId22" xr:uid="{69E1134F-3116-4058-838E-440309247FBB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21476,7 +21715,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FAFF3B6-AF11-4BFB-8078-829FF6F2F366}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -21567,10 +21806,57 @@
         <v>25</v>
       </c>
     </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>3904</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3906</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3907</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3764</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3908</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1957</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3909</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3910</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>3911</v>
+      </c>
+      <c r="K3" t="s">
+        <v>3905</v>
+      </c>
+      <c r="L3" s="33" t="s">
+        <v>3182</v>
+      </c>
+      <c r="M3" s="34" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="15" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{71BC0DAF-9651-41D4-BC90-0CA5C5CA063D}"/>
     <hyperlink ref="J2" r:id="rId2" xr:uid="{B8956BA2-569B-4007-9354-F99A76E81F8D}"/>
+    <hyperlink ref="I3" r:id="rId3" xr:uid="{360B4179-45EE-4DEA-AE1A-A9A674637B6A}"/>
+    <hyperlink ref="J3" r:id="rId4" xr:uid="{9FAEC919-51DF-4619-9BEF-284521DA0E38}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -27787,7 +28073,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N191"/>
+  <dimension ref="A1:N192"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="19.90625" customWidth="1"/>
@@ -36193,6 +36479,47 @@
         <v>57</v>
       </c>
       <c r="N191" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="192" spans="1:14">
+      <c r="A192" s="16" t="s">
+        <v>3912</v>
+      </c>
+      <c r="B192" t="s">
+        <v>3913</v>
+      </c>
+      <c r="C192" s="16" t="s">
+        <v>3914</v>
+      </c>
+      <c r="D192" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E192" s="39" t="s">
+        <v>3915</v>
+      </c>
+      <c r="F192" s="30" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G192" s="41" t="s">
+        <v>3916</v>
+      </c>
+      <c r="H192" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I192" s="26" t="s">
+        <v>3917</v>
+      </c>
+      <c r="K192" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L192" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M192" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N192" t="s">
         <v>25</v>
       </c>
     </row>
@@ -36370,9 +36697,10 @@
     <hyperlink ref="J190" r:id="rId169" xr:uid="{0416598A-C30A-47A1-9871-D973FB462120}"/>
     <hyperlink ref="I191" r:id="rId170" xr:uid="{1A8D28AA-426F-4991-A638-E362EF62E8B7}"/>
     <hyperlink ref="J191" r:id="rId171" xr:uid="{0D368A4C-5099-4A8A-AFA4-4A14478071B4}"/>
+    <hyperlink ref="I192" r:id="rId172" xr:uid="{22F61D15-F86A-45C4-8028-A72154D709C5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId172"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId173"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
015-0005 to 015-0008 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D1E6CF-664F-49E7-AAF4-A6FF5EE364FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7342A5A7-F98A-43CC-839B-CA2D7AA9867C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25812" yWindow="1992" windowWidth="23256" windowHeight="12456" firstSheet="20" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25812" yWindow="2292" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8003" uniqueCount="3976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8059" uniqueCount="4005">
   <si>
     <t>ID</t>
   </si>
@@ -11977,6 +11977,93 @@
   </si>
   <si>
     <t>710-657004240101</t>
+  </si>
+  <si>
+    <t>015-0005</t>
+  </si>
+  <si>
+    <t>015-0006</t>
+  </si>
+  <si>
+    <t>015-0007</t>
+  </si>
+  <si>
+    <t>015-0008</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD WRIS-KWKH 0.62Ohms 1% 1W +200ppm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">620mΩ 1W ±1% </t>
+  </si>
+  <si>
+    <t>1206 (Reversed)</t>
+  </si>
+  <si>
+    <t>561070332081</t>
+  </si>
+  <si>
+    <t>710-561070332081</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/561070332081.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/Wurth-Elektronik/561070332081?qs=unwgFEO1A6sUBr71YhIMeA%3D%3D</t>
+  </si>
+  <si>
+    <t>RES SMD 1206 Reversed</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD WRIS-KWKH 0.15Ohms 1% 1W +350ppm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150mΩ 1W ±1% </t>
+  </si>
+  <si>
+    <t>561070332055</t>
+  </si>
+  <si>
+    <t>710-561070332055</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/components/products/datasheet/561070332055.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/Wurth-Elektronik/561070332055?qs=sGAEpiMZZMtlubZbdhIBIKUWFMOULdJiXOgwA76%2FMU4%3D</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD RLW73 B2 1% R039 200ppm 1k RL</t>
+  </si>
+  <si>
+    <t>RLW73B2FR039TDF</t>
+  </si>
+  <si>
+    <t>279-RLW73B2FR039TDF</t>
+  </si>
+  <si>
+    <t>https://www.te.com/commerce/DocumentDelivery/DDEController?Action=showdoc&amp;DocId=Data+Sheet%7Fcgs-wide-terminal-rlw73%7F2211%7Fpdf%7FEnglish%7FENG_DS_cgs-wide-terminal-rlw73_2211.pdf%7F2176535-1</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/TE-Connectivity-CGS/RLW73B2FR039TDF?qs=8Wlm6%252BaMh8Slhw8Q%252Bucv7g%3D%3D</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD RLW73 B2 1% R068 200ppm 1k RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39mΩ 750mW ±1% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">68mΩ 750mW ±1% </t>
+  </si>
+  <si>
+    <t>RLW73B2FR068TDF</t>
+  </si>
+  <si>
+    <t>279-RLW73B2FR068TDF</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/TE-Connectivity-CGS/RLW73B2FR068TDF?qs=8Wlm6%252BaMh8Q8YtMhJjj3hA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -12231,7 +12318,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -28211,10 +28298,10 @@
       <c r="A71" s="16" t="s">
         <v>3971</v>
       </c>
-      <c r="B71" s="42" t="s">
+      <c r="B71" s="16" t="s">
         <v>3972</v>
       </c>
-      <c r="C71" s="42" t="s">
+      <c r="C71" s="16" t="s">
         <v>2452</v>
       </c>
       <c r="D71" s="16" t="s">
@@ -37119,7 +37206,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="20.26953125" customWidth="1"/>
@@ -37342,6 +37429,182 @@
         <v>1647</v>
       </c>
       <c r="N5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>3976</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3980</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3981</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3982</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>3983</v>
+      </c>
+      <c r="F6" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G6" t="s">
+        <v>3984</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>3985</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>3986</v>
+      </c>
+      <c r="K6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M6" s="42" t="s">
+        <v>3987</v>
+      </c>
+      <c r="N6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>3977</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3988</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3989</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3982</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>3990</v>
+      </c>
+      <c r="F7" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G7" t="s">
+        <v>3991</v>
+      </c>
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>3992</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>3993</v>
+      </c>
+      <c r="K7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M7" s="42" t="s">
+        <v>3987</v>
+      </c>
+      <c r="N7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>3978</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3994</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4000</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3982</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3995</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2192</v>
+      </c>
+      <c r="G8" t="s">
+        <v>3996</v>
+      </c>
+      <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>3997</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>3998</v>
+      </c>
+      <c r="K8" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M8" s="42" t="s">
+        <v>3987</v>
+      </c>
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>3979</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3999</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4001</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3982</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4002</v>
+      </c>
+      <c r="F9" t="s">
+        <v>2192</v>
+      </c>
+      <c r="G9" t="s">
+        <v>4003</v>
+      </c>
+      <c r="H9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>3997</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>4004</v>
+      </c>
+      <c r="K9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M9" s="42" t="s">
+        <v>3987</v>
+      </c>
+      <c r="N9" t="s">
         <v>25</v>
       </c>
     </row>
@@ -37354,8 +37617,17 @@
     <hyperlink ref="I4" r:id="rId4" xr:uid="{DA619253-40A2-482C-A99F-F72A13182916}"/>
     <hyperlink ref="J4" r:id="rId5" xr:uid="{65BF95D6-EB54-41F9-8886-7DFC774FFE44}"/>
     <hyperlink ref="I5" r:id="rId6" xr:uid="{E9BE5DD3-9340-403D-9879-EBA54F1D68BE}"/>
+    <hyperlink ref="I6" r:id="rId7" xr:uid="{A0FEDAF8-B077-4E91-A533-0BF21B3850D4}"/>
+    <hyperlink ref="J6" r:id="rId8" xr:uid="{7E76CE16-8D3D-41D0-B66B-54075687FCB0}"/>
+    <hyperlink ref="I7" r:id="rId9" xr:uid="{588AF41D-5865-4683-B4AC-FFCE2EEF92A4}"/>
+    <hyperlink ref="J7" r:id="rId10" xr:uid="{BDBCF452-A59D-494E-A080-4E069519929D}"/>
+    <hyperlink ref="I8" r:id="rId11" xr:uid="{745537AE-849B-4D1C-9F73-038DE1A2228B}"/>
+    <hyperlink ref="J8" r:id="rId12" xr:uid="{2522A19B-C8CE-448A-B70B-CFD7C4AFEEF0}"/>
+    <hyperlink ref="I9" r:id="rId13" xr:uid="{6C0457D9-CE57-4F5A-8777-E39EA4F17352}"/>
+    <hyperlink ref="J9" r:id="rId14" xr:uid="{BA2A9F42-701A-48EA-BFA8-1B1F3BDDF2F6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
040-0031, 015-0009, 015-0010 added
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4235B249-C6B6-4632-BAF5-38B9C2EE1155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADE0EC3-3018-4F1A-B8F6-A072442F8C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25812" yWindow="2292" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25812" yWindow="2292" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8179" uniqueCount="4058">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8220" uniqueCount="4076">
   <si>
     <t>ID</t>
   </si>
@@ -12224,6 +12224,60 @@
   </si>
   <si>
     <t>https://www.mouser.es/en/ProductDetail/YAGEO/JB12S1002R?qs=iLKYxzqNS77KhcIWcFZ8Jg%3D%3D</t>
+  </si>
+  <si>
+    <t>015-0009</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD TLRP 1206 1.0W R005 1% 100PPM 5K RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5mΩ 1W ±1% </t>
+  </si>
+  <si>
+    <t>TLRP2B10ER005FTD</t>
+  </si>
+  <si>
+    <t>279-TLRP2B10ER005FTD</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/80/46/ENG_DS_1773449_4_D3.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/TE-Connectivity-Holsworthy/TLRP2B10ER005FTD?qs=QNEnbhJQKvZ8E9Cd3elZSA%3D%3D</t>
+  </si>
+  <si>
+    <t>015-0010</t>
+  </si>
+  <si>
+    <t>Current Sense Resistors - SMD RLW73 B2 1% R010 600ppm 1k RL</t>
+  </si>
+  <si>
+    <t>10mΩ 750mW ±1%</t>
+  </si>
+  <si>
+    <t>RLW73B2FR010TDF</t>
+  </si>
+  <si>
+    <t>279-RLW73B2FR010TDF</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/TE-Connectivity-CGS/RLW73B2FR010TDF?qs=8Wlm6%252BaMh8Rd4lNQaStk%252BQ%3D%3D</t>
+  </si>
+  <si>
+    <t>040-0031</t>
+  </si>
+  <si>
+    <t>Surface Mount Fuses JB12S SMD Fuse 63V 5A Slow 1206 3.2mm X 1.6mm</t>
+  </si>
+  <si>
+    <t>JB12S5001R</t>
+  </si>
+  <si>
+    <t>603-JB12S5001R</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/en/ProductDetail/YAGEO/JB12S5001R?qs=iLKYxzqNS7562RQIsLPvYw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -12414,7 +12468,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -12479,7 +12533,6 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -21531,7 +21584,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="13" max="13" width="13.36328125" customWidth="1"/>
@@ -22874,25 +22927,25 @@
       <c r="A31" t="s">
         <v>4053</v>
       </c>
-      <c r="B31" s="43" t="s">
+      <c r="B31" s="16" t="s">
         <v>4054</v>
       </c>
-      <c r="C31" s="43" t="s">
+      <c r="C31" s="16" t="s">
         <v>1754</v>
       </c>
       <c r="D31" s="16">
         <v>1206</v>
       </c>
-      <c r="E31" s="43" t="s">
+      <c r="E31" s="16" t="s">
         <v>4055</v>
       </c>
-      <c r="F31" s="43" t="s">
+      <c r="F31" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G31" s="42" t="s">
+      <c r="G31" s="3" t="s">
         <v>4056</v>
       </c>
-      <c r="H31" s="43" t="s">
+      <c r="H31" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I31" s="26" t="s">
@@ -22911,6 +22964,50 @@
         <v>1701</v>
       </c>
       <c r="N31" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" t="s">
+        <v>4071</v>
+      </c>
+      <c r="B32" s="42" t="s">
+        <v>4072</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D32" s="16">
+        <v>1206</v>
+      </c>
+      <c r="E32" s="42" t="s">
+        <v>4073</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G32" t="s">
+        <v>4074</v>
+      </c>
+      <c r="H32" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I32" s="26" t="s">
+        <v>4011</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>4075</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="L32" t="s">
+        <v>55</v>
+      </c>
+      <c r="M32" s="7" t="s">
+        <v>1701</v>
+      </c>
+      <c r="N32" t="s">
         <v>25</v>
       </c>
     </row>
@@ -22951,6 +23048,8 @@
     <hyperlink ref="J30" r:id="rId32" xr:uid="{B4F8AF74-EF6D-49F1-9CE8-29F632F7A754}"/>
     <hyperlink ref="I31" r:id="rId33" xr:uid="{912C6D59-6DD8-4011-9862-E5A138D7CA88}"/>
     <hyperlink ref="J31" r:id="rId34" xr:uid="{1B54DD8B-3D21-4E72-85BA-7DE1FAD354B9}"/>
+    <hyperlink ref="I32" r:id="rId35" xr:uid="{BB2566A3-B905-4C4D-9CFF-2A1A7A61DA85}"/>
+    <hyperlink ref="J32" r:id="rId36" xr:uid="{80802204-A2D9-4DFF-95F9-BC9A208CDE12}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -38437,7 +38536,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="20.26953125" customWidth="1"/>
@@ -38836,6 +38935,94 @@
         <v>3987</v>
       </c>
       <c r="N9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>4058</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4059</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4060</v>
+      </c>
+      <c r="D10" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" t="s">
+        <v>4061</v>
+      </c>
+      <c r="F10" t="s">
+        <v>2192</v>
+      </c>
+      <c r="G10" t="s">
+        <v>4062</v>
+      </c>
+      <c r="H10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>4063</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>4064</v>
+      </c>
+      <c r="K10" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>1645</v>
+      </c>
+      <c r="N10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="s">
+        <v>4065</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4066</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4067</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3982</v>
+      </c>
+      <c r="E11" t="s">
+        <v>4068</v>
+      </c>
+      <c r="F11" t="s">
+        <v>2192</v>
+      </c>
+      <c r="G11" t="s">
+        <v>4069</v>
+      </c>
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>3997</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>4070</v>
+      </c>
+      <c r="K11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>3987</v>
+      </c>
+      <c r="N11" t="s">
         <v>25</v>
       </c>
     </row>
@@ -38856,9 +39043,13 @@
     <hyperlink ref="J8" r:id="rId12" xr:uid="{2522A19B-C8CE-448A-B70B-CFD7C4AFEEF0}"/>
     <hyperlink ref="I9" r:id="rId13" xr:uid="{6C0457D9-CE57-4F5A-8777-E39EA4F17352}"/>
     <hyperlink ref="J9" r:id="rId14" xr:uid="{BA2A9F42-701A-48EA-BFA8-1B1F3BDDF2F6}"/>
+    <hyperlink ref="I10" r:id="rId15" xr:uid="{2428C7CE-5D0C-41C3-BF1F-988F71D4EF48}"/>
+    <hyperlink ref="J10" r:id="rId16" xr:uid="{15EF6D95-7C3C-42B3-90E3-4546110523C9}"/>
+    <hyperlink ref="I11" r:id="rId17" xr:uid="{6467E5F2-4786-4C6B-A3A3-F0D4C5A67B79}"/>
+    <hyperlink ref="J11" r:id="rId18" xr:uid="{40DA6A61-E97A-4D1C-9CF4-22EC82276332}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added 041-0003 / 100-0024 / 010-0193
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javier\Desktop\MOTO\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD534D5-C995-4D9E-8F7A-DA58D9B04565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9F1710-DA72-4BCB-A729-9827A484C635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10710" yWindow="0" windowWidth="10920" windowHeight="13770" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8275" uniqueCount="4090">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8317" uniqueCount="4115">
   <si>
     <t>ID</t>
   </si>
@@ -12322,6 +12322,81 @@
   </si>
   <si>
     <t>IND 0402</t>
+  </si>
+  <si>
+    <t>041-0003</t>
+  </si>
+  <si>
+    <t>Optoacopladores para salidas de transistores WL-OCPT 35V 5KVrms 10pF Dip 4 S-Type</t>
+  </si>
+  <si>
+    <t>DIP-4</t>
+  </si>
+  <si>
+    <t>710-140817142400</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/catalog/datasheet/140817142400.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/es/ProductDetail/Wurth-Elektronik/140817142400?qs=81r%252BiQLm7BQPLeRqqgk3BQ%3D%3D</t>
+  </si>
+  <si>
+    <t>100-0024</t>
+  </si>
+  <si>
+    <t>Relés universales SPST-NO Flux-Tight 24VDC High-Capacity</t>
+  </si>
+  <si>
+    <t>200mW 8,3mA coil</t>
+  </si>
+  <si>
+    <t>20,5x7,2x15,3mm</t>
+  </si>
+  <si>
+    <t>G5NB-1A-E-DC24</t>
+  </si>
+  <si>
+    <t>Aratas</t>
+  </si>
+  <si>
+    <t>653-G5NB-1A-E-DC24</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/datasheet/3/39/1/J143-E1.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/es/ProductDetail/Aratas/G5NB-1A-E-DC24?qs=3jhwTwe4bOHjt65REhrORA%3D%3D</t>
+  </si>
+  <si>
+    <t>RELE G5NB-1A</t>
+  </si>
+  <si>
+    <t>G5NB-1A</t>
+  </si>
+  <si>
+    <t>010-0193</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD 0.5W 2.2Kohm 1% AEC-Q200</t>
+  </si>
+  <si>
+    <t>0.5W 2.2Kohm 1%</t>
+  </si>
+  <si>
+    <t>SG73P1JTTD2201F</t>
+  </si>
+  <si>
+    <t>660-SG73P1JTTD2201F</t>
+  </si>
+  <si>
+    <t>https://www.koaspeer.com/pdfs/SG73P.pdf</t>
+  </si>
+  <si>
+    <t>https://www.mouser.es/es/ProductDetail/KOA-Speer/SG73P1JTTD2201F?qs=sGAEpiMZZMtlubZbdhIBIMav4eZf%2FxzgRyo3bnq6lCo%3D</t>
+  </si>
+  <si>
+    <t>140817142400</t>
   </si>
 </sst>
 </file>
@@ -12331,7 +12406,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -12461,6 +12536,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -12512,7 +12599,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -12577,6 +12664,13 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -12861,22 +12955,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" customWidth="1"/>
-    <col min="2" max="2" width="29.6328125" customWidth="1"/>
-    <col min="3" max="3" width="14.90625" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" customWidth="1"/>
-    <col min="9" max="9" width="11.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.7265625" customWidth="1"/>
+    <col min="1" max="1" width="11.21875" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.77734375" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="13.1796875" customWidth="1"/>
-    <col min="13" max="13" width="12.54296875" customWidth="1"/>
-    <col min="14" max="14" width="17.6328125" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" customWidth="1"/>
+    <col min="13" max="13" width="12.5546875" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="13.5" customHeight="1">
@@ -12923,7 +13017,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="14" customHeight="1">
+    <row r="2" spans="1:14" ht="13.95" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>58</v>
       </c>
@@ -12967,7 +13061,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="14" customHeight="1">
+    <row r="3" spans="1:14" ht="13.95" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>73</v>
       </c>
@@ -13011,7 +13105,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="14" customHeight="1">
+    <row r="4" spans="1:14" ht="13.95" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>81</v>
       </c>
@@ -13055,7 +13149,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="14" customHeight="1">
+    <row r="5" spans="1:14" ht="13.95" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>88</v>
       </c>
@@ -13099,7 +13193,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="14" customHeight="1">
+    <row r="6" spans="1:14" ht="13.95" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>95</v>
       </c>
@@ -13143,7 +13237,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="14" customHeight="1">
+    <row r="7" spans="1:14" ht="13.95" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>103</v>
       </c>
@@ -13187,7 +13281,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="14" customHeight="1">
+    <row r="8" spans="1:14" ht="13.95" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>110</v>
       </c>
@@ -13231,7 +13325,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="14" customHeight="1">
+    <row r="9" spans="1:14" ht="13.95" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>117</v>
       </c>
@@ -13275,7 +13369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="14" customHeight="1">
+    <row r="10" spans="1:14" ht="13.95" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -13319,7 +13413,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="14" customHeight="1">
+    <row r="11" spans="1:14" ht="13.95" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>131</v>
       </c>
@@ -13363,7 +13457,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="14" customHeight="1">
+    <row r="12" spans="1:14" ht="13.95" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>138</v>
       </c>
@@ -13407,7 +13501,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="14" customHeight="1">
+    <row r="13" spans="1:14" ht="13.95" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>145</v>
       </c>
@@ -13451,7 +13545,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="14" customHeight="1">
+    <row r="14" spans="1:14" ht="13.95" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>153</v>
       </c>
@@ -13495,7 +13589,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="14" customHeight="1">
+    <row r="15" spans="1:14" ht="13.95" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>160</v>
       </c>
@@ -13539,7 +13633,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="14" customHeight="1">
+    <row r="16" spans="1:14" ht="13.95" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>167</v>
       </c>
@@ -13583,7 +13677,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="14" customHeight="1">
+    <row r="17" spans="1:14" ht="13.95" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>174</v>
       </c>
@@ -13627,7 +13721,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="14" customHeight="1">
+    <row r="18" spans="1:14" ht="13.95" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>180</v>
       </c>
@@ -13671,7 +13765,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="14" customHeight="1">
+    <row r="19" spans="1:14" ht="13.95" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>187</v>
       </c>
@@ -13715,7 +13809,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="14" customHeight="1">
+    <row r="20" spans="1:14" ht="13.95" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>194</v>
       </c>
@@ -13759,7 +13853,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="14" customHeight="1">
+    <row r="21" spans="1:14" ht="13.95" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>201</v>
       </c>
@@ -13803,7 +13897,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="14" customHeight="1">
+    <row r="22" spans="1:14" ht="13.95" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>208</v>
       </c>
@@ -13847,7 +13941,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="14" customHeight="1">
+    <row r="23" spans="1:14" ht="13.95" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>216</v>
       </c>
@@ -13891,7 +13985,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="14" customHeight="1">
+    <row r="24" spans="1:14" ht="13.95" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>223</v>
       </c>
@@ -13935,7 +14029,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="14" customHeight="1">
+    <row r="25" spans="1:14" ht="13.95" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>230</v>
       </c>
@@ -13979,7 +14073,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="14" customHeight="1">
+    <row r="26" spans="1:14" ht="13.95" customHeight="1">
       <c r="A26" s="4" t="s">
         <v>237</v>
       </c>
@@ -14023,7 +14117,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="14" customHeight="1">
+    <row r="27" spans="1:14" ht="13.95" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>246</v>
       </c>
@@ -14067,7 +14161,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="14" customHeight="1">
+    <row r="28" spans="1:14" ht="13.95" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>254</v>
       </c>
@@ -14111,7 +14205,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="14" customHeight="1">
+    <row r="29" spans="1:14" ht="13.95" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>261</v>
       </c>
@@ -14155,7 +14249,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="14" customHeight="1">
+    <row r="30" spans="1:14" ht="13.95" customHeight="1">
       <c r="A30" s="4" t="s">
         <v>268</v>
       </c>
@@ -14199,7 +14293,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="14" customHeight="1">
+    <row r="31" spans="1:14" ht="13.95" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>275</v>
       </c>
@@ -14243,7 +14337,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="14" customHeight="1">
+    <row r="32" spans="1:14" ht="13.95" customHeight="1">
       <c r="A32" s="4" t="s">
         <v>282</v>
       </c>
@@ -14287,7 +14381,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="14" customHeight="1">
+    <row r="33" spans="1:14" ht="13.95" customHeight="1">
       <c r="A33" s="4" t="s">
         <v>288</v>
       </c>
@@ -14331,7 +14425,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="14" customHeight="1">
+    <row r="34" spans="1:14" ht="13.95" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>295</v>
       </c>
@@ -14375,7 +14469,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="14" customHeight="1">
+    <row r="35" spans="1:14" ht="13.95" customHeight="1">
       <c r="A35" s="4" t="s">
         <v>302</v>
       </c>
@@ -14419,7 +14513,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="14" customHeight="1">
+    <row r="36" spans="1:14" ht="13.95" customHeight="1">
       <c r="A36" s="4" t="s">
         <v>308</v>
       </c>
@@ -14463,7 +14557,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="14" customHeight="1">
+    <row r="37" spans="1:14" ht="13.95" customHeight="1">
       <c r="A37" s="4" t="s">
         <v>315</v>
       </c>
@@ -14507,7 +14601,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="14" customHeight="1">
+    <row r="38" spans="1:14" ht="13.95" customHeight="1">
       <c r="A38" s="4" t="s">
         <v>322</v>
       </c>
@@ -14551,7 +14645,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="14" customHeight="1">
+    <row r="39" spans="1:14" ht="13.95" customHeight="1">
       <c r="A39" s="4" t="s">
         <v>329</v>
       </c>
@@ -14595,7 +14689,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="14" customHeight="1">
+    <row r="40" spans="1:14" ht="13.95" customHeight="1">
       <c r="A40" s="4" t="s">
         <v>336</v>
       </c>
@@ -14639,7 +14733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="14" customHeight="1">
+    <row r="41" spans="1:14" ht="13.95" customHeight="1">
       <c r="A41" s="4" t="s">
         <v>343</v>
       </c>
@@ -14683,7 +14777,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="14" customHeight="1">
+    <row r="42" spans="1:14" ht="13.95" customHeight="1">
       <c r="A42" s="4" t="s">
         <v>350</v>
       </c>
@@ -14727,7 +14821,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="14" customHeight="1">
+    <row r="43" spans="1:14" ht="13.95" customHeight="1">
       <c r="A43" s="4" t="s">
         <v>357</v>
       </c>
@@ -14771,7 +14865,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="14" customHeight="1">
+    <row r="44" spans="1:14" ht="13.95" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>364</v>
       </c>
@@ -14815,7 +14909,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="14" customHeight="1">
+    <row r="45" spans="1:14" ht="13.95" customHeight="1">
       <c r="A45" s="4" t="s">
         <v>371</v>
       </c>
@@ -14859,7 +14953,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="14" customHeight="1">
+    <row r="46" spans="1:14" ht="13.95" customHeight="1">
       <c r="A46" s="4" t="s">
         <v>378</v>
       </c>
@@ -14903,7 +14997,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="14" customHeight="1">
+    <row r="47" spans="1:14" ht="13.95" customHeight="1">
       <c r="A47" s="4" t="s">
         <v>384</v>
       </c>
@@ -14947,7 +15041,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="14" customHeight="1">
+    <row r="48" spans="1:14" ht="13.95" customHeight="1">
       <c r="A48" s="4" t="s">
         <v>391</v>
       </c>
@@ -14991,7 +15085,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="14" customHeight="1">
+    <row r="49" spans="1:14" ht="13.95" customHeight="1">
       <c r="A49" s="4" t="s">
         <v>398</v>
       </c>
@@ -15035,7 +15129,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="14" customHeight="1">
+    <row r="50" spans="1:14" ht="13.95" customHeight="1">
       <c r="A50" s="4" t="s">
         <v>405</v>
       </c>
@@ -15079,7 +15173,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="14" customHeight="1">
+    <row r="51" spans="1:14" ht="13.95" customHeight="1">
       <c r="A51" s="4" t="s">
         <v>413</v>
       </c>
@@ -15123,7 +15217,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="14" customHeight="1">
+    <row r="52" spans="1:14" ht="13.95" customHeight="1">
       <c r="A52" s="4" t="s">
         <v>420</v>
       </c>
@@ -15167,7 +15261,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="14" customHeight="1">
+    <row r="53" spans="1:14" ht="13.95" customHeight="1">
       <c r="A53" s="4" t="s">
         <v>427</v>
       </c>
@@ -15211,7 +15305,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="14" customHeight="1">
+    <row r="54" spans="1:14" ht="13.95" customHeight="1">
       <c r="A54" s="4" t="s">
         <v>434</v>
       </c>
@@ -15255,7 +15349,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="14" customHeight="1">
+    <row r="55" spans="1:14" ht="13.95" customHeight="1">
       <c r="A55" s="4" t="s">
         <v>441</v>
       </c>
@@ -15299,7 +15393,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="14" customHeight="1">
+    <row r="56" spans="1:14" ht="13.95" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>448</v>
       </c>
@@ -15343,7 +15437,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="14" customHeight="1">
+    <row r="57" spans="1:14" ht="13.95" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>455</v>
       </c>
@@ -15385,7 +15479,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="14" customHeight="1">
+    <row r="58" spans="1:14" ht="13.95" customHeight="1">
       <c r="A58" s="4" t="s">
         <v>461</v>
       </c>
@@ -15429,7 +15523,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="14" customHeight="1">
+    <row r="59" spans="1:14" ht="13.95" customHeight="1">
       <c r="A59" s="4" t="s">
         <v>467</v>
       </c>
@@ -15473,7 +15567,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="14" customHeight="1">
+    <row r="60" spans="1:14" ht="13.95" customHeight="1">
       <c r="A60" s="4" t="s">
         <v>474</v>
       </c>
@@ -15517,7 +15611,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="14" customHeight="1">
+    <row r="61" spans="1:14" ht="13.95" customHeight="1">
       <c r="A61" s="4" t="s">
         <v>482</v>
       </c>
@@ -15561,7 +15655,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14" customHeight="1">
+    <row r="62" spans="1:14" ht="13.95" customHeight="1">
       <c r="A62" s="4" t="s">
         <v>490</v>
       </c>
@@ -15605,7 +15699,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="14" customHeight="1">
+    <row r="63" spans="1:14" ht="13.95" customHeight="1">
       <c r="A63" s="4" t="s">
         <v>497</v>
       </c>
@@ -15649,7 +15743,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="14" customHeight="1">
+    <row r="64" spans="1:14" ht="13.95" customHeight="1">
       <c r="A64" s="4" t="s">
         <v>504</v>
       </c>
@@ -15693,7 +15787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="14" customHeight="1">
+    <row r="65" spans="1:14" ht="13.95" customHeight="1">
       <c r="A65" s="4" t="s">
         <v>511</v>
       </c>
@@ -15737,7 +15831,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="14" customHeight="1">
+    <row r="66" spans="1:14" ht="13.95" customHeight="1">
       <c r="A66" s="4" t="s">
         <v>517</v>
       </c>
@@ -15781,7 +15875,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="14" customHeight="1">
+    <row r="67" spans="1:14" ht="13.95" customHeight="1">
       <c r="A67" s="4" t="s">
         <v>525</v>
       </c>
@@ -15825,7 +15919,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="14" customHeight="1">
+    <row r="68" spans="1:14" ht="13.95" customHeight="1">
       <c r="A68" s="4" t="s">
         <v>531</v>
       </c>
@@ -15869,7 +15963,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="14" customHeight="1">
+    <row r="69" spans="1:14" ht="13.95" customHeight="1">
       <c r="A69" s="4" t="s">
         <v>538</v>
       </c>
@@ -15913,7 +16007,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="14" customHeight="1">
+    <row r="70" spans="1:14" ht="13.95" customHeight="1">
       <c r="A70" s="4" t="s">
         <v>545</v>
       </c>
@@ -15957,7 +16051,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="14" customHeight="1">
+    <row r="71" spans="1:14" ht="13.95" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>552</v>
       </c>
@@ -16001,7 +16095,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="14" customHeight="1">
+    <row r="72" spans="1:14" ht="13.95" customHeight="1">
       <c r="A72" s="4" t="s">
         <v>560</v>
       </c>
@@ -16045,7 +16139,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="14" customHeight="1">
+    <row r="73" spans="1:14" ht="13.95" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>567</v>
       </c>
@@ -16089,7 +16183,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="14" customHeight="1">
+    <row r="74" spans="1:14" ht="13.95" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>574</v>
       </c>
@@ -16133,7 +16227,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="14" customHeight="1">
+    <row r="75" spans="1:14" ht="13.95" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>582</v>
       </c>
@@ -16177,7 +16271,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="14" customHeight="1">
+    <row r="76" spans="1:14" ht="13.95" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>589</v>
       </c>
@@ -16221,7 +16315,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="14" customHeight="1">
+    <row r="77" spans="1:14" ht="13.95" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>595</v>
       </c>
@@ -16265,7 +16359,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="14" customHeight="1">
+    <row r="78" spans="1:14" ht="13.95" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>602</v>
       </c>
@@ -16309,7 +16403,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="14" customHeight="1">
+    <row r="79" spans="1:14" ht="13.95" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>608</v>
       </c>
@@ -16353,7 +16447,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="14" customHeight="1">
+    <row r="80" spans="1:14" ht="13.95" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>615</v>
       </c>
@@ -16397,7 +16491,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="14" customHeight="1">
+    <row r="81" spans="1:14" ht="13.95" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>622</v>
       </c>
@@ -16441,7 +16535,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="14" customHeight="1">
+    <row r="82" spans="1:14" ht="13.95" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>628</v>
       </c>
@@ -16485,7 +16579,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="14" customHeight="1">
+    <row r="83" spans="1:14" ht="13.95" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>635</v>
       </c>
@@ -16529,7 +16623,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="14" customHeight="1">
+    <row r="84" spans="1:14" ht="13.95" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>642</v>
       </c>
@@ -16573,7 +16667,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="14" customHeight="1">
+    <row r="85" spans="1:14" ht="13.95" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>643</v>
       </c>
@@ -16617,7 +16711,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="14" customHeight="1">
+    <row r="86" spans="1:14" ht="13.95" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>650</v>
       </c>
@@ -16661,7 +16755,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="14" customHeight="1">
+    <row r="87" spans="1:14" ht="13.95" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>656</v>
       </c>
@@ -16705,7 +16799,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="14" customHeight="1">
+    <row r="88" spans="1:14" ht="13.95" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>663</v>
       </c>
@@ -16749,7 +16843,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="14" customHeight="1">
+    <row r="89" spans="1:14" ht="13.95" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>670</v>
       </c>
@@ -16793,7 +16887,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="14" customHeight="1">
+    <row r="90" spans="1:14" ht="13.95" customHeight="1">
       <c r="A90" s="4" t="s">
         <v>677</v>
       </c>
@@ -16837,7 +16931,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="14" customHeight="1">
+    <row r="91" spans="1:14" ht="13.95" customHeight="1">
       <c r="A91" s="4" t="s">
         <v>684</v>
       </c>
@@ -16881,7 +16975,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="14" customHeight="1">
+    <row r="92" spans="1:14" ht="13.95" customHeight="1">
       <c r="A92" s="4" t="s">
         <v>691</v>
       </c>
@@ -18680,7 +18774,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652841DA-3619-42EE-A536-61B58BE1B457}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -19092,9 +19186,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2008B-4BF4-4C9A-883A-FEE5873AEAF4}">
   <dimension ref="A1:N14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="16" customHeight="1">
+    <row r="1" spans="1:14" ht="16.05" customHeight="1">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -19138,7 +19232,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="16" customHeight="1">
+    <row r="2" spans="1:14" ht="16.05" customHeight="1">
       <c r="A2" s="7" t="s">
         <v>1911</v>
       </c>
@@ -19182,7 +19276,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="16" customHeight="1">
+    <row r="3" spans="1:14" ht="16.05" customHeight="1">
       <c r="A3" s="7" t="s">
         <v>1920</v>
       </c>
@@ -19226,7 +19320,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="16" customHeight="1">
+    <row r="4" spans="1:14" ht="16.05" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>1928</v>
       </c>
@@ -19270,7 +19364,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="16" customHeight="1">
+    <row r="5" spans="1:14" ht="16.05" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>1936</v>
       </c>
@@ -19314,7 +19408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="16" customHeight="1">
+    <row r="6" spans="1:14" ht="16.05" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>1944</v>
       </c>
@@ -19358,7 +19452,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="16" customHeight="1">
+    <row r="7" spans="1:14" ht="16.05" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>1952</v>
       </c>
@@ -19402,7 +19496,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="16" customHeight="1">
+    <row r="8" spans="1:14" ht="16.05" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>1961</v>
       </c>
@@ -19446,7 +19540,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="16" customHeight="1">
+    <row r="9" spans="1:14" ht="16.05" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>1969</v>
       </c>
@@ -19490,7 +19584,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="16" customHeight="1">
+    <row r="10" spans="1:14" ht="16.05" customHeight="1">
       <c r="A10" s="16" t="s">
         <v>1977</v>
       </c>
@@ -19534,7 +19628,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="16" customHeight="1">
+    <row r="11" spans="1:14" ht="16.05" customHeight="1">
       <c r="A11" s="16" t="s">
         <v>1986</v>
       </c>
@@ -19578,7 +19672,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="16" customHeight="1">
+    <row r="12" spans="1:14" ht="16.05" customHeight="1">
       <c r="A12" s="16" t="s">
         <v>1995</v>
       </c>
@@ -19735,9 +19829,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E65951-BFD2-4888-A0A6-19D5130CB4A6}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="41.1796875" customWidth="1"/>
+    <col min="2" max="2" width="41.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -20806,9 +20900,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="14.5" customHeight="1">
+    <row r="1" spans="1:14" ht="14.55" customHeight="1">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -21160,7 +21254,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="14.5" customHeight="1">
+    <row r="9" spans="1:14" ht="14.55" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>2827</v>
       </c>
@@ -21891,7 +21985,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED8913B-580D-466F-B6D1-947424810FAF}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -22040,10 +22134,10 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
   <dimension ref="A1:O32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="13" max="13" width="13.36328125" customWidth="1"/>
-    <col min="14" max="14" width="16.1796875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -23512,8 +23606,11 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA7E41C9-E62B-4149-A5B5-E7986E8877E6}">
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -23644,6 +23741,50 @@
         <v>3939</v>
       </c>
       <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>4090</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>4091</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4092</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>4114</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G4" s="43" t="s">
+        <v>4093</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>4094</v>
+      </c>
+      <c r="J4" t="s">
+        <v>4095</v>
+      </c>
+      <c r="K4" s="37" t="s">
+        <v>3647</v>
+      </c>
+      <c r="L4" t="s">
+        <v>3648</v>
+      </c>
+      <c r="M4" t="s">
+        <v>4092</v>
+      </c>
+      <c r="N4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -23655,13 +23796,14 @@
     <hyperlink ref="J3" r:id="rId3" xr:uid="{6CF2E8FA-2871-441E-B367-030778224566}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FAFF3B6-AF11-4BFB-8078-829FF6F2F366}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -23810,7 +23952,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E5535EA-E186-4751-BC7F-9B3A0221302E}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -23959,17 +24101,17 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="43.7265625" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" customWidth="1"/>
-    <col min="6" max="6" width="17.81640625" customWidth="1"/>
-    <col min="7" max="7" width="16.7265625" customWidth="1"/>
-    <col min="9" max="9" width="24.7265625" customWidth="1"/>
-    <col min="10" max="10" width="23.6328125" customWidth="1"/>
-    <col min="12" max="12" width="32.453125" customWidth="1"/>
-    <col min="13" max="13" width="14.90625" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" customWidth="1"/>
+    <col min="2" max="2" width="43.77734375" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="17.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="24.77734375" customWidth="1"/>
+    <col min="10" max="10" width="23.6640625" customWidth="1"/>
+    <col min="12" max="12" width="32.44140625" customWidth="1"/>
+    <col min="13" max="13" width="14.88671875" customWidth="1"/>
+    <col min="14" max="14" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -24390,7 +24532,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB39079-151D-4B88-9E1F-4966291E2A6B}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24497,7 +24639,7 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316C64E0-14FB-467C-956A-E132FAFB0232}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24551,7 +24693,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201D74E2-3547-4E9B-8216-09A22645AC2A}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -24653,7 +24795,7 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24848,7 +24990,7 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4185B0A-D162-4EBC-935B-7159E365DD54}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24997,9 +25139,9 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -25465,7 +25607,7 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="32" t="s">
@@ -25623,7 +25765,7 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -26680,7 +26822,48 @@
       </c>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="16"/>
+      <c r="A25" s="16" t="s">
+        <v>4096</v>
+      </c>
+      <c r="B25" s="42" t="s">
+        <v>4097</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>4098</v>
+      </c>
+      <c r="D25" s="46" t="s">
+        <v>4099</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>4100</v>
+      </c>
+      <c r="F25" s="46" t="s">
+        <v>4101</v>
+      </c>
+      <c r="G25" s="43" t="s">
+        <v>4102</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I25" t="s">
+        <v>4103</v>
+      </c>
+      <c r="J25" t="s">
+        <v>4104</v>
+      </c>
+      <c r="K25" s="45" t="s">
+        <v>4105</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>2765</v>
+      </c>
+      <c r="M25" s="45" t="s">
+        <v>4106</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="15" type="noConversion"/>
@@ -26710,11 +26893,11 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
   <dimension ref="A1:N77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.26953125" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30014,7 +30197,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CA19F58-1F35-4F25-A924-B809C68C5457}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="24" t="s">
@@ -30112,9 +30295,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30263,9 +30446,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E940ACE-72CF-4504-B730-2719484575BC}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30414,12 +30597,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N193"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <dimension ref="A1:N194"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="19.90625" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -38905,6 +39088,50 @@
         <v>57</v>
       </c>
       <c r="N193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14">
+      <c r="A194" s="16" t="s">
+        <v>4107</v>
+      </c>
+      <c r="B194" s="42" t="s">
+        <v>4108</v>
+      </c>
+      <c r="C194" s="42" t="s">
+        <v>4109</v>
+      </c>
+      <c r="D194" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="E194" s="43" t="s">
+        <v>4110</v>
+      </c>
+      <c r="F194" s="47" t="s">
+        <v>3547</v>
+      </c>
+      <c r="G194" s="43" t="s">
+        <v>4111</v>
+      </c>
+      <c r="H194" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I194" t="s">
+        <v>4112</v>
+      </c>
+      <c r="J194" t="s">
+        <v>4113</v>
+      </c>
+      <c r="K194" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="L194" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M194" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N194" t="s">
         <v>25</v>
       </c>
     </row>
@@ -39094,9 +39321,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="20.26953125" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -39613,7 +39840,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C6B0FD-D8A3-44EC-9532-03DDA232F922}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -39808,7 +40035,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D956EFE-E955-4E62-8478-2294E6413DC1}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -39956,9 +40183,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A9FAC0-03F3-45B5-A0EF-8375716CA489}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">

</xml_diff>

<commit_message>
Added 051-0001 / 051-0002 / 051-0003 / 051-0004 / 010-0194
</commit_message>
<xml_diff>
--- a/eUSR_Database.xlsx
+++ b/eUSR_Database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\LIB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javier\Desktop\MOTO\LIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F62F1B-5C29-40BE-8B4F-95094F880476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDC6E1D-3CB4-47BC-9DDD-F77C8A250563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10710" yWindow="0" windowWidth="10980" windowHeight="13770" firstSheet="24" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="001 - Capacitors - SMD Ceramics" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8398" uniqueCount="4153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8467" uniqueCount="4189">
   <si>
     <t>ID</t>
   </si>
@@ -12511,6 +12511,114 @@
   </si>
   <si>
     <t>430783034816</t>
+  </si>
+  <si>
+    <t>Puertas lógicas Quad 2-Input A 595-S N74HCT32N A 595-SN7 A 595-SN74HCT32N</t>
+  </si>
+  <si>
+    <t>OR Gate</t>
+  </si>
+  <si>
+    <t>SOIC-14</t>
+  </si>
+  <si>
+    <t>SN74HC32DR</t>
+  </si>
+  <si>
+    <t>051-0001</t>
+  </si>
+  <si>
+    <t>595-SN74HC32DR</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/gpn/sn74hc32</t>
+  </si>
+  <si>
+    <t>https://eu.mouser.com/es/ProductDetail/Texas-Instruments/SN74HC32DR?qs=JHHQeKcAU3Du%2FzZijx6RtA%3D%3D</t>
+  </si>
+  <si>
+    <t>Puertas lógicas Quad 2-Input A 595-S N74HC08D A 595-SN74 A 595-SN74HC08D</t>
+  </si>
+  <si>
+    <t>AND Gate</t>
+  </si>
+  <si>
+    <t>SN74HC08DR</t>
+  </si>
+  <si>
+    <t>595-SN74HC08DR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/gpn/sn54hc08-sp</t>
+  </si>
+  <si>
+    <t>https://eu.mouser.com/es/ProductDetail/Texas-Instruments/SN74HC08DR?qs=sGAEpiMZZMutXGli8Ay4kEEIpW4eUuOm7aqjfwxQiBw%3D</t>
+  </si>
+  <si>
+    <t>051-0002</t>
+  </si>
+  <si>
+    <t>051-0003</t>
+  </si>
+  <si>
+    <t>SN74HC04DR</t>
+  </si>
+  <si>
+    <t>Inversores Hex A 595-SN74HC04D A 595-SN74HC04D A 59 A 595-SN74HC04D</t>
+  </si>
+  <si>
+    <t>NOT Gate</t>
+  </si>
+  <si>
+    <t>595-SN74HC04DR</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/gpn/sn54hc04-sp</t>
+  </si>
+  <si>
+    <t>https://eu.mouser.com/es/ProductDetail/Texas-Instruments/SN74HC04DR?qs=5BZzbFV4k2tw1CBjnu%2F%252B9Q%3D%3D</t>
+  </si>
+  <si>
+    <t>051-0004</t>
+  </si>
+  <si>
+    <t>Temporizadores y productos de apoyo CMOS Timer A 595-LMC 555IM/NOPB A 595-LM A 595-LMC555IM/NOPB</t>
+  </si>
+  <si>
+    <t>"555"</t>
+  </si>
+  <si>
+    <t>LMC555IMX/NOPB</t>
+  </si>
+  <si>
+    <t>595-LMC555IMX/NOPB</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/gpn/lmc555</t>
+  </si>
+  <si>
+    <t>https://eu.mouser.com/es/ProductDetail/Texas-Instruments/LMC555IMX-NOPB?qs=sGAEpiMZZMutXGli8Ay4kNAnUfdQpJkZNpfT8w9oXWg%3D</t>
+  </si>
+  <si>
+    <t>010-0195</t>
+  </si>
+  <si>
+    <t>Resistores de película gruesa - SMD WRIS-RSKS 6.8 kOhms 1 % 0.1 W 0603 AEC-Q200</t>
+  </si>
+  <si>
+    <t>6.8 kOhms 1 % 0.1 W</t>
+  </si>
+  <si>
+    <t>710-560112116007</t>
+  </si>
+  <si>
+    <t>https://www.we-online.com/catalog/datasheet/560112116007.pdf</t>
+  </si>
+  <si>
+    <t>https://eu.mouser.com/es/ProductDetail/Wurth-Elektronik/560112116007?qs=mELouGlnn3fJYtngcFqTrA%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -12520,7 +12628,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -12686,6 +12794,24 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF212529"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -12737,7 +12863,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -12810,8 +12936,11 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -13096,22 +13225,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N129"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" customWidth="1"/>
-    <col min="2" max="2" width="29.6328125" customWidth="1"/>
-    <col min="3" max="3" width="14.90625" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" customWidth="1"/>
-    <col min="9" max="9" width="11.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.81640625" customWidth="1"/>
+    <col min="1" max="1" width="11.21875" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.77734375" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="13.1796875" customWidth="1"/>
-    <col min="13" max="13" width="12.54296875" customWidth="1"/>
-    <col min="14" max="14" width="17.6328125" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" customWidth="1"/>
+    <col min="13" max="13" width="12.5546875" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="13.5" customHeight="1">
@@ -13158,7 +13287,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="14" customHeight="1">
+    <row r="2" spans="1:14" ht="13.95" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>58</v>
       </c>
@@ -13202,7 +13331,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="14" customHeight="1">
+    <row r="3" spans="1:14" ht="13.95" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>73</v>
       </c>
@@ -13246,7 +13375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="14" customHeight="1">
+    <row r="4" spans="1:14" ht="13.95" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>81</v>
       </c>
@@ -13290,7 +13419,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="14" customHeight="1">
+    <row r="5" spans="1:14" ht="13.95" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>88</v>
       </c>
@@ -13334,7 +13463,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="14" customHeight="1">
+    <row r="6" spans="1:14" ht="13.95" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>95</v>
       </c>
@@ -13378,7 +13507,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="14" customHeight="1">
+    <row r="7" spans="1:14" ht="13.95" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>103</v>
       </c>
@@ -13422,7 +13551,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="14" customHeight="1">
+    <row r="8" spans="1:14" ht="13.95" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>110</v>
       </c>
@@ -13466,7 +13595,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="14" customHeight="1">
+    <row r="9" spans="1:14" ht="13.95" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>117</v>
       </c>
@@ -13510,7 +13639,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="14" customHeight="1">
+    <row r="10" spans="1:14" ht="13.95" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -13554,7 +13683,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="14" customHeight="1">
+    <row r="11" spans="1:14" ht="13.95" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>131</v>
       </c>
@@ -13598,7 +13727,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="14" customHeight="1">
+    <row r="12" spans="1:14" ht="13.95" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>138</v>
       </c>
@@ -13642,7 +13771,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="14" customHeight="1">
+    <row r="13" spans="1:14" ht="13.95" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>145</v>
       </c>
@@ -13686,7 +13815,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="14" customHeight="1">
+    <row r="14" spans="1:14" ht="13.95" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>153</v>
       </c>
@@ -13730,7 +13859,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="14" customHeight="1">
+    <row r="15" spans="1:14" ht="13.95" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>160</v>
       </c>
@@ -13774,7 +13903,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="14" customHeight="1">
+    <row r="16" spans="1:14" ht="13.95" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>167</v>
       </c>
@@ -13818,7 +13947,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="14" customHeight="1">
+    <row r="17" spans="1:14" ht="13.95" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>174</v>
       </c>
@@ -13862,7 +13991,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="14" customHeight="1">
+    <row r="18" spans="1:14" ht="13.95" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>180</v>
       </c>
@@ -13906,7 +14035,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="14" customHeight="1">
+    <row r="19" spans="1:14" ht="13.95" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>187</v>
       </c>
@@ -13950,7 +14079,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="14" customHeight="1">
+    <row r="20" spans="1:14" ht="13.95" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>194</v>
       </c>
@@ -13994,7 +14123,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="14" customHeight="1">
+    <row r="21" spans="1:14" ht="13.95" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>201</v>
       </c>
@@ -14038,7 +14167,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="14" customHeight="1">
+    <row r="22" spans="1:14" ht="13.95" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>208</v>
       </c>
@@ -14082,7 +14211,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="14" customHeight="1">
+    <row r="23" spans="1:14" ht="13.95" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>216</v>
       </c>
@@ -14126,7 +14255,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="14" customHeight="1">
+    <row r="24" spans="1:14" ht="13.95" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>223</v>
       </c>
@@ -14170,7 +14299,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="14" customHeight="1">
+    <row r="25" spans="1:14" ht="13.95" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>230</v>
       </c>
@@ -14214,7 +14343,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="14" customHeight="1">
+    <row r="26" spans="1:14" ht="13.95" customHeight="1">
       <c r="A26" s="4" t="s">
         <v>237</v>
       </c>
@@ -14258,7 +14387,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="14" customHeight="1">
+    <row r="27" spans="1:14" ht="13.95" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>246</v>
       </c>
@@ -14302,7 +14431,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="14" customHeight="1">
+    <row r="28" spans="1:14" ht="13.95" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>254</v>
       </c>
@@ -14346,7 +14475,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="14" customHeight="1">
+    <row r="29" spans="1:14" ht="13.95" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>261</v>
       </c>
@@ -14390,7 +14519,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="14" customHeight="1">
+    <row r="30" spans="1:14" ht="13.95" customHeight="1">
       <c r="A30" s="4" t="s">
         <v>268</v>
       </c>
@@ -14434,7 +14563,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="14" customHeight="1">
+    <row r="31" spans="1:14" ht="13.95" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>275</v>
       </c>
@@ -14478,7 +14607,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="14" customHeight="1">
+    <row r="32" spans="1:14" ht="13.95" customHeight="1">
       <c r="A32" s="4" t="s">
         <v>282</v>
       </c>
@@ -14522,7 +14651,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="14" customHeight="1">
+    <row r="33" spans="1:14" ht="13.95" customHeight="1">
       <c r="A33" s="4" t="s">
         <v>288</v>
       </c>
@@ -14566,7 +14695,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="14" customHeight="1">
+    <row r="34" spans="1:14" ht="13.95" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>295</v>
       </c>
@@ -14610,7 +14739,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="14" customHeight="1">
+    <row r="35" spans="1:14" ht="13.95" customHeight="1">
       <c r="A35" s="4" t="s">
         <v>302</v>
       </c>
@@ -14654,7 +14783,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="14" customHeight="1">
+    <row r="36" spans="1:14" ht="13.95" customHeight="1">
       <c r="A36" s="4" t="s">
         <v>308</v>
       </c>
@@ -14698,7 +14827,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="14" customHeight="1">
+    <row r="37" spans="1:14" ht="13.95" customHeight="1">
       <c r="A37" s="4" t="s">
         <v>315</v>
       </c>
@@ -14742,7 +14871,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="14" customHeight="1">
+    <row r="38" spans="1:14" ht="13.95" customHeight="1">
       <c r="A38" s="4" t="s">
         <v>322</v>
       </c>
@@ -14786,7 +14915,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="14" customHeight="1">
+    <row r="39" spans="1:14" ht="13.95" customHeight="1">
       <c r="A39" s="4" t="s">
         <v>329</v>
       </c>
@@ -14830,7 +14959,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="14" customHeight="1">
+    <row r="40" spans="1:14" ht="13.95" customHeight="1">
       <c r="A40" s="4" t="s">
         <v>336</v>
       </c>
@@ -14874,7 +15003,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="14" customHeight="1">
+    <row r="41" spans="1:14" ht="13.95" customHeight="1">
       <c r="A41" s="4" t="s">
         <v>343</v>
       </c>
@@ -14918,7 +15047,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="14" customHeight="1">
+    <row r="42" spans="1:14" ht="13.95" customHeight="1">
       <c r="A42" s="4" t="s">
         <v>350</v>
       </c>
@@ -14962,7 +15091,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="14" customHeight="1">
+    <row r="43" spans="1:14" ht="13.95" customHeight="1">
       <c r="A43" s="4" t="s">
         <v>357</v>
       </c>
@@ -15006,7 +15135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="14" customHeight="1">
+    <row r="44" spans="1:14" ht="13.95" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>364</v>
       </c>
@@ -15050,7 +15179,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="14" customHeight="1">
+    <row r="45" spans="1:14" ht="13.95" customHeight="1">
       <c r="A45" s="4" t="s">
         <v>371</v>
       </c>
@@ -15094,7 +15223,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="14" customHeight="1">
+    <row r="46" spans="1:14" ht="13.95" customHeight="1">
       <c r="A46" s="4" t="s">
         <v>378</v>
       </c>
@@ -15138,7 +15267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="14" customHeight="1">
+    <row r="47" spans="1:14" ht="13.95" customHeight="1">
       <c r="A47" s="4" t="s">
         <v>384</v>
       </c>
@@ -15182,7 +15311,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="14" customHeight="1">
+    <row r="48" spans="1:14" ht="13.95" customHeight="1">
       <c r="A48" s="4" t="s">
         <v>391</v>
       </c>
@@ -15226,7 +15355,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="14" customHeight="1">
+    <row r="49" spans="1:14" ht="13.95" customHeight="1">
       <c r="A49" s="4" t="s">
         <v>398</v>
       </c>
@@ -15270,7 +15399,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="14" customHeight="1">
+    <row r="50" spans="1:14" ht="13.95" customHeight="1">
       <c r="A50" s="4" t="s">
         <v>405</v>
       </c>
@@ -15314,7 +15443,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="14" customHeight="1">
+    <row r="51" spans="1:14" ht="13.95" customHeight="1">
       <c r="A51" s="4" t="s">
         <v>413</v>
       </c>
@@ -15358,7 +15487,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="14" customHeight="1">
+    <row r="52" spans="1:14" ht="13.95" customHeight="1">
       <c r="A52" s="4" t="s">
         <v>420</v>
       </c>
@@ -15402,7 +15531,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="14" customHeight="1">
+    <row r="53" spans="1:14" ht="13.95" customHeight="1">
       <c r="A53" s="4" t="s">
         <v>427</v>
       </c>
@@ -15446,7 +15575,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="14" customHeight="1">
+    <row r="54" spans="1:14" ht="13.95" customHeight="1">
       <c r="A54" s="4" t="s">
         <v>434</v>
       </c>
@@ -15490,7 +15619,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="14" customHeight="1">
+    <row r="55" spans="1:14" ht="13.95" customHeight="1">
       <c r="A55" s="4" t="s">
         <v>441</v>
       </c>
@@ -15534,7 +15663,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="14" customHeight="1">
+    <row r="56" spans="1:14" ht="13.95" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>448</v>
       </c>
@@ -15578,7 +15707,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="14" customHeight="1">
+    <row r="57" spans="1:14" ht="13.95" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>455</v>
       </c>
@@ -15620,7 +15749,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="14" customHeight="1">
+    <row r="58" spans="1:14" ht="13.95" customHeight="1">
       <c r="A58" s="4" t="s">
         <v>461</v>
       </c>
@@ -15664,7 +15793,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="14" customHeight="1">
+    <row r="59" spans="1:14" ht="13.95" customHeight="1">
       <c r="A59" s="4" t="s">
         <v>467</v>
       </c>
@@ -15708,7 +15837,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="14" customHeight="1">
+    <row r="60" spans="1:14" ht="13.95" customHeight="1">
       <c r="A60" s="4" t="s">
         <v>474</v>
       </c>
@@ -15752,7 +15881,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="14" customHeight="1">
+    <row r="61" spans="1:14" ht="13.95" customHeight="1">
       <c r="A61" s="4" t="s">
         <v>482</v>
       </c>
@@ -15796,7 +15925,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14" customHeight="1">
+    <row r="62" spans="1:14" ht="13.95" customHeight="1">
       <c r="A62" s="4" t="s">
         <v>490</v>
       </c>
@@ -15840,7 +15969,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="14" customHeight="1">
+    <row r="63" spans="1:14" ht="13.95" customHeight="1">
       <c r="A63" s="4" t="s">
         <v>497</v>
       </c>
@@ -15884,7 +16013,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="14" customHeight="1">
+    <row r="64" spans="1:14" ht="13.95" customHeight="1">
       <c r="A64" s="4" t="s">
         <v>504</v>
       </c>
@@ -15928,7 +16057,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="14" customHeight="1">
+    <row r="65" spans="1:14" ht="13.95" customHeight="1">
       <c r="A65" s="4" t="s">
         <v>511</v>
       </c>
@@ -15972,7 +16101,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="14" customHeight="1">
+    <row r="66" spans="1:14" ht="13.95" customHeight="1">
       <c r="A66" s="4" t="s">
         <v>517</v>
       </c>
@@ -16016,7 +16145,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="14" customHeight="1">
+    <row r="67" spans="1:14" ht="13.95" customHeight="1">
       <c r="A67" s="4" t="s">
         <v>525</v>
       </c>
@@ -16060,7 +16189,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="14" customHeight="1">
+    <row r="68" spans="1:14" ht="13.95" customHeight="1">
       <c r="A68" s="4" t="s">
         <v>531</v>
       </c>
@@ -16104,7 +16233,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="14" customHeight="1">
+    <row r="69" spans="1:14" ht="13.95" customHeight="1">
       <c r="A69" s="4" t="s">
         <v>538</v>
       </c>
@@ -16148,7 +16277,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="14" customHeight="1">
+    <row r="70" spans="1:14" ht="13.95" customHeight="1">
       <c r="A70" s="4" t="s">
         <v>545</v>
       </c>
@@ -16192,7 +16321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="14" customHeight="1">
+    <row r="71" spans="1:14" ht="13.95" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>552</v>
       </c>
@@ -16236,7 +16365,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="14" customHeight="1">
+    <row r="72" spans="1:14" ht="13.95" customHeight="1">
       <c r="A72" s="4" t="s">
         <v>560</v>
       </c>
@@ -16280,7 +16409,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="14" customHeight="1">
+    <row r="73" spans="1:14" ht="13.95" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>567</v>
       </c>
@@ -16324,7 +16453,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="14" customHeight="1">
+    <row r="74" spans="1:14" ht="13.95" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>574</v>
       </c>
@@ -16368,7 +16497,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="14" customHeight="1">
+    <row r="75" spans="1:14" ht="13.95" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>582</v>
       </c>
@@ -16412,7 +16541,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="14" customHeight="1">
+    <row r="76" spans="1:14" ht="13.95" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>589</v>
       </c>
@@ -16456,7 +16585,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="14" customHeight="1">
+    <row r="77" spans="1:14" ht="13.95" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>595</v>
       </c>
@@ -16500,7 +16629,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="14" customHeight="1">
+    <row r="78" spans="1:14" ht="13.95" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>602</v>
       </c>
@@ -16544,7 +16673,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="14" customHeight="1">
+    <row r="79" spans="1:14" ht="13.95" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>608</v>
       </c>
@@ -16588,7 +16717,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="14" customHeight="1">
+    <row r="80" spans="1:14" ht="13.95" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>615</v>
       </c>
@@ -16632,7 +16761,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="14" customHeight="1">
+    <row r="81" spans="1:14" ht="13.95" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>622</v>
       </c>
@@ -16676,7 +16805,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="14" customHeight="1">
+    <row r="82" spans="1:14" ht="13.95" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>628</v>
       </c>
@@ -16720,7 +16849,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="14" customHeight="1">
+    <row r="83" spans="1:14" ht="13.95" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>635</v>
       </c>
@@ -16764,7 +16893,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="14" customHeight="1">
+    <row r="84" spans="1:14" ht="13.95" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>642</v>
       </c>
@@ -16808,7 +16937,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="14" customHeight="1">
+    <row r="85" spans="1:14" ht="13.95" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>643</v>
       </c>
@@ -16852,7 +16981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="14" customHeight="1">
+    <row r="86" spans="1:14" ht="13.95" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>650</v>
       </c>
@@ -16896,7 +17025,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="14" customHeight="1">
+    <row r="87" spans="1:14" ht="13.95" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>656</v>
       </c>
@@ -16940,7 +17069,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="14" customHeight="1">
+    <row r="88" spans="1:14" ht="13.95" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>663</v>
       </c>
@@ -16984,7 +17113,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="14" customHeight="1">
+    <row r="89" spans="1:14" ht="13.95" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>670</v>
       </c>
@@ -17028,7 +17157,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="14" customHeight="1">
+    <row r="90" spans="1:14" ht="13.95" customHeight="1">
       <c r="A90" s="4" t="s">
         <v>677</v>
       </c>
@@ -17072,7 +17201,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="14" customHeight="1">
+    <row r="91" spans="1:14" ht="13.95" customHeight="1">
       <c r="A91" s="4" t="s">
         <v>684</v>
       </c>
@@ -17116,7 +17245,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="14" customHeight="1">
+    <row r="92" spans="1:14" ht="13.95" customHeight="1">
       <c r="A92" s="4" t="s">
         <v>691</v>
       </c>
@@ -18915,7 +19044,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652841DA-3619-42EE-A536-61B58BE1B457}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -19372,9 +19501,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE2008B-4BF4-4C9A-883A-FEE5873AEAF4}">
   <dimension ref="A1:N14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="16" customHeight="1">
+    <row r="1" spans="1:14" ht="16.05" customHeight="1">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -19418,7 +19547,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="16" customHeight="1">
+    <row r="2" spans="1:14" ht="16.05" customHeight="1">
       <c r="A2" s="7" t="s">
         <v>1911</v>
       </c>
@@ -19462,7 +19591,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="16" customHeight="1">
+    <row r="3" spans="1:14" ht="16.05" customHeight="1">
       <c r="A3" s="7" t="s">
         <v>1920</v>
       </c>
@@ -19506,7 +19635,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="16" customHeight="1">
+    <row r="4" spans="1:14" ht="16.05" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>1928</v>
       </c>
@@ -19550,7 +19679,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="16" customHeight="1">
+    <row r="5" spans="1:14" ht="16.05" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>1936</v>
       </c>
@@ -19594,7 +19723,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="16" customHeight="1">
+    <row r="6" spans="1:14" ht="16.05" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>1944</v>
       </c>
@@ -19638,7 +19767,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="16" customHeight="1">
+    <row r="7" spans="1:14" ht="16.05" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>1952</v>
       </c>
@@ -19682,7 +19811,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="16" customHeight="1">
+    <row r="8" spans="1:14" ht="16.05" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>1961</v>
       </c>
@@ -19726,7 +19855,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="16" customHeight="1">
+    <row r="9" spans="1:14" ht="16.05" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>1969</v>
       </c>
@@ -19770,7 +19899,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="16" customHeight="1">
+    <row r="10" spans="1:14" ht="16.05" customHeight="1">
       <c r="A10" s="16" t="s">
         <v>1977</v>
       </c>
@@ -19814,7 +19943,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="16" customHeight="1">
+    <row r="11" spans="1:14" ht="16.05" customHeight="1">
       <c r="A11" s="16" t="s">
         <v>1986</v>
       </c>
@@ -19858,7 +19987,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="16" customHeight="1">
+    <row r="12" spans="1:14" ht="16.05" customHeight="1">
       <c r="A12" s="16" t="s">
         <v>1995</v>
       </c>
@@ -20015,9 +20144,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E65951-BFD2-4888-A0A6-19D5130CB4A6}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="41.1796875" customWidth="1"/>
+    <col min="2" max="2" width="41.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -21086,9 +21215,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BFA1EF-29B2-41E4-A9D1-F8E90A663FA1}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="14.5" customHeight="1">
+    <row r="1" spans="1:14" ht="14.55" customHeight="1">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -21440,7 +21569,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="14.5" customHeight="1">
+    <row r="9" spans="1:14" ht="14.55" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>2827</v>
       </c>
@@ -22171,7 +22300,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED8913B-580D-466F-B6D1-947424810FAF}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -22320,10 +22449,10 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6F0D32-9CE2-4DF7-927E-42E7BA331F12}">
   <dimension ref="A1:O32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="13" max="13" width="13.36328125" customWidth="1"/>
-    <col min="14" max="14" width="16.1796875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -23793,9 +23922,9 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA7E41C9-E62B-4149-A5B5-E7986E8877E6}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -23989,7 +24118,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FAFF3B6-AF11-4BFB-8078-829FF6F2F366}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -24182,7 +24311,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E5535EA-E186-4751-BC7F-9B3A0221302E}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -24331,17 +24460,17 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98E1A12-072F-4773-8CB5-47FFE077E85B}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="43.81640625" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" customWidth="1"/>
-    <col min="6" max="6" width="17.81640625" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" customWidth="1"/>
-    <col min="9" max="9" width="24.81640625" customWidth="1"/>
-    <col min="10" max="10" width="23.6328125" customWidth="1"/>
-    <col min="12" max="12" width="32.453125" customWidth="1"/>
-    <col min="13" max="13" width="14.90625" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" customWidth="1"/>
+    <col min="2" max="2" width="43.77734375" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="17.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="24.77734375" customWidth="1"/>
+    <col min="10" max="10" width="23.6640625" customWidth="1"/>
+    <col min="12" max="12" width="32.44140625" customWidth="1"/>
+    <col min="13" max="13" width="14.88671875" customWidth="1"/>
+    <col min="14" max="14" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -24762,7 +24891,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB39079-151D-4B88-9E1F-4966291E2A6B}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24868,8 +24997,8 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316C64E0-14FB-467C-956A-E132FAFB0232}">
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -24915,7 +25044,184 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>4157</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4153</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4154</v>
+      </c>
+      <c r="D2" s="51" t="s">
+        <v>4155</v>
+      </c>
+      <c r="E2" s="42" t="s">
+        <v>4156</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4159</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>4158</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>4160</v>
+      </c>
+      <c r="J2" t="s">
+        <v>4161</v>
+      </c>
+      <c r="K2" t="s">
+        <v>4156</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" t="s">
+        <v>4155</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>4168</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>4162</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4163</v>
+      </c>
+      <c r="D3" s="51" t="s">
+        <v>4155</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>4164</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4159</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>4165</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>4166</v>
+      </c>
+      <c r="J3" t="s">
+        <v>4167</v>
+      </c>
+      <c r="K3" t="s">
+        <v>4164</v>
+      </c>
+      <c r="L3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" t="s">
+        <v>4155</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>4169</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>4171</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4172</v>
+      </c>
+      <c r="D4" s="51" t="s">
+        <v>4155</v>
+      </c>
+      <c r="E4" s="42" t="s">
+        <v>4170</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4159</v>
+      </c>
+      <c r="G4" s="42" t="s">
+        <v>4173</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>4174</v>
+      </c>
+      <c r="J4" t="s">
+        <v>4175</v>
+      </c>
+      <c r="K4" t="s">
+        <v>4170</v>
+      </c>
+      <c r="L4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" t="s">
+        <v>4155</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>4176</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>4177</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4178</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>3768</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>4179</v>
+      </c>
+      <c r="F5" t="s">
+        <v>4159</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>4180</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>4181</v>
+      </c>
+      <c r="J5" t="s">
+        <v>4182</v>
+      </c>
+      <c r="K5" t="s">
+        <v>4179</v>
+      </c>
+      <c r="L5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" s="51" t="s">
+        <v>3768</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -24923,7 +25229,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201D74E2-3547-4E9B-8216-09A22645AC2A}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="32" t="s">
@@ -25025,7 +25331,7 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BC8B2E-A067-463D-937A-30E88D8BECD0}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -25220,7 +25526,7 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4185B0A-D162-4EBC-935B-7159E365DD54}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -25369,9 +25675,9 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4BBBCF5-BAC9-459C-ABE9-2526B85FD81E}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="4" max="4" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -25837,7 +26143,7 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9EB2F5-2977-493B-BFA2-5CD20F8A3BC4}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="32" t="s">
@@ -25995,10 +26301,10 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A1C46E-DEF3-467B-A5BD-162AB66E6A86}">
   <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.36328125" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -27147,10 +27453,10 @@
       <c r="A27" s="16" t="s">
         <v>4146</v>
       </c>
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="3" t="s">
         <v>4147</v>
       </c>
-      <c r="C27" s="51" t="s">
+      <c r="C27" s="16" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="16" t="s">
@@ -27159,13 +27465,13 @@
       <c r="E27">
         <v>430783034816</v>
       </c>
-      <c r="F27" s="51" t="s">
+      <c r="F27" s="16" t="s">
         <v>2695</v>
       </c>
-      <c r="G27" s="51" t="s">
+      <c r="G27" s="16" t="s">
         <v>4149</v>
       </c>
-      <c r="H27" s="51" t="s">
+      <c r="H27" s="16" t="s">
         <v>21</v>
       </c>
       <c r="I27" s="26" t="s">
@@ -27217,11 +27523,11 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE14AD29-8DB0-4C42-AB91-A73B867AE121}">
   <dimension ref="A1:N77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1796875" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30567,7 +30873,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CA19F58-1F35-4F25-A924-B809C68C5457}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="24" t="s">
@@ -30665,9 +30971,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05CC479-3669-40F7-BE22-BA5CFBFF29E9}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30816,9 +31122,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E940ACE-72CF-4504-B730-2719484575BC}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -30967,12 +31273,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E8291E-4293-4634-B9E9-80CB520CA181}">
-  <dimension ref="A1:N195"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <dimension ref="A1:N196"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="19.90625" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -39546,6 +39852,50 @@
         <v>57</v>
       </c>
       <c r="N195" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14">
+      <c r="A196" s="16" t="s">
+        <v>4183</v>
+      </c>
+      <c r="B196" s="52" t="s">
+        <v>4184</v>
+      </c>
+      <c r="C196" s="53" t="s">
+        <v>4185</v>
+      </c>
+      <c r="D196" s="53" t="s">
+        <v>59</v>
+      </c>
+      <c r="E196" s="42">
+        <v>560112116007</v>
+      </c>
+      <c r="F196" s="30" t="s">
+        <v>2100</v>
+      </c>
+      <c r="G196" s="42" t="s">
+        <v>4186</v>
+      </c>
+      <c r="H196" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I196" t="s">
+        <v>4187</v>
+      </c>
+      <c r="J196" t="s">
+        <v>4188</v>
+      </c>
+      <c r="K196" s="54" t="s">
+        <v>34</v>
+      </c>
+      <c r="L196" s="17" t="s">
+        <v>1648</v>
+      </c>
+      <c r="M196" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N196" t="s">
         <v>25</v>
       </c>
     </row>
@@ -39735,9 +40085,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F9848D-6D60-47C0-9F84-A561FE4F106E}">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="20.1796875" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -40254,7 +40604,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C6B0FD-D8A3-44EC-9532-03DDA232F922}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -40449,7 +40799,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D956EFE-E955-4E62-8478-2294E6413DC1}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
@@ -40597,9 +40947,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A9FAC0-03F3-45B5-A0EF-8375716CA489}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">

</xml_diff>